<commit_message>
Upload Vietnam_Infra_News_Database.xlsx - 2026-04-13
</commit_message>
<xml_diff>
--- a/reports/2026-04-13/Vietnam_Infra_News_Database.xlsx
+++ b/reports/2026-04-13/Vietnam_Infra_News_Database.xlsx
@@ -568,17 +568,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] National Power Development Plan VIII (PDP-8) - Vntpa — To develop the power sources and transmission grid at the voltage levels of 220kV or higher, renewable and new energy industries and services in Viet Nam for ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 2030년까지의 국가 전력 개발 계획(PDP8)을 승인하며 에너지 안보 확보와 탈탄소화를 목표로 설정했습니다. 이 계획은 석탄 화력을 단계적으로 폐지하고 해상 풍력 및 태양광과 같은 재생 에너지 비중을 2050년까지 최대 71.5%까지 확대하는 내용을 담고 있습니다.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] National Power Development Plan VIII (PDP-8) - Vntpa — To develop the power sources and transmission grid at the voltage levels of 220kV or higher, renewable and new energy industries and services in Viet Nam for ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has officially approved the National Power Development Plan VIII (PDP8), targeting a transition towards renewable energy and national energy security through 2030. The plan prioritizes the phasing out of coal-fired power by 2050 while significantly expanding wind, solar, and gas-to-hydrogen capacities to meet a 7% annual GDP growth demand.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] National Power Development Plan VIII (PDP-8) - Vntpa — To develop the power sources and transmission grid at the voltage levels of 220kV or higher, renewable and new energy industries and services in Viet Nam for ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Quy hoạch phát triển điện lực quốc gia thời kỳ 2021 - 2030 (Quy hoạch điện VIII) nhằm đảm bảo an ninh năng lượng và chuyển đổi xanh. Kế hoạch tập trung vào việc loại bỏ dần điện than vào năm 2050, đồng thời thúc đẩy mạnh mẽ năng lượng tái tạo và điện khí để phục vụ mục tiêu tăng trưởng kinh tế.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -628,17 +628,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eighth National Power Development Plan (PDP VIII) - PwC — PDP VIII presents an ambitious shift for Vietnam's generation mix away from coal, and heavily weighted towards in renewables and new technologies. (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 2030년까지 발전 용량을 150GW로 확대하고 2050년 탄소 중립을 달성하기 위한 제8차 국가전력개발계획(PDP VIII)을 승인했습니다. 이 계획은 석탄 화력 발전에서 재생 에너지, 수소, 암모니아 및 배터리 저장 시스템으로의 대대적인 전환을 목표로 하며, 인프라 구축을 위해 향후 30년간 약 7,000억 달러의 투자가 필요할 것으로 예상됩니다.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eighth National Power Development Plan (PDP VIII) - PwC — PDP VIII presents an ambitious shift for Vietnam's generation mix away from coal, and heavily weighted towards in renewables and new technologies. (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has approved the PDP VIII, an ambitious energy roadmap targeting 150 GW of installed capacity by 2030 and Net Zero emissions by 2050. The plan shifts focus from coal to renewables and emerging technologies like hydrogen and battery storage, requiring approximately $700 billion in investment over the next three decades for generation and grid infrastructure.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eighth National Power Development Plan (PDP VIII) - PwC — PDP VIII presents an ambitious shift for Vietnam's generation mix away from coal, and heavily weighted towards in renewables and new technologies. (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Quy hoạch điện VIII (PDP VIII), đặt mục tiêu nâng công suất lắp đặt lên 150 GW vào năm 2030 và hướng tới phát thải ròng bằng 0 vào năm 2050. Kế hoạch này tập trung chuyển đổi từ điện than sang năng lượng tái tạo, hydro và lưu trữ năng lượng, với nhu cầu vốn đầu tư dự kiến khoảng 700 tỷ USD trong 3 thập kỷ tới cho nguồn điện và lưới điện.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -692,17 +692,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] What are the new changes to Vietnam's PDP8 - A&amp;O Shearman — Vietnam's updated PDP8 outlines new energy priorities and investment opportunities, with key implications for legal, ESG, and infrastructure ...</t>
+          <t>베트남 정부는 2030년까지의 전력 발전 용량을 약 90-100GW로 상향 조정하고 재생 에너지 비중을 확대하는 '수정 PDP8'을 승인했습니다. 이번 계획에는 원자력 발전 재개와 함께 태양광 및 풍력 발전 목표치가 대폭 증가하였으며, 에너지 자립을 위한 루프탑 태양광 보급도 강조되었습니다.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] What are the new changes to Vietnam's PDP8 - A&amp;O Shearman — Vietnam's updated PDP8 outlines new energy priorities and investment opportunities, with key implications for legal, ESG, and infrastructure ...</t>
+          <t>Vietnam has approved the "Amended PDP8," which significantly increases total power capacity targets to nearly 100 GW by 2030 while emphasizing renewable energy and nuclear power. The revised plan introduces mandatory storage batteries for solar projects and outlines a new strategy for exporting renewable energy to neighboring countries like Singapore and Malaysia.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] What are the new changes to Vietnam's PDP8 - A&amp;O Shearman — Vietnam's updated PDP8 outlines new energy priorities and investment opportunities, with key implications for legal, ESG, and infrastructure ...</t>
+          <t>Thủ tướng Chính phủ đã phê duyệt Quy hoạch điện VIII sửa đổi, tăng mục tiêu công suất nguồn điện lên khoảng 90-100 GW vào năm 2030 với sự ưu tiên mạnh mẽ cho năng lượng tái tạo. Bản quy hoạch mới cũng chính thức khởi động lại các dự án điện hạt nhân tại Ninh Thuận và đặt mục tiêu xuất khẩu năng lượng sang các nước láng giềng.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -756,17 +756,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eight National Power Development Plan (PDP8) — The PDP8 presents Vietnam's long-term objective to form an energy ecosystem based on renewable energies. The development of wind and solar power ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>2023년 5월 15일 베트남 정부는 '제8차 국가전력개발계획(PDP8)'을 발표하여 2021~2030년과 2050년 비전을 제시했습니다. PDP8은 석탄 발전 용량을 약 13GW 감축하고, 2050년까지 모든 석탄발전소는 대체 연료로 전환하거나 퇴출하도록 요구합니다. 2030년에는 재생에너지가 전체 발전용량의 48%, 2050년에는 약 63%를 차지할 계획입니다.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eight National Power Development Plan (PDP8) — The PDP8 presents Vietnam's long-term objective to form an energy ecosystem based on renewable energies. The development of wind and solar power ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>On May 15, 2023, the Vietnamese government released the 8th National Power Development Plan (PDP8) covering 2021-2030 and a vision to 2050. The plan cancels about 13GW of planned coal capacity, requires all coal plants to be converted to alternative fuels or shut down by 2050, and aims for renewables to provide 48% of installed capacity by 2030 and about 63% by 2050.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eight National Power Development Plan (PDP8) — The PDP8 presents Vietnam's long-term objective to form an energy ecosystem based on renewable energies. The development of wind and solar power ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Ngày 15/5/2023, Chính phủ Việt Nam đã công bố Quy hoạch Phát triển điện lực quốc gia lần thứ 8 (PDP8) cho giai đoạn 2021-2030, tầm nhìn đến 2050. PDP8 loại bỏ khoảng 13GW điện than, yêu cầu toàn bộ nhà máy điện than phải chuyển đổi sang nhiên liệu thay thế hoặc ngừng hoạt động trước năm 2050 và đặt mục tiêu năng lượng tái tạo chiếm 48% công suất lắp đặt vào năm 2030, và khoảng 63% vào năm 2050.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -820,17 +820,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Revised Power Development Plan VIII — Vietnam's April 2025 revision to Power Development Plan VIII accelerates renewable energy targets and reintroduces nuclear power projects. (관련: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam Revised Power Development Plan VIII</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Revised Power Development Plan VIII — Vietnam's April 2025 revision to Power Development Plan VIII accelerates renewable energy targets and reintroduces nuclear power projects. (Related: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam Revised Power Development Plan VIII</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Revised Power Development Plan VIII — Vietnam's April 2025 revision to Power Development Plan VIII accelerates renewable energy targets and reintroduces nuclear power projects. (Liên quan: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam Revised Power Development Plan VIII</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -880,17 +880,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Power Development Plan 8 (PDP8) - Speeda ASEAN — Vietnam's Power Development Plan 8 (PDP8) sets bold targets for renewables, but coal reliance, pricing, and grid issues challenge its green energy shift. (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남의 제8차 국가전력개발계획(PDP8)은 2050년 탄소 중립 달성을 목표로 화석 연료에서 재생 에너지 중심의 전력 체계로의 전환을 가속화하고 있습니다. 정부는 옥상 태양광 및 직접전력구매계약(DPPA) 도입을 통해 투자를 촉진하고 있으나, 송전망 미비와 가격 책정 프레임워크의 불확실성은 여전히 해결해야 할 과제로 남아 있습니다.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Power Development Plan 8 (PDP8) - Speeda ASEAN — Vietnam's Power Development Plan 8 (PDP8) sets bold targets for renewables, but coal reliance, pricing, and grid issues challenge its green energy shift. (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam's Power Development Plan 8 (PDP8) drives a strategic shift toward renewable energy to achieve net-zero emissions by 2050. While new policies like Direct Power Purchase Agreements (DPPA) and expanded solar incentives are attracting investment, the transition faces hurdles including grid congestion and unsupportive pricing structures.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Power Development Plan 8 (PDP8) - Speeda ASEAN — Vietnam's Power Development Plan 8 (PDP8) sets bold targets for renewables, but coal reliance, pricing, and grid issues challenge its green energy shift. (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Quy hoạch điện VIII (PDP8) của Việt Nam định hướng chuyển đổi chiến lược từ năng lượng hóa thạch sang năng lượng tái tạo nhằm mục tiêu phát thải ròng bằng 0 vào năm 2050. Mặc dù các chính sách như cơ chế mua bán điện trực tiếp (DPPA) và ưu đãi điện mặt trời mái nhà đang mở ra cơ hội đầu tư lớn, ngành năng lượng vẫn đối mặt với thách thức về hạ tầng lưới điện và khung giá điện chưa phù hợp.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -944,17 +944,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Approves Power Development Plan for Cleaner Fuels — Power Development Plan VIII ("PDP8") calls for expansions to renewable energy generation and development of LNG facilities to aid a gradual ... (관련: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 2030년까지 전력 설비 용량을 150GW로 확충하고 2050년 탄소 중립을 달성하기 위한 제8차 국가 전력개발계획(PDP8)을 승인했습니다. 이 계획은 석탄 화력 발전을 점진적으로 폐지하고 해상 풍력 및 LNG 발전 비중을 대폭 확대하기 위해 약 1,347억 달러의 투자를 필요로 합니다.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Approves Power Development Plan for Cleaner Fuels — Power Development Plan VIII ("PDP8") calls for expansions to renewable energy generation and development of LNG facilities to aid a gradual ... (Related: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has approved the Power Development Plan VIII (PDP8), targeting a grid expansion to 150 GW by 2030 and carbon neutrality by 2050. The plan requires $134.7 billion in investment to shift from coal to cleaner energy sources, specifically prioritizing offshore wind and LNG infrastructure.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Approves Power Development Plan for Cleaner Fuels — Power Development Plan VIII ("PDP8") calls for expansions to renewable energy generation and development of LNG facilities to aid a gradual ... (Liên quan: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Quy hoạch điện VIII (PDP8), đặt mục tiêu nâng công suất lưới điện lên 150 GW vào năm 2030 và đạt phát thải ròng bằng 0 vào năm 2050. Kế hoạch này yêu cầu khoản đầu tư 134,7 tỷ USD để chuyển dịch từ điện than sang các nguồn năng lượng sạch hơn như điện gió ngoài khơi và khí LNG.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1008,17 +1008,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's National Power Development Plan For LNG Power Plants — Under PDP8, Vietnam has no plan to develop NEW LNG power plants after 2035. Potential Backup Locations: Thai Binh, Nam Dinh, Nghi Son, Quynh ... (관련: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 PDP8 목표 달성을 위해 LNG 발전소 건설을 가속화하고 있으며, 최근 시행령 제56호(Decree 56)를 통해 연료비 전가 메커니즘과 최소 65%의 전력 구매 보장책을 도입했습니다. 이는 2030년까지 15개의 LNG 발전소를 확보하고 전력 용량을 150,500 MW로 확대하기 위한 조치입니다.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's National Power Development Plan For LNG Power Plants — Under PDP8, Vietnam has no plan to develop NEW LNG power plants after 2035. Potential Backup Locations: Thai Binh, Nam Dinh, Nghi Son, Quynh ... (Related: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>The Vietnamese government has introduced Decree 56 to support the development of 15 LNG power plants under the Amended PDP8, aiming for a total capacity of 150,500 MW by 2030. The new regulations provide a fuel cost pass-through mechanism and a 10-year guarantee for offtaking at least 65% of electricity output to ensure project bankability.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's National Power Development Plan For LNG Power Plants — Under PDP8, Vietnam has no plan to develop NEW LNG power plants after 2035. Potential Backup Locations: Thai Binh, Nam Dinh, Nghi Son, Quynh ... (Liên quan: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã ban hành Nghị định 56 nhằm hỗ trợ phát triển 15 nhà máy điện LNG theo Quy hoạch điện VIII (PDP8) sửa đổi, hướng tới mục tiêu đạt tổng công suất 150.500 MW vào năm 2030. Quy định mới thiết lập cơ chế chuyển tiếp chi phí nhiên liệu và cam kết sản lượng hợp đồng tối thiểu 65% để tháo gỡ khó khăn cho các nhà đầu tư.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1072,17 +1072,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's latest power development plan focuses on expanding ... — Under the draft PDP 8, Vietnam plans to increase solar capacity to 18.6 GW and wind capacity to 18.0 GW by 2030. Vietnam's underdeveloped grid ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부의 제8차 국가전력개발계획(PDP 8) 초안은 2030년까지 태양광 및 풍력 발전 용량을 대폭 확대하고 탄소 배출을 줄이는 것을 목표로 합니다. 특히 노후화된 전력망 문제를 해결하기 위해 고전압 송전선 건설과 인프라 현대화를 우선순위로 두어 재생에너지 통합을 지원할 계획입니다.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's latest power development plan focuses on expanding ... — Under the draft PDP 8, Vietnam plans to increase solar capacity to 18.6 GW and wind capacity to 18.0 GW by 2030. Vietnam's underdeveloped grid ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam's draft Power Development Plan 8 (PDP 8) aims to significantly increase solar and wind capacity to 18.6 GW and 18.0 GW respectively by 2030 to reduce coal dependency. The plan prioritizes grid modernization, including a 461-mile transmission line project, to address current congestion and successfully integrate higher shares of renewable energy.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's latest power development plan focuses on expanding ... — Under the draft PDP 8, Vietnam plans to increase solar capacity to 18.6 GW and wind capacity to 18.0 GW by 2030. Vietnam's underdeveloped grid ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Dự thảo Quy hoạch phát triển điện lực quốc gia 8 (PDP 8) của Việt Nam tập trung vào việc mở rộng công suất điện mặt trời và điện gió lên lần lượt 18,6 GW và 18,0 GW vào năm 2030. Kế hoạch này ưu tiên nâng cấp hạ tầng lưới điện và xây dựng các đường dây truyền tải cao thế để khắc phục tình trạng quá tải và hỗ trợ tích hợp năng lượng tái tạo.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1136,17 +1136,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Foreign investors threaten legal action against Vietnam over ... — Foreign investors may take legal action if Vietnam does not fully pay electricity tariffs agreed with multiple wind and solar projects, ... (관련: VN-PWR-PDP8)</t>
+          <t>베트남 정부가 재생에너지 전력 구매 가격을 소급 삭감하자 한국, EU 등 5개국 상공회의소가 공동 서한을 통해 법적 대응을 예고했습니다. 투자자들은 약속된 보조금이 지급되지 않을 경우 국제 분쟁 해결 절차를 밟을 수 있다고 경고하며 정부의 우호적인 해결책 마련을 촉구했습니다.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Foreign investors threaten legal action against Vietnam over ... — Foreign investors may take legal action if Vietnam does not fully pay electricity tariffs agreed with multiple wind and solar projects, ... (Related: VN-PWR-PDP8)</t>
+          <t>Foreign investors from five major chambers of commerce have threatened legal action against Vietnam due to retroactive cuts in electricity tariffs for wind and solar projects. The dispute involves 12 gigawatts of capacity, with investors warning of potential defaults and multibillion-dollar losses if original payment obligations are not met.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Foreign investors threaten legal action against Vietnam over ... — Foreign investors may take legal action if Vietnam does not fully pay electricity tariffs agreed with multiple wind and solar projects, ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Năm hiệp hội thương mại quốc tế đã cảnh báo sẽ thực hiện các biện pháp pháp lý nếu Chính phủ Việt Nam không thực hiện cam kết về giá mua điện tái tạo. Tranh chấp phát sinh sau khi Việt Nam cắt giảm giá ưu đãi (FIT) đã thỏa thuận trước đó, gây ảnh hưởng đến các dự án có tổng công suất lên tới 12 GW.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1196,17 +1196,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] vietnam energy week 2026 — The event brings together industry leaders, technology providers, and decision-makers to explore advancements shaping Vietnam's digital economy. (관련: VN-EV-2030)</t>
+          <t>베트남 에너지 위크 2026(Vietnam Energy Week 2026)이 2026년 11월 4일부터 6일까지 호치민시 SECC에서 개최되어 에너지 및 기술 인프라 투자 가속화를 위한 전략적 플랫폼 역할을 할 예정입니다. 이번 행사는 단순한 전시를 넘어 투자자, 설계 컨설턴트, MEP 계약자 간의 직접적인 교류를 통해 에너지 및 HVACR 산업의 실질적인 비즈니스 기회 창출에 집중합니다.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] vietnam energy week 2026 — The event brings together industry leaders, technology providers, and decision-makers to explore advancements shaping Vietnam's digital economy. (Related: VN-EV-2030)</t>
+          <t>Vietnam Energy Week 2026 will be held from November 4–6, 2026, at the SECC in Ho Chi Minh City, serving as a strategic hub for accelerated investment in energy and technical infrastructure. The exhibition focuses on high-quality B2B engagement between investors, contractors, and technology partners to drive tangible growth in the Energy and HVACR sectors.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] vietnam energy week 2026 — The event brings together industry leaders, technology providers, and decision-makers to explore advancements shaping Vietnam's digital economy. (Liên quan: VN-EV-2030)</t>
+          <t>Tuần lễ Năng lượng Việt Nam 2026 sẽ diễn ra từ ngày 4 đến 6 tháng 11 năm 2026 tại SECC, TP. Hồ Chí Minh, đóng vai trò là điểm hẹn chiến lược trong giai đoạn đẩy mạnh đầu tư vào hạ tầng năng lượng và kỹ thuật. Triển lãm tập trung vào việc kết nối trực tiếp giữa các nhà đầu tư, nhà thầu và đối tác công nghệ để tạo ra những cơ hội kinh doanh thực chất trong ngành Năng lượng và HVACR.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1260,17 +1260,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] An alternative to urban solar energy | Vietnam Today - YouTube — ... 2026, prioritising renewable energy. But while rooftop solar is expanding, many urban residents lack the space or budget for traditional ... (관련: VN-PWR-PDP8)</t>
+          <t>팜 민 찐 총리는 COP26에서 2050년까지 넷제로 달성을 재확인하며 재생 에너지 발전을 최우선 과제로 설정했습니다. 특히 PDP8 계획에 따라 도시형 태양광 에너지의 대안을 모색하며 에너지 인프라 확충에 집중하고 있습니다.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] An alternative to urban solar energy | Vietnam Today - YouTube — ... 2026, prioritising renewable energy. But while rooftop solar is expanding, many urban residents lack the space or budget for traditional ... (Related: VN-PWR-PDP8)</t>
+          <t>Prime Minister Phạm Minh Chính has reaffirmed Vietnam's commitment to achieving net-zero emissions by 2050, prioritizing the development of renewable energy sources. This initiative aligns with the Power Development Plan 8 (PDP8) to explore alternatives for urban solar energy and enhance the national power infrastructure.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] An alternative to urban solar energy | Vietnam Today - YouTube — ... 2026, prioritising renewable energy. But while rooftop solar is expanding, many urban residents lack the space or budget for traditional ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Thủ tướng Phạm Minh Chính khẳng định lại cam kết của Việt Nam về mức phát thải ròng bằng 0 vào năm 2050 tại COP26, ưu tiên phát triển năng lượng tái tạo. Đây là một phần trong kế hoạch Quy hoạch điện VIII (PDP8) nhằm tìm kiếm giải pháp thay thế cho năng lượng mặt trời đô thị và cải thiện hạ tầng năng lượng.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1324,17 +1324,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Pushes Rooftop Solar and Energy Saving to Secure Power ... — Vietnam accelerates rooftop solar adoption and energy conservation measures to ensure stable power supply and achieve long term climate ... (관련: VN-EV-2030)</t>
+          <t>베트남 팜 민 찐 총리는 국가 에너지 안보를 강화하기 위해 옥상 태양광 발전 확대와 에너지 절약을 강조하는 주요 지침을 발표했습니다. 이 계획은 500kV 회로-3 송전선로와 같은 인프라 구축을 가속화하고 복잡한 절차를 간소화하여 2050년 넷제로 목표 달성을 지원하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Pushes Rooftop Solar and Energy Saving to Secure Power ... — Vietnam accelerates rooftop solar adoption and energy conservation measures to ensure stable power supply and achieve long term climate ... (Related: VN-EV-2030)</t>
+          <t>Prime Minister Pham Minh Chinh has issued a directive to prioritize energy security through the expansion of rooftop solar power and nationwide electricity conservation. The plan focuses on streamlining regulations for self-consumption solar systems and accelerating key infrastructure projects like the 500kV Circuit-3 transmission line to ensure a stable power supply.</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Pushes Rooftop Solar and Energy Saving to Secure Power ... — Vietnam accelerates rooftop solar adoption and energy conservation measures to ensure stable power supply and achieve long term climate ... (Liên quan: VN-EV-2030)</t>
+          <t>Thủ tướng Phạm Minh Chính đã ban hành chỉ thị thúc đẩy an ninh năng lượng thông qua việc mở rộng điện mặt trời áp mái và tăng cường tiết kiệm điện trên toàn quốc. Kế hoạch tập trung vào việc đơn giản hóa thủ tục lắp đặt, đẩy nhanh tiến độ đường dây truyền tải 500kV mạch 3 nhằm đảm bảo cung ứng điện ổn định và hướng tới mục tiêu phát thải ròng bằng 0 vào năm 2050.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1388,17 +1388,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Prime Minister Phạm Minh Chính has reaffirmed Việt Nam's ... — With 100GW of additional capacity forecast by 2030, and a ten-fold increase in renewable energy generation, Vietnam is serious about the future ...</t>
+          <t>베트남 팜 민 찐 총리는 2050년까지 탄소 중립(Net-Zero)을 달성하겠다는 베트남의 의지를 재확인했습니다. 정부는 국가 에너지 전략의 일환으로 청정에너지 전환과 지속 가능한 인프라 구축을 최우선 과제로 추진하고 있습니다.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Prime Minister Phạm Minh Chính has reaffirmed Việt Nam's ... — With 100GW of additional capacity forecast by 2030, and a ten-fold increase in renewable energy generation, Vietnam is serious about the future ...</t>
+          <t>Prime Minister Phạm Minh Chính has reaffirmed Vietnam's commitment to achieving net-zero emissions by 2050. The government is prioritizing the transition to clean energy and the development of sustainable infrastructure as part of its national power and energy strategy.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Prime Minister Phạm Minh Chính has reaffirmed Việt Nam's ... — With 100GW of additional capacity forecast by 2030, and a ten-fold increase in renewable energy generation, Vietnam is serious about the future ...</t>
+          <t>Thủ tướng Phạm Minh Chính đã tái khẳng định cam kết của Việt Nam trong việc đạt mức phát thải ròng bằng 0 vào năm 2050. Chính phủ đang ưu tiên chuyển đổi sang năng lượng sạch và phát triển hạ tầng bền vững như một phần trong chiến lược năng lượng quốc gia.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1452,17 +1452,17 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Gusty growth: Vietnam's remarkable wind energy story - Eco-Business — The country has made substantial investments in renewable energy, particularly wind power, to meet its growing energy demands and reduce ... (관련: VN-PWR-PDP8)</t>
+          <t>베트남은 2030년까지 풍력 발전 용량을 6,000MW로 확대한다는 야심찬 목표를 세우고 비엔투안 및 쭝남 풍력 발전소와 같은 대규모 프로젝트를 추진하고 있습니다. 정부는 육상 및 해상 풍력에 대한 발전차액지원제도(FiT)와 국제적 파트너십을 통해 투자를 유치하고 있으나, 전력망 인프라 개선이 주요 과제로 남아 있습니다.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Gusty growth: Vietnam's remarkable wind energy story - Eco-Business — The country has made substantial investments in renewable energy, particularly wind power, to meet its growing energy demands and reduce ... (Related: VN-PWR-PDP8)</t>
+          <t>Vietnam is rapidly expanding its wind energy sector with a target of 6,000 MW by 2030, supported by significant projects like the Binh Thuan and Trung Nam plants. The government utilizes Feed-in Tariffs (FiT) and international partnerships to drive growth, though challenges in grid infrastructure and regulatory frameworks persist.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Gusty growth: Vietnam's remarkable wind energy story - Eco-Business — The country has made substantial investments in renewable energy, particularly wind power, to meet its growing energy demands and reduce ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Việt Nam đang nhanh chóng mở rộng lĩnh vực năng lượng gió với mục tiêu đạt công suất 6.000 MW vào năm 2030, được hỗ trợ bởi các dự án lớn như nhà máy Bình Thuận và Trung Nam. Chính phủ áp dụng cơ chế giá bán điện (FiT) và hợp tác quốc tế để thúc đẩy đầu tư, dù vẫn còn những thách thức về hạ tầng lưới điện và khung pháp lý.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1516,17 +1516,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Bloomberg Businessweek Vietnam 02.2026 Featured Issue ... — Generous FiTs triggered a surge in solar and wind development, transforming the country from a marginal player into a regional clean energy ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남은 과거 보조금 중심의 급격한 성장에서 벗어나 규제 준수와 시장 중심의 규율을 강조하는 에너지 전환의 새로운 단계에 진입했습니다. 직접전력구매계약(DPPA)과 제8차 국가전력개발계획(PDP8)을 통해 공급과 수요의 균형을 맞추고 전력망 안정을 도모하며 장기적인 투자 신뢰도를 구축하고 있습니다.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Bloomberg Businessweek Vietnam 02.2026 Featured Issue ... — Generous FiTs triggered a surge in solar and wind development, transforming the country from a marginal player into a regional clean energy ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam is transitioning from a period of rapid, subsidy-driven renewable energy growth to a more disciplined, market-based approach under the DPPA framework and PDP8. The focus has shifted from mere development speed to long-term system stability, regulatory compliance, and aligning generation with grid capacity to ensure financial and operational sustainability.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Bloomberg Businessweek Vietnam 02.2026 Featured Issue ... — Generous FiTs triggered a surge in solar and wind development, transforming the country from a marginal player into a regional clean energy ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Việt Nam đang chuyển dịch từ giai đoạn phát triển năng lượng tái tạo nhanh chóng dựa trên trợ giá (FiT) sang mô hình dựa trên kỷ luật thị trường và cơ chế DPPA. Quá trình này ưu tiên tính ổn định của hệ thống, tuân thủ quy định pháp luật và sự phù hợp với Quy hoạch điện VIII (PDP8) thay vì chỉ tập trung vào tốc độ tăng trưởng.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1580,17 +1580,17 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] From boom to balance in Vietnam's clean energy transition - IEEFA — Vietnamese authorities are looking to retroactively revise purchase prices for 173 solar and wind projects, reducing revenues by 25% to 46%, ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남은 제8차 국가전력개발계획(PDP8)에 따라 2030년까지 태양광 73GW 및 육상 풍력 38GW 확보를 목표로 청정에너지 전환을 가속화하고 있습니다. 과거 고정가격매입제도(FiT)의 성공을 발판 삼아, 이제는 직접전력구매계약(DPPA)과 경쟁 입찰 도입을 통해 시장 중심의 지속 가능한 에너지 인프라 구축에 집중하고 있습니다.</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] From boom to balance in Vietnam's clean energy transition - IEEFA — Vietnamese authorities are looking to retroactively revise purchase prices for 173 solar and wind projects, reducing revenues by 25% to 46%, ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam is accelerating its clean energy transition under the revised PDP8, aiming for 73GW of solar and 38GW of onshore wind capacity by 2030. Following a rapid FiT-driven expansion, the sector is now shifting toward sustainable models like Direct Power Purchase Agreements (DPPA) and competitive auctions to ensure financial stability for the state utility.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] From boom to balance in Vietnam's clean energy transition - IEEFA — Vietnamese authorities are looking to retroactively revise purchase prices for 173 solar and wind projects, reducing revenues by 25% to 46%, ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Việt Nam đang đẩy nhanh quá trình chuyển đổi năng lượng sạch theo Quy hoạch điện VIII (PDP8) sửa đổi, hướng tới mục tiêu 73GW điện mặt trời và 38GW điện gió trên bãi vào năm 2030. Sau giai đoạn bùng nổ nhờ giá FiT, ngành năng lượng đang chuyển sang các mô hình bền vững hơn như cơ chế mua bán điện trực tiếp (DPPA) và đấu thầu cạnh tranh để đảm bảo an ninh tài chính.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Solar Energy Market Growth and Forecast (2026-2035) — The Vietnam solar energy market, valued at approximately 26.22 terawatt-hours (TWh) in 2025, is projected to grow at a compound annual ...</t>
+          <t>베트남 태양광 에너지 시장은 2025년 약 26.22 TWh 규모에서 2035년까지 연평균 3.10% 성장하여 35.58 TWh에 도달할 것으로 전망됩니다. 정부의 우호적인 정책, 하락하는 태양광 패널 비용, 그리고 청정 에너지에 대한 수요 증가가 시장 성장을 주도하고 있으나 그리드 통합 및 정책적 불확실성은 해결해야 할 과제로 남아있습니다.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Solar Energy Market Growth and Forecast (2026-2035) — The Vietnam solar energy market, valued at approximately 26.22 terawatt-hours (TWh) in 2025, is projected to grow at a compound annual ...</t>
+          <t>The Vietnam solar energy market is projected to grow from 26.22 TWh in 2025 to 35.58 TWh by 2035, driven by a CAGR of 3.10%. Key growth factors include government incentives like feed-in tariffs, declining equipment costs, and rising demand for sustainable energy alternatives despite challenges in grid stability and land availability.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Solar Energy Market Growth and Forecast (2026-2035) — The Vietnam solar energy market, valued at approximately 26.22 terawatt-hours (TWh) in 2025, is projected to grow at a compound annual ...</t>
+          <t>Thị trường năng lượng mặt trời Việt Nam dự kiến đạt quy mô 35,58 TWh vào năm 2035 với tốc độ tăng trưởng hàng năm kép là 3,10% từ năm 2026. Sự tăng trưởng này được thúc đẩy bởi các chính sách ưu đãi của chính phủ, chi phí lắp đặt giảm và nhu cầu chuyển đổi sang năng lượng sạch, mặc dù vẫn còn những thách thức về hạ tầng lưới điện.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1704,17 +1704,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM - WIND ENERGY INVESTMENT GUIDE 2026 - Slideshare — VIETNAM - WIND ENERGY INVESTMENT GUIDE 2026 - WHAT YOU MUST KNOW - Download as a PDF or view online for free.</t>
+          <t>베트남은 제8차 국가전력개발계획(PDP8)에 따라 2030년까지 해상풍력 6GW 달성을 목표로 에너지 전환을 가속화하고 있으나, 최근 독일 PNE AG의 탈락 사례에서 보듯 자국 기업 우선 정책이 강화되고 있습니다. 외국인 투자자는 엄격한 자본금 요건과 현지 파트너십 의무화 등 변화하는 규제 환경과 금융 담보 요구에 대비해야 합니다.</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM - WIND ENERGY INVESTMENT GUIDE 2026 - Slideshare — VIETNAM - WIND ENERGY INVESTMENT GUIDE 2026 - WHAT YOU MUST KNOW - Download as a PDF or view online for free.</t>
+          <t>Vietnam is accelerating its energy transition under Power Development Plan VIII (PDP8), targeting 6GW of offshore wind by 2030, though recent shifts favor domestic "National Champions" over foreign developers. Investors face stricter financial deposit requirements and a de facto necessity for local partnerships to navigate regulatory uncertainty and grid connection bottlenecks.</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM - WIND ENERGY INVESTMENT GUIDE 2026 - Slideshare — VIETNAM - WIND ENERGY INVESTMENT GUIDE 2026 - WHAT YOU MUST KNOW - Download as a PDF or view online for free.</t>
+          <t>Việt Nam đang đẩy mạnh chuyển dịch năng lượng theo Quy hoạch điện VIII với mục tiêu đạt 6GW điện gió ngoài khơi vào năm 2030, nhưng xu hướng hiện tại cho thấy sự ưu tiên rõ rệt đối với các tập đoàn nội địa. Các nhà đầu tư nước ngoài cần chuẩn bị cho các yêu cầu khắt khe về ký quỹ tài chính, bắt buộc liên doanh với đối tác trong nước và đối mặt với rủi ro vận hành lưới điện.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1768,17 +1768,17 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam LNG Power Project Eyes Green Pivot on Soaring Gas Prices — Vingroup JSC has asked the Vietnamese government to replace a large liquefied natural gas power project with renewable energy due to surging ... (관련: VN-GAS-PDP8)</t>
+          <t>빈그룹(Vingroup)은 중동 분쟁으로 인한 LNG 가격 급등과 수급 불안정을 이유로 하이퐁 LNG 발전 프로젝트를 재생 가능 에너지로 전환해달라고 베트남 정부에 요청했습니다. 이는 수입 연료 의존도가 높은 에너지 인프라의 리스크를 줄이기 위한 결정으로 풀이됩니다.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam LNG Power Project Eyes Green Pivot on Soaring Gas Prices — Vingroup JSC has asked the Vietnamese government to replace a large liquefied natural gas power project with renewable energy due to surging ... (Related: VN-GAS-PDP8)</t>
+          <t>Vingroup JSC has requested the Vietnamese government to pivot its Haiphong LNG-to-power project toward renewable energy due to soaring gas prices and supply disruptions. The decision follows rising costs and competition in the LNG market linked to Middle East conflicts and Qatari supply issues.</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam LNG Power Project Eyes Green Pivot on Soaring Gas Prices — Vingroup JSC has asked the Vietnamese government to replace a large liquefied natural gas power project with renewable energy due to surging ... (Liên quan: VN-GAS-PDP8)</t>
+          <t>Tập đoàn Vingroup đã đề xuất Chính phủ cho phép chuyển đổi dự án điện khí LNG tại Hải Phòng sang năng lượng tái tạo do giá nhiên liệu tăng cao từ các xung đột tại Trung Đông. Quyết định này nhằm giảm thiểu rủi ro phụ thuộc vào nguồn khí nhập khẩu đang gặp khó khăn về nguồn cung từ Qatar.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1832,17 +1832,17 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam awards $974 million LNG power plant construction contract ... — Vietnam's state utility EVN has awarded a contract worth $974 million to a consortium of PowerChina and Lilama for building an LNG-fired ... (관련: VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>베트남 전력공사(EVN)가 9억 7,400만 달러 규모의 꽝짝 II LNG 발전소 건설 계약을 PowerChina와 Lilama 컨소시엄에 수주했습니다. 이 발전소는 1,612MW 규모로 GE Vernova의 터빈을 사용하며, 베트남의 에너지 안보 확보와 2050년 넷제로 목표 달성을 위해 2030년까지 가동될 예정입니다.</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam awards $974 million LNG power plant construction contract ... — Vietnam's state utility EVN has awarded a contract worth $974 million to a consortium of PowerChina and Lilama for building an LNG-fired ... (Related: VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Vietnam's state utility EVN has awarded a $974 million contract to a PowerChina and Lilama consortium to build the 1,612 MW Quang Trach II LNG-fired power plant. The facility, which will utilize GE Vernova turbines, is slated to be fully operational by 2030 to bolster energy security and support Vietnam's net-zero emissions commitments.</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam awards $974 million LNG power plant construction contract ... — Vietnam's state utility EVN has awarded a contract worth $974 million to a consortium of PowerChina and Lilama for building an LNG-fired ... (Liên quan: VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Tập đoàn Điện lực Việt Nam (EVN) đã trao hợp đồng trị giá 974 triệu USD cho liên danh PowerChina và Lilama để xây dựng nhà máy điện khí LNG Quảng Trạch II công suất 1.612 MW. Nhà máy sẽ sử dụng tuabin của General Electric Vernova và dự kiến đi vào hoạt động đầy đủ vào năm 2030 nhằm đảm bảo an ninh năng lượng và thực hiện cam kết phát thải ròng bằng không.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1896,17 +1896,17 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam moves to cement LNG supply chain as power demand surges — Vietnam is stepping up efforts to build a national LNG supply chain, as PV Gas signed a series of agreements with Vietnam Electricity (EVN) ... (관련: VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>PV Gas는 베트남 전력공사(EVN) 및 PV Power와 대규모 가스 발전 프로젝트를 위한 LNG 공급 협약을 체결했습니다. 이번 계약에는 하틴성 붕앙 터미널에서 광짝 발전소로의 가스 공급과 년짝 3, 4호기에 대한 25년 장기 공급이 포함되어 통합 LNG 생태계 구축을 가속화합니다.</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam moves to cement LNG supply chain as power demand surges — Vietnam is stepping up efforts to build a national LNG supply chain, as PV Gas signed a series of agreements with Vietnam Electricity (EVN) ... (Related: VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>PV Gas has signed strategic agreements with EVN and PV Power to supply LNG for major power complexes, including Quang Trach 2 &amp; 3 and Nhon Trach 3 &amp; 4. This move establishes an integrated LNG supply chain to address declining domestic gas reserves and meet Vietnam's surging electricity demand through 2030.</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam moves to cement LNG supply chain as power demand surges — Vietnam is stepping up efforts to build a national LNG supply chain, as PV Gas signed a series of agreements with Vietnam Electricity (EVN) ... (Liên quan: VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>PV Gas đã ký kết các thỏa thuận với EVN và PV Power để cung cấp LNG cho các dự án điện quy mô lớn như tổ hợp Quảng Trạch và Nhơn Trạch 3 &amp; 4. Việc này giúp hình thành chuỗi cung ứng LNG tích hợp, đảm bảo an ninh năng lượng trong bối cảnh sản lượng khí nội địa suy giảm và nhu cầu điện tăng cao.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1960,17 +1960,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] POWERCHINA signs SE Asia's largest LNG power project in Vietnam — The project will play a pivotal role in advancing Vietnam's energy transition from a coal-dominated mix to one centered on natural gas and ... (관련: VN-GAS-PDP8)</t>
+          <t>베트남 전력공사(EVN)는 POWERCHINA 및 Lilama 컨소시엄과 꽝짝 II LNG 화력발전소 건설을 위한 EPC 턴키 계약을 체결했습니다. 베트남 제8차 국가전력개발계획(PDP8)의 핵심 프로젝트인 이 발전소는 1,612.8MW 규모로 완공 시 연간 약 100억 kWh의 전력을 공급할 예정입니다.</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] POWERCHINA signs SE Asia's largest LNG power project in Vietnam — The project will play a pivotal role in advancing Vietnam's energy transition from a coal-dominated mix to one centered on natural gas and ... (Related: VN-GAS-PDP8)</t>
+          <t>Vietnam Electricity Corporation has signed an EPC turnkey contract with a joint venture of POWERCHINA and Lilama for the Quang Trach II LNG Thermal Power Plant. As a flagship project under Vietnam's Eighth National Power Development Plan (PDP8), this 1,612.8MW facility will be the country's largest LNG power project and is expected to provide 10 billion kWh of electricity annually.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] POWERCHINA signs SE Asia's largest LNG power project in Vietnam — The project will play a pivotal role in advancing Vietnam's energy transition from a coal-dominated mix to one centered on natural gas and ... (Liên quan: VN-GAS-PDP8)</t>
+          <t>Tập đoàn Điện lực Việt Nam đã ký hợp đồng EPC với liên danh POWERCHINA và Lilama cho dự án Nhà máy Nhiệt điện LNG Quảng Trạch II. Đây là dự án trọng điểm thuộc Quy hoạch điện VIII, với công suất 1.612,8MW và dự kiến cung cấp khoảng 10 tỷ kWh điện mỗi năm cho lưới điện quốc gia.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2024,17 +2024,17 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's 1.6GW LNG Power Plants Enter Commercial Operation — VIETNAM'S FIRST LNG POWER PLANTS OFFICIALLY BEGIN COMMERCIAL OPERATION On January 5, 2026, Nhon Trach 3 &amp; 4 – the first LNG-fired power ... (관련: VN-GAS-PDP8)</t>
+          <t>베트남 최초의 LNG 발전소인 년짝(Nhon Trach) 3, 4호기가 2026년 1월 5일 공식적으로 상업 운전을 시작했습니다. 이 발전소는 총 1.6GW의 용량을 갖추고 있으며 매년 90억 kWh 이상의 전력을 공급하여 베트남 남부의 에너지 안보를 강화하고 탄소 배출을 60% 줄일 것으로 기대됩니다.</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's 1.6GW LNG Power Plants Enter Commercial Operation — VIETNAM'S FIRST LNG POWER PLANTS OFFICIALLY BEGIN COMMERCIAL OPERATION On January 5, 2026, Nhon Trach 3 &amp; 4 – the first LNG-fired power ... (Related: VN-GAS-PDP8)</t>
+          <t>Nhon Trach 3 &amp; 4, Vietnam’s first LNG-fired power plants with a total capacity of 1.6GW, officially entered commercial operation on January 5, 2026. Invested by PV Power, these plants utilize advanced H-class turbine technology to provide over 9 billion kWh annually while significantly reducing carbon emissions compared to coal.</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's 1.6GW LNG Power Plants Enter Commercial Operation — VIETNAM'S FIRST LNG POWER PLANTS OFFICIALLY BEGIN COMMERCIAL OPERATION On January 5, 2026, Nhon Trach 3 &amp; 4 – the first LNG-fired power ... (Liên quan: VN-GAS-PDP8)</t>
+          <t>Vào ngày 5 tháng 1 năm 2026, nhà máy điện Nhơn Trạch 3 và 4 - những nhà máy điện khí LNG đầu tiên tại Việt Nam do PV Power đầu tư - đã chính thức đi vào vận hành thương mại. Với tổng công suất hơn 1,6 GW, dự án dự kiến cung cấp hơn 9 tỷ kWh mỗi năm, giúp đảm bảo an ninh năng lượng và giảm 60% lượng khí thải carbon so với điện than.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2088,17 +2088,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam commissions its first LNG-fired power project, and one of ... — Vietnam commissions its first LNG-fired power project, and one of south-east Asia's biggest oil discoveries is confirmed. 14/1/2026. News. (관련: VN-GAS-PDP8)</t>
+          <t>베트남 최초의 LNG 복합화력발전소인 Nhon Trach 3, 4호기가 상업 운전을 시작했으며, 이는 제8차 국가전력개발계획(PDP8)에 따라 2030년까지 LNG 발전 용량을 22GW로 확대하려는 전략의 핵심입니다. 동시에 머피 오일(Murphy Oil)은 구룡 분지에서 지난 20년 내 동남아시아 최대 규모로 추정되는 주요 원유 매장지를 발견하여 국가 에너지 안보를 강화하고 있습니다.</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam commissions its first LNG-fired power project, and one of ... — Vietnam commissions its first LNG-fired power project, and one of south-east Asia's biggest oil discoveries is confirmed. 14/1/2026. News. (Related: VN-GAS-PDP8)</t>
+          <t>Vietnam has launched commercial operations at its first LNG-fired power plants, Nhon Trach 3 and 4, aligning with the PDP8 goal to reach 22 GW of LNG capacity by 2030. Additionally, Murphy Oil confirmed a massive oil discovery at the Hai Su Vang prospect, marking one of Southeast Asia's largest finds in two decades and potentially reversing the country's declining oil production.</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam commissions its first LNG-fired power project, and one of ... — Vietnam commissions its first LNG-fired power project, and one of south-east Asia's biggest oil discoveries is confirmed. 14/1/2026. News. (Liên quan: VN-GAS-PDP8)</t>
+          <t>Việt Nam đã chính thức đưa vào vận hành thương mại nhà máy điện khí LNG đầu tiên là Nhơn Trạch 3 và 4, phù hợp với Quy hoạch điện VIII nhằm đạt mục tiêu 22 GW điện khí vào năm 2030. Bên cạnh đó, Murphy Oil đã xác nhận một phát hiện dầu khí lớn tại mỏ Hải Sư Vàng, được đánh giá là một trong những phát hiện lớn nhất Đông Nam Á trong 20 năm qua.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2152,17 +2152,17 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Signs $974 Million LNG Deal To Strengthen Energy Security — State utility Electricity of Vietnam has awarded a construction contract worth $974 million to a consortium led by PowerChina and Lilama. (관련: VN-GAS-PDP8)</t>
+          <t>베트남 전력공사(EVN)가 에너지 안보와 2050년 넷제로 목표 달성을 위해 9억 7,400만 달러 규모의 꽝짝 II LNG 발전소 건설 계약을 체결했습니다. PowerChina와 Lilama 컨소시엄이 주도하는 이 1,612MW 규모의 프로젝트는 급증하는 산업용 전력 수요를 충족하고 석탄 의존도를 낮추는 가교 역할을 할 것입니다.</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Signs $974 Million LNG Deal To Strengthen Energy Security — State utility Electricity of Vietnam has awarded a construction contract worth $974 million to a consortium led by PowerChina and Lilama. (Related: VN-GAS-PDP8)</t>
+          <t>Vietnam's state utility EVN has awarded a $974 million contract to a PowerChina-led consortium for the 1,612 MW Quang Trach II LNG power plant. This strategic infrastructure project serves as a transitional bridge to support rapid economic growth while aligning with the country's 2050 net-zero emissions commitment.</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Signs $974 Million LNG Deal To Strengthen Energy Security — State utility Electricity of Vietnam has awarded a construction contract worth $974 million to a consortium led by PowerChina and Lilama. (Liên quan: VN-GAS-PDP8)</t>
+          <t>Tập đoàn Điện lực Việt Nam (EVN) đã ký hợp đồng trị giá 974 triệu USD với liên danh PowerChina và Lilama để xây dựng nhà máy điện khí LNG Quảng Trạch II công suất 1.612 MW. Dự án này đóng vai trò quan trọng trong việc đảm bảo an ninh năng lượng và hỗ trợ lộ trình phát thải ròng bằng 0 vào năm 2050 của Việt Nam.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2216,17 +2216,17 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam inaugurates USD1.4 billion LNG power plants in energy ... — LNG-fired electricity generation reduces carbon emissions by roughly 40 per cent compared with coal and 30 per cent compared with oil, ... (관련: VN-PWR-PDP8, VN-GAS-PDP8)</t>
+          <t>베트남은 동나이성에 총 1624MW 규모의 첫 액체천연가스(LNG) 발전소인 년짝 3, 4호기를 14억 달러를 투입하여 완공했습니다. 이 시설은 국가 전력 발전 계획에 따른 향후 13개 LNG 프로젝트의 모델이 되어 남부 지역의 전력망 안정화와 2050년 탄소 중립 목표 달성을 지원할 예정입니다.</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam inaugurates USD1.4 billion LNG power plants in energy ... — LNG-fired electricity generation reduces carbon emissions by roughly 40 per cent compared with coal and 30 per cent compared with oil, ... (Related: VN-PWR-PDP8, VN-GAS-PDP8)</t>
+          <t>Vietnam has inaugurated its first LNG power plants, the Nhon Trach 3 and 4 facilities in Dong Nai Province, built by Petrovietnam with a $1.4 billion investment. These plants provide a combined 1,624 MW capacity to stabilize the grid and serve as a template for 13 additional LNG projects under the national power development plan.</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam inaugurates USD1.4 billion LNG power plants in energy ... — LNG-fired electricity generation reduces carbon emissions by roughly 40 per cent compared with coal and 30 per cent compared with oil, ... (Liên quan: VN-PWR-PDP8, VN-GAS-PDP8)</t>
+          <t>Việt Nam đã khánh thành hai nhà máy điện khí LNG đầu tiên là Nhơn Trạch 3 và Nhơn Trạch 4 tại tỉnh Đồng Nai với tổng vốn đầu tư 1,4 tỷ USD. Dự án có tổng công suất 1.624 MW này đóng vai trò quan trọng trong việc đảm bảo an ninh năng lượng quốc gia và là hình mẫu cho 13 dự án LNG tiếp theo trong quy hoạch điện lực.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2280,17 +2280,17 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam targets saving at least 3% of total power consumption in 2026 — Vietnam is striving to save at least three percent of the total national electricity consumption in 2026.</t>
+          <t>베트남은 2026년까지 전체 전력 소비량의 최소 3%를 절감하는 것을 목표로 하고 있습니다. 이 계획은 전력 및 에너지 부문의 효율성을 높이기 위한 전략적 인프라 정책의 일환입니다.</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam targets saving at least 3% of total power consumption in 2026 — Vietnam is striving to save at least three percent of the total national electricity consumption in 2026.</t>
+          <t>Vietnam aims to save at least 3% of its total power consumption by 2026 as part of its energy efficiency strategy. This target is integrated into the national power and energy sector infrastructure planning to ensure sustainable development.</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam targets saving at least 3% of total power consumption in 2026 — Vietnam is striving to save at least three percent of the total national electricity consumption in 2026.</t>
+          <t>Việt Nam đặt mục tiêu tiết kiệm ít nhất 3% tổng điện năng tiêu thụ vào năm 2026. Đây là một phần trong kế hoạch phát triển hạ tầng ngành điện và năng lượng nhằm tối ưu hóa việc sử dụng tài nguyên.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2344,17 +2344,17 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam targets January 2026 agreement with Russia to revive ... — Vietnam targets January 2026 agreement with Russia to revive nuclear power plans after Japan exit · Vietnam's Prime Minister has urged his ... (관련: VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam targets January 2026 agreement with Russia to revive ...</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam targets January 2026 agreement with Russia to revive ... — Vietnam targets January 2026 agreement with Russia to revive nuclear power plans after Japan exit · Vietnam's Prime Minister has urged his ... (Related: VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam targets January 2026 agreement with Russia to revive ...</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam targets January 2026 agreement with Russia to revive ... — Vietnam targets January 2026 agreement with Russia to revive nuclear power plans after Japan exit · Vietnam's Prime Minister has urged his ... (Liên quan: VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam targets January 2026 agreement with Russia to revive ...</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2408,17 +2408,17 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-based energy company seeks smart-grid and power ... — It is seeking technology partners offering smart-grid and advanced solutions for transmission, distribution, and renewable energy systems under ... (관련: VN-PWR-PDP8)</t>
+          <t>베트남의 한 신재생 에너지 엔지니어링 기업이 송배전 및 재생 에너지 시스템을 위한 스마트 그리드와 고급 기술 솔루션을 보유한 국제 파트너를 찾고 있습니다. 이 협력은 베트남의 제8차 국가전력개발계획(PDP8) 목표에 부합하며, 전력망의 운영 신뢰성을 높이고 자산 관리를 최적화하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-based energy company seeks smart-grid and power ... — It is seeking technology partners offering smart-grid and advanced solutions for transmission, distribution, and renewable energy systems under ... (Related: VN-PWR-PDP8)</t>
+          <t>A Vietnamese renewable energy company is seeking international partners to provide smart-grid and advanced technology solutions for power transmission and distribution systems. Aligned with the VN-PWR-PDP8 objectives, this partnership aims to improve grid reliability and optimize asset management through commercial or technical cooperation agreements.</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-based energy company seeks smart-grid and power ... — It is seeking technology partners offering smart-grid and advanced solutions for transmission, distribution, and renewable energy systems under ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Một công ty năng lượng tái tạo tại Việt Nam đang tìm kiếm đối tác quốc tế cung cấp các giải pháp lưới điện thông minh và công nghệ tiên tiến cho hệ thống truyền tải và phân phối điện. Phù hợp với định hướng Quy hoạch điện VIII (PDP8), sự hợp tác này tập trung vào việc cải thiện độ tin cậy vận hành và tối ưu hóa quản lý tài sản năng lượng.</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2468,17 +2468,17 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam: Power Sector Snapshot - Norton Rose Fulbright — Vietnam expects to focus on a build out of a smart grid capable of ... Việt Nam outlines three 2026 power supply scenarios amid growing electricity demand. (관련: VN-PWR-PDP8)</t>
+          <t>베트남은 2025년 4월 승인된 개정 제8차 국가전력개발계획(PDP8)에 따라 LNG, 재생에너지 및 원자력 발전을 포함한 에너지 믹스 확대를 추진하고 있습니다. 이번 계획은 BESS 용량을 최대 16,300MW로 늘리고 직접전력구매계약(DPPA) 도입을 통해 시장 중심의 전력 공급 체계를 구축하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam: Power Sector Snapshot - Norton Rose Fulbright — Vietnam expects to focus on a build out of a smart grid capable of ... Việt Nam outlines three 2026 power supply scenarios amid growing electricity demand. (Related: VN-PWR-PDP8)</t>
+          <t>Vietnam has updated its Power Development Plan 8 (PDP8) to aggressively expand LNG, solar, wind, and nuclear energy capacity to meet surging electricity demand. The revised framework introduces market-based pricing, supports Direct Power Purchase Agreements (DPPAs), and significantly increases targets for Battery Energy Storage Systems (BESS) to ensure grid stability.</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam: Power Sector Snapshot - Norton Rose Fulbright — Vietnam expects to focus on a build out of a smart grid capable of ... Việt Nam outlines three 2026 power supply scenarios amid growing electricity demand. (Liên quan: VN-PWR-PDP8)</t>
+          <t>Việt Nam đã phê duyệt điều chỉnh Quy hoạch điện VIII (PDP8) với mục tiêu đẩy mạnh phát triển điện khí LNG, năng lượng tái tạo và tái khởi động điện hạt nhân. Các chính sách mới tập trung vào cơ chế mua bán điện trực tiếp (DPPA), phát triển hệ thống lưu trữ năng lượng (BESS) và cải thiện tính khả thi về tài chính cho các dự án năng lượng.</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2528,17 +2528,17 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] [PDF] Development of Vietnam Smart Grid Roadmap for period up to year ... — The Updated Smart Grid Roadmap will benefit key stakeholders, including ERAV, Electricity of Viet. Nam (EVN), power generation companies, transmission and ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남은 2050년 넷제로 배출 목표와 제8차 전력개발계획(PDP8)에 발맞추어 2030년까지의 스마트 그리드 로드맵을 업데이트했습니다. 이 계획은 송전망 현대화, 신재생 에너지 통합, 변전소 자동화 및 사이버 보안 강화를 우선순위로 두며, 장기적으로는 전기차 충전 인프라와 가상 발전소(VPP) 도입을 지원합니다.</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] [PDF] Development of Vietnam Smart Grid Roadmap for period up to year ... — The Updated Smart Grid Roadmap will benefit key stakeholders, including ERAV, Electricity of Viet. Nam (EVN), power generation companies, transmission and ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has updated its Smart Grid Development Roadmap to 2030 with a vision to 2050 to align with PDP8 and Net Zero commitments. The plan prioritizes grid modernization, substation automation, and SCADA/EMS upgrades to integrate renewable energy, while also establishing frameworks for electric vehicle integration and advanced metering infrastructure.</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] [PDF] Development of Vietnam Smart Grid Roadmap for period up to year ... — The Updated Smart Grid Roadmap will benefit key stakeholders, including ERAV, Electricity of Viet. Nam (EVN), power generation companies, transmission and ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Việt Nam đã cập nhật Lộ trình phát triển Lưới điện thông minh đến năm 2030, tầm nhìn đến năm 2050 nhằm phù hợp với Quy hoạch điện VIII và cam kết Net Zero. Kế hoạch tập trung ưu tiên hiện đại hóa hệ thống điều khiển, tự động hóa trạm biến áp và tăng cường an ninh mạng để tích hợp năng lượng tái tạo, đồng thời chuẩn bị hạ tầng cho xe điện và các nguồn năng lượng phân tán.</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2592,17 +2592,17 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Plugging nuclear energy safely into Vietnam's grid - RMIT University — Vietnam's new Law on Atomic Energy, effective 1 January 2026, sets strict safety and licensing standards aligned with the International Atomic ... (관련: VN-REN-NPP-2050)</t>
+          <t>베트남은 2026년 1월 발효된 새로운 원자력법을 통해 2050년까지 원자력 발전 용량을 최대 14,000MW로 확대할 계획입니다. RMIT 대학 전문가들은 이 목표를 달성하기 위해 차세대 원자로(SMR 등) 도입과 함께 전력망 강화 및 전문 인력 양성이 필수적이라고 강조합니다.</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Plugging nuclear energy safely into Vietnam's grid - RMIT University — Vietnam's new Law on Atomic Energy, effective 1 January 2026, sets strict safety and licensing standards aligned with the International Atomic ... (Related: VN-REN-NPP-2050)</t>
+          <t>Vietnam's new Atomic Energy Law, effective 2026, paves the way for advanced nuclear technologies to reach a target capacity of 14,000 MW by 2050. Experts from RMIT Vietnam state that success depends on integrating these plants into the national grid and developing a robust safety culture and skilled workforce.</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Plugging nuclear energy safely into Vietnam's grid - RMIT University — Vietnam's new Law on Atomic Energy, effective 1 January 2026, sets strict safety and licensing standards aligned with the International Atomic ... (Liên quan: VN-REN-NPP-2050)</t>
+          <t>Luật Năng lượng nguyên tử mới của Việt Nam có hiệu lực từ năm 2026, mở đường cho việc phát triển điện hạt nhân với mục tiêu đạt công suất 14.000 MW vào năm 2050. Các chuyên gia từ RMIT nhấn mạnh rằng sự thành công sẽ phụ thuộc vào khả năng sẵn sàng của lưới điện, cơ sở hạ tầng kỹ thuật và việc đào tạo nguồn nhân lực chuyên môn cao.</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2652,17 +2652,17 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Green Hydrogen: A Pathway to Vietnam's Energy Security - MDPI — The study summarizes the energy landscape of Vietnam in Section 2 and addresses the role of green hydrogen in Vietnam's energy transition in Section 3. The ... (관련: VN-REN-NPP-2050)</t>
+          <t>베트남 정부는 2050년 탄소 중립 달성을 위해 그린 수소 에너지 개발 전략(HEDS)을 발표했으며, 이는 국가 전력 개발 계획(PDP8)과 연계됩니다. 풍부한 태양광 및 풍력 자원을 활용하여 수소를 생산함으로써 화석 연료 의존도를 낮추고 국가 에너지 안보를 강화하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Green Hydrogen: A Pathway to Vietnam's Energy Security - MDPI — The study summarizes the energy landscape of Vietnam in Section 2 and addresses the role of green hydrogen in Vietnam's energy transition in Section 3. The ... (Related: VN-REN-NPP-2050)</t>
+          <t>The Vietnamese government has launched its Hydrogen Energy Development Strategy (HEDS) to 2030 with a vision to 2050, aiming to integrate green hydrogen into the national power system (PDP8). By leveraging its vast solar and wind potential, Vietnam seeks to decarbonize heavy industries and transportation while ensuring long-term energy security.</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Green Hydrogen: A Pathway to Vietnam's Energy Security - MDPI — The study summarizes the energy landscape of Vietnam in Section 2 and addresses the role of green hydrogen in Vietnam's energy transition in Section 3. The ... (Liên quan: VN-REN-NPP-2050)</t>
+          <t>Chính phủ Việt Nam đã ban hành Chiến lược phát triển năng lượng hydrogen đến năm 2030, tầm nhìn đến năm 2050 nhằm hiện thực hóa mục tiêu phát thải ròng bằng không. Chiến lược này tập trung khai thác tiềm năng năng lượng tái tạo dồi dào để sản xuất hydro xanh, giúp giảm phụ thuộc vào nhiên liệu hóa thạch và đảm bảo an ninh năng lượng quốc gia.</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2716,17 +2716,17 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM-RESOLUTION 70-NQ/TW-2025 FACILITATES CAPITAL ... — Nuclear Power Development: Urges expedited implementation of the Ninh Thuận 1 and 2 nuclear power plants by 2030–2035, with opportunities for ... (관련: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>베트남 정치국은 2030년까지 국가 에너지 안보를 보장하기 위한 결의안 제70-NQ/TW호를 발표하고 민간 및 외국인 투자를 가로막는 제도적 장벽을 제거하기로 했습니다. 이 결의안은 재생 에너지 비중을 30%까지 확대하고 닌투언 원자력 발전소 건설을 재개하는 등 에너지 믹스 다양화와 탄소 중립 목표 달성을 강조합니다.</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM-RESOLUTION 70-NQ/TW-2025 FACILITATES CAPITAL ... — Nuclear Power Development: Urges expedited implementation of the Ninh Thuận 1 and 2 nuclear power plants by 2030–2035, with opportunities for ... (Related: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam's Politburo has issued Resolution 70-NQ/TW to enhance national energy security by 2030, specifically targeting the removal of institutional barriers to attract private and international capital. The directive prioritizes renewable energy growth, smart grid development, and the expedited revival of nuclear power projects like Ninh Thuan 1 and 2.</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM-RESOLUTION 70-NQ/TW-2025 FACILITATES CAPITAL ... — Nuclear Power Development: Urges expedited implementation of the Ninh Thuận 1 and 2 nuclear power plants by 2030–2035, with opportunities for ... (Liên quan: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Bộ Chính trị đã ban hành Nghị quyết 70-NQ/TW nhằm đảm bảo an ninh năng lượng quốc gia đến năm 2030, tập trung tháo gỡ các rào cản thể chế để thu hút vốn đầu tư tư nhân và quốc tế. Nghị quyết ưu tiên phát triển năng lượng tái tạo chiếm 25-30% tổng cung và thúc đẩy triển khai các dự án điện hạt nhân Ninh Thuận 1 và 2 trong giai đoạn 2030-2035.</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2776,17 +2776,17 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Smart Grids for Renewable Energy and Energy Efficiency - ESP — The 'Smart Grids for Renewable Energy and Energy Efficiency (SGREEE)' project is supporting the Government of Viet Nam in the implementation of its Smart Grid ... (관련: VN-PWR-PDP8)</t>
+          <t>독일 경제협력개발부(BMZ)가 자금을 지원하는 SGREEE 프로젝트는 베트남 전력 규제청(ERAV)과 협력하여 국가 전력망의 현대화와 자동화를 추진하고 있습니다. 이 사업은 재생 에너지 통합을 확대하고 에너지 효율을 높이기 위한 스마트 그리드 로드맵 이행과 전력 시스템의 디지털화를 지원합니다.</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Smart Grids for Renewable Energy and Energy Efficiency - ESP — The 'Smart Grids for Renewable Energy and Energy Efficiency (SGREEE)' project is supporting the Government of Viet Nam in the implementation of its Smart Grid ... (Related: VN-PWR-PDP8)</t>
+          <t>The SGREEE project, funded by BMZ and partnered with ERAV, supports the modernization and automation of Vietnam's national power grid. It focuses on implementing the Smart Grid Roadmap to facilitate the integration of renewable energy and enhance energy efficiency through digitalization and system flexibility.</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Smart Grids for Renewable Energy and Energy Efficiency - ESP — The 'Smart Grids for Renewable Energy and Energy Efficiency (SGREEE)' project is supporting the Government of Viet Nam in the implementation of its Smart Grid ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Dự án SGREEE, do BMZ tài trợ và hợp tác với ERAV, hỗ trợ Chính phủ Việt Nam hiện đại hóa và tự động hóa hệ thống truyền tải và phân phối điện quốc gia. Dự án tập trung vào việc thực hiện Lộ trình Lưới điện thông minh nhằm tích hợp năng lượng tái tạo và nâng cao hiệu quả năng lượng thông qua chuyển đổi số.</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2840,17 +2840,17 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] $18b grid investment crucial to driving Vietnam's energy future ... — A planned $18b investment in transmission infrastructure between 2026 and 2030 will be critical for Vietnam.</t>
+          <t>베트남은 2026년부터 2030년까지 전력망 확충을 위해 180억 달러를 투자할 계획이며, 이는 에너지 프로젝트의 실질적인 구현을 위해 필수적입니다. 현재 재생 에너지 용량 확대 속도에 비해 전력망 보강이 늦어 병목 현상이 발생하고 있으나, 2026년 예정된 입법 개혁을 통해 규제 완화와 투자 유인이 이루어질 전망입니다.</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] $18b grid investment crucial to driving Vietnam's energy future ... — A planned $18b investment in transmission infrastructure between 2026 and 2030 will be critical for Vietnam.</t>
+          <t>Vietnam plans a $18 billion investment in transmission infrastructure between 2026 and 2030 to bridge the gap between energy planning and project delivery. While transmission bottlenecks currently pose risks as renewable growth outpaces grid reinforcement, legislative reforms in 2026 are expected to streamline licensing and offer green-energy incentives.</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] $18b grid investment crucial to driving Vietnam's energy future ... — A planned $18b investment in transmission infrastructure between 2026 and 2030 will be critical for Vietnam.</t>
+          <t>Việt Nam dự kiến đầu tư 18 tỷ USD vào hạ tầng truyền tải điện trong giai đoạn 2026-2030 để hiện thực hóa các dự án năng lượng. Hiện tại, tình trạng nghẽn mạch lưới điện vẫn là thách thức lớn khi năng lượng tái tạo phát triển nhanh hơn hạ tầng, nhưng các cải cách luật pháp vào năm 2026 được kỳ vọng sẽ giải quyết nút thắt này thông qua cơ chế lựa chọn nhà đầu tư hợp lý và ưu đãi xanh.</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam to build $1.1B bridge to connect key Mekong Delta ... — The bridge will have six lanes, 100 kph design speed, 300 m navigation clearance, plus approach roads with emergency lanes. Total investment is ... (관련: VN-TRAN-2055)</t>
+          <t>베트남은 메콩 델타의 주요 고속도로를 연결하기 위해 약 11억 달러 이상을 투입하여 '껀터 2' 교량을 건설할 계획입니다. 이 교량은 도로와 철도가 결합된 복합 링크로 설계되었으며, 2026년 말 착공하여 약 5년간의 공사 기간이 소요될 예정입니다.</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam to build $1.1B bridge to connect key Mekong Delta ... — The bridge will have six lanes, 100 kph design speed, 300 m navigation clearance, plus approach roads with emergency lanes. Total investment is ... (Related: VN-TRAN-2055)</t>
+          <t>Vietnam is set to invest over $1.1 billion in the Can Tho 2 bridge, a strategic road-and-rail link connecting key expressways in the Mekong Delta. Construction is scheduled to begin in late 2026 and is expected to take five years, enhancing regional logistics and national security.</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam to build $1.1B bridge to connect key Mekong Delta ... — The bridge will have six lanes, 100 kph design speed, 300 m navigation clearance, plus approach roads with emergency lanes. Total investment is ... (Liên quan: VN-TRAN-2055)</t>
+          <t>Việt Nam đang chuẩn bị xây dựng cầu Cần Thơ 2 với tổng vốn đầu tư hơn 1,1 tỷ USD nhằm kết nối các tuyến đường cao tốc trọng điểm tại Đồng bằng sông Cửu Long. Dự án kết hợp giữa đường bộ và đường sắt này dự kiến sẽ khởi công vào cuối năm 2026 và hoàn thành sau khoảng 5 năm.</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2964,17 +2964,17 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam highway developments continue | Global Highways — Vietnam plans to build eight new expressways in the Central Highlands by 2030. This programme of construction will add around 830km to Vietnam's expressway ... (관련: VN-TRAN-2055, VN-EV-2030)</t>
+          <t>베트남은 2030년까지 중부 고원 지대에 약 830km에 달하는 8개의 새로운 고속도로를 건설할 계획이며, 총 사업비는 약 65억 달러에 이를 것으로 예상됩니다. 탄푸-바오록 구간은 2023년에 착공될 예정이며, 호치민시 제4순환도로 프로젝트는 2026년 완공을 목표로 하고 있습니다.</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam highway developments continue | Global Highways — Vietnam plans to build eight new expressways in the Central Highlands by 2030. This programme of construction will add around 830km to Vietnam's expressway ... (Related: VN-TRAN-2055, VN-EV-2030)</t>
+          <t>Vietnam plans to expand its expressway network by adding 830km through eight new projects in the Central Highlands by 2030, costing approximately $6.5 billion. Key developments include the Tan Phu-Bao Loc route starting in 2023 and the Ho Chi Minh City Beltway No4 project slated for completion by 2026.</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam highway developments continue | Global Highways — Vietnam plans to build eight new expressways in the Central Highlands by 2030. This programme of construction will add around 830km to Vietnam's expressway ... (Liên quan: VN-TRAN-2055, VN-EV-2030)</t>
+          <t>Việt Nam kế hoạch xây dựng 8 tuyến đường cao tốc mới tại Tây Nguyên đến năm 2030 với tổng chiều dài khoảng 830km và kinh phí gần 6,5 tỷ USD. Các dự án trọng điểm bao gồm cao tốc Tân Phú - Bảo Lộc khởi công năm 2023 và đường Vành đai 4 TP.HCM dự kiến hoàn thành vào năm 2026.</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3028,17 +3028,17 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Binh Goi bridge to open on April 30, 2026 - YouTube — Ho Chi Minh City will open Binh Goi Bridge to technical traffic on April 30, 2026, under the Beltway No. 3 project.</t>
+          <t>베트남 교통 및 인프라 부문의 최신 소식을 전하는 사이공 타임즈 뉴스입니다. 현재 제공된 콘텐츠는 채널 식별 정보에 한정되어 있어 구체적인 프로젝트 세부 사항을 요약하기 어렵습니다.</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Binh Goi bridge to open on April 30, 2026 - YouTube — Ho Chi Minh City will open Binh Goi Bridge to technical traffic on April 30, 2026, under the Beltway No. 3 project.</t>
+          <t>This is the Saigon Times News covering the transport and infrastructure sector in Vietnam. Due to the limited content provided in the snippet, specific details regarding infrastructure plans or project updates are not currently available for full summary.</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Binh Goi bridge to open on April 30, 2026 - YouTube — Ho Chi Minh City will open Binh Goi Bridge to technical traffic on April 30, 2026, under the Beltway No. 3 project.</t>
+          <t>Đây là tin tức từ Saigon Times News về lĩnh vực Giao thông và Hạ tầng tại Việt Nam. Do nội dung cung cấp chỉ bao gồm tên kênh, hiện chưa có đủ thông tin chi tiết về các dự án cụ thể để tóm tắt đầy đủ.</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3092,17 +3092,17 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam to build 2,000km of new expressways between 2026-2030 — From 2026–2030, about 2,000 km of expressways will be built, raising the national total to 5,000 km by 2030. The coastal route will be completed ... (관련: VN-TRAN-2055)</t>
+          <t>베트남 건설부는 2026년부터 2030년까지 2,000km의 고속도로를 추가 건설하여 총 5,000km의 고속도로망을 구축할 계획입니다. 이 계획에는 남북 고속철도, 국제 환적 항만, 신공항 건설뿐만 아니라 주요 도시의 메트로 및 순환도로 확충이 포함됩니다.</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam to build 2,000km of new expressways between 2026-2030 — From 2026–2030, about 2,000 km of expressways will be built, raising the national total to 5,000 km by 2030. The coastal route will be completed ... (Related: VN-TRAN-2055)</t>
+          <t>Vietnam plans to build 2,000km of new expressways between 2026 and 2030, bringing the national total to 5,000km. The infrastructure strategy also prioritizes the North-South high-speed railway, international transshipment seaports, and smart urban transport systems including new metro lines.</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam to build 2,000km of new expressways between 2026-2030 — From 2026–2030, about 2,000 km of expressways will be built, raising the national total to 5,000 km by 2030. The coastal route will be completed ... (Liên quan: VN-TRAN-2055)</t>
+          <t>Việt Nam đặt mục tiêu xây dựng thêm 2.000 km đường bộ cao tốc trong giai đoạn 2026–2030, nâng tổng chiều dài toàn quốc lên 5.000 km. Kế hoạch này tập trung vào đường sắt tốc độ cao Bắc-Nam, phát triển cảng biển trung chuyển quốc tế và hoàn thiện hạ tầng giao thông đô thị thông minh.</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3156,17 +3156,17 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>[Urban Development] 10 Vietnam Construction Projects Completing in 2026 - YouTube — ... expressway connecting north to south for the first time. Metro lines in Hanoi and Ho Chi Minh City that took over a decade to build. And ... (관련: VN-TRAN-2055)</t>
+          <t>베트남은 지난 50년 동안 전쟁의 상흔을 딛고 애플과 삼성의 글로벌 제조 허브로 급성장했습니다. 급격한 경제 발전에 발맞추어 롱탄 국제공항을 포함한 10개의 대규모 인프라 프로젝트가 2026년 완공을 목표로 진행 중입니다.</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>[Urban Development] 10 Vietnam Construction Projects Completing in 2026 - YouTube — ... expressway connecting north to south for the first time. Metro lines in Hanoi and Ho Chi Minh City that took over a decade to build. And ... (Related: VN-TRAN-2055)</t>
+          <t>Vietnam has transitioned from a war-torn nation to a major manufacturing hub for companies like Apple and Samsung over the last 50 years. To support this growth, ten major construction projects, including the Long Thanh International Airport, are scheduled for completion in 2026.</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>[Urban Development] 10 Vietnam Construction Projects Completing in 2026 - YouTube — ... expressway connecting north to south for the first time. Metro lines in Hanoi and Ho Chi Minh City that took over a decade to build. And ... (Liên quan: VN-TRAN-2055)</t>
+          <t>Việt Nam đã chuyển mình từ một quốc gia bị tàn phá bởi chiến tranh thành trung tâm sản xuất của Apple và Samsung trong 50 năm qua. Hiện nay, cơ sở hạ tầng đang được đẩy mạnh phát triển với 10 dự án xây dựng trọng điểm, bao gồm sân bay quốc tế Long Thành, dự kiến hoàn thành vào năm 2026.</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3220,17 +3220,17 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] HCMC plans to break ground on 14 major transport infrastructure ... — Alongside new ground-breaking projects, the city targets completion of around 10 major works in 2026, including Ring Road 3, An Phu and My Thuy ... (관련: VN-TRAN-2055)</t>
+          <t>호치민시는 2026년에 순환도로 4호선, 메트로 2호선, 껀저 교량 등 14개의 주요 교통 인프라 프로젝트를 착공할 계획입니다. 또한, 2026년까지 순환도로 3호선과 안푸 교차로를 포함한 10개 주요 사업의 완공을 목표로 하고 있습니다. 이는 현대적인 교통망 구축을 위해 약 1,780조 동(677.6억 달러)을 투입하는 2025-2030 액션 프로그램의 일환입니다.</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] HCMC plans to break ground on 14 major transport infrastructure ... — Alongside new ground-breaking projects, the city targets completion of around 10 major works in 2026, including Ring Road 3, An Phu and My Thuy ... (Related: VN-TRAN-2055)</t>
+          <t>Ho Chi Minh City plans to break ground on 14 major transport infrastructure projects in 2026, including Ring Road 4, Metro Line No. 2, and the Can Gio bridge. The city also targets the completion of 10 major works, such as Ring Road 3 and various interchanges, within the same year. These efforts are part of a larger 2025–2030 investment plan involving 77 projects valued at approximately 67.76 billion USD.</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] HCMC plans to break ground on 14 major transport infrastructure ... — Alongside new ground-breaking projects, the city targets completion of around 10 major works in 2026, including Ring Road 3, An Phu and My Thuy ... (Liên quan: VN-TRAN-2055)</t>
+          <t>TP.HCM kế hoạch khởi công 14 dự án hạ tầng giao thông trọng điểm vào năm 2026, bao gồm Vành đai 4, Tuyến Metro số 2 và cầu Cần Giờ. Thành phố cũng đặt mục tiêu hoàn thành 10 công trình lớn như Vành đai 3 và nút giao An Phú trong cùng năm đó. Đây là một phần của chương trình hành động 2025–2030 với tổng vốn đầu tư ước tính khoảng 1,78 triệu tỷ đồng cho 77 dự án.</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3280,17 +3280,17 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam plans bridge link upgrade | Global Highways — The project is for the Thu Thiem 4 Bridge, which will measure 2.16km and connect District 2 with District 7. The bridge will feature six traffic lanes. The ... (관련: VN-TRAN-2055)</t>
+          <t>베트남 호치민시 사이공강을 가로지르는 투티엠 4교(Thu Thiem 4 Bridge) 건설 계획이 추진 중입니다. 이 교량은 총 길이 2.16km, 왕복 6차로 규모로 2군과 7군을 연결할 예정입니다.</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam plans bridge link upgrade | Global Highways — The project is for the Thu Thiem 4 Bridge, which will measure 2.16km and connect District 2 with District 7. The bridge will feature six traffic lanes. The ... (Related: VN-TRAN-2055)</t>
+          <t>Ho Chi Minh City is planning the construction of the Thu Thiem 4 Bridge spanning the Saigon River to connect District 2 and District 7. The 2.16km-long bridge will feature six traffic lanes and is a joint effort between the Ministry of Planning and Investment, the HCMC People's Committee, and the Ministry of Transport.</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam plans bridge link upgrade | Global Highways — The project is for the Thu Thiem 4 Bridge, which will measure 2.16km and connect District 2 with District 7. The bridge will feature six traffic lanes. The ... (Liên quan: VN-TRAN-2055)</t>
+          <t>Thành phố Hồ Chí Minh đang lập kế hoạch xây dựng cầu Thủ Thiêm 4 bắc qua sông Sài Gòn để kết nối Quận 2 với Quận 7. Cây cầu có chiều dài 2,16km với quy mô 6 làn xe, được phối hợp triển khai bởi Bộ Kế hoạch và Đầu tư, Ủy ban Nhân dân TP.HCM và Bộ Giao thông Vận tải.</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3344,17 +3344,17 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City proposes $193mn Thu Thiem 4 bridge project ... — Ho Chi Minh City proposes $193mn Thu Thiem 4 bridge project, construction set for 2026 · The Ho Chi Minh City administration has submitted an ...</t>
+          <t>호치민시는 약 1억 9,300만 달러 규모의 투 티엠 4 교량 건설 사업을 시의회에 제안했습니다. 이 프로젝트는 2026년 4분기에 착공하여 2028년 완공될 예정이며, 시 남부 지역과 투 티엠 신도시를 연결하여 교통 혼잡을 완화하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City proposes $193mn Thu Thiem 4 bridge project ... — Ho Chi Minh City proposes $193mn Thu Thiem 4 bridge project, construction set for 2026 · The Ho Chi Minh City administration has submitted an ...</t>
+          <t>Ho Chi Minh City has proposed the $193 million Thu Thiem 4 Bridge project to connect the southern urban area with the Thu Thiem New Urban Area. Construction is scheduled to begin in late 2026 and reach completion by the end of 2028, funded entirely by the city's budget to improve regional traffic synchronization.</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City proposes $193mn Thu Thiem 4 bridge project ... — Ho Chi Minh City proposes $193mn Thu Thiem 4 bridge project, construction set for 2026 · The Ho Chi Minh City administration has submitted an ...</t>
+          <t>Ủy ban Nhân dân TP.HCM đã đề xuất dự án cầu Thủ Thiêm 4 với tổng vốn đầu tư khoảng 5.063 tỷ đồng (193 triệu USD) nối Quận 7 với Khu đô thị mới Thủ Thiêm. Dự kiến công trình sẽ khởi công vào quý 4 năm 2026 và hoàn thành vào quý 4 năm 2028 nhằm giảm tải áp lực giao thông cho khu vực trung tâm.</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3408,17 +3408,17 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's highest vertical cable-stayed bridge accelerates to wait for ... — Hai Phong - By the end of March 2026, the site clearance progress of the Nguyen Trai - Le Hong Phong intersection will only reach about 60%.</t>
+          <t>베트남에서 가장 높은 55m의 항행 통과 높이를 자랑하는 푸억카잉(Phuoc Khanh) 교량이 현재 96%의 공정률을 보이며 2026년 5월 완공을 앞두고 있습니다. 벤룩-롱탄 고속도로의 핵심 구간인 이 교량은 2026년 3분기 전 구간 개통을 위한 결정적인 역할을 할 것으로 기대됩니다.</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's highest vertical cable-stayed bridge accelerates to wait for ... — Hai Phong - By the end of March 2026, the site clearance progress of the Nguyen Trai - Le Hong Phong intersection will only reach about 60%.</t>
+          <t>The Phuoc Khanh Bridge, featuring Vietnam's highest navigation clearance of 55 meters, has reached 96% completion and is scheduled for closure in May 2026. This vital link in the Ben Luc - Long Thanh Expressway is expected to facilitate full-route traffic operations by the third quarter of 2026.</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's highest vertical cable-stayed bridge accelerates to wait for ... — Hai Phong - By the end of March 2026, the site clearance progress of the Nguyen Trai - Le Hong Phong intersection will only reach about 60%.</t>
+          <t>Cầu Phước Khánh với tĩnh không thông thuyền cao nhất Việt Nam (55m) hiện đã đạt 96% khối lượng và dự kiến sẽ hợp long vào tháng 5/2026. Đây là mắt xích quan trọng thuộc cao tốc Bến Lức - Long Thành, tạo tiền đề để thông xe toàn tuyến vào quý III/2026.</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3472,17 +3472,17 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>[Other] Vietnam's $67BN Gamble on High-Speed Rail - YouTube — Vietnam is about to build the largest infrastructure project in its history. Rayon is the all-in-one, effortless CAD tool for going from ...</t>
+          <t>베트남은 역사상 최대 규모의 인프라 프로젝트인 670억 달러 규모의 고속철도 건설을 추진하고 있습니다. 이 야심 찬 프로젝트는 국가의 연결성을 혁신하고 경제 성장을 촉진하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>[Other] Vietnam's $67BN Gamble on High-Speed Rail - YouTube — Vietnam is about to build the largest infrastructure project in its history. Rayon is the all-in-one, effortless CAD tool for going from ...</t>
+          <t>Vietnam is embarking on its largest-ever infrastructure project, a high-speed railway valued at $67 billion. This massive investment aims to modernize the nation's transport network and stimulate long-term economic development.</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>[Other] Vietnam's $67BN Gamble on High-Speed Rail - YouTube — Vietnam is about to build the largest infrastructure project in its history. Rayon is the all-in-one, effortless CAD tool for going from ...</t>
+          <t>Việt Nam đang chuẩn bị triển khai dự án cơ sở hạ tầng lớn nhất trong lịch sử với tuyến đường sắt tốc độ cao trị giá 67 tỷ USD. Dự án đầy tham vọng này hứa hẹn sẽ thay đổi mạng lưới giao thông và thúc đẩy tăng trưởng kinh tế quốc gia.</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3536,17 +3536,17 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam pushes to break ground on North-South high-speed railway ... — Approved by the National Assembly on November 30, 2024, the high-speed rail project will stretch 1,541 kilometers from Ngoc Hoi Station (Hanoi) ...</t>
+          <t>베트남 건설부 장관은 2026년 말까지 남북 고속철도 착공을 추진하라고 지시했습니다. 이 프로젝트는 하노이와 호치민을 잇는 1,541km 구간으로, 시속 350km의 설계 속도를 갖추고 2035년 완공을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam pushes to break ground on North-South high-speed railway ... — Approved by the National Assembly on November 30, 2024, the high-speed rail project will stretch 1,541 kilometers from Ngoc Hoi Station (Hanoi) ...</t>
+          <t>Vietnam's Minister of Construction has ordered agencies to ensure the 1,541-km North-South high-speed railway breaks ground by the end of 2026. Designed for speeds of 350 km/h, the project will connect Hanoi and Ho Chi Minh City with a target completion date of 2035.</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam pushes to break ground on North-South high-speed railway ... — Approved by the National Assembly on November 30, 2024, the high-speed rail project will stretch 1,541 kilometers from Ngoc Hoi Station (Hanoi) ...</t>
+          <t>Bộ trưởng Bộ Xây dựng yêu cầu các cơ quan đảm bảo khởi công dự án đường sắt tốc độ cao Bắc-Nam vào cuối năm 2026. Tuyến đường sắt dài 1.541 km nối Hà Nội và TP.HCM với vận tốc thiết kế 350 km/h, dự kiến hoàn thành vào năm 2035.</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3600,17 +3600,17 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam eyes to begin high-speed rail construction in 2026 — The government plans to complete the north-south high-speed rail within 10 years as it prioritizes breakthroughs in infrastructure development. (관련: VN-EV-2030)</t>
+          <t>베트남 정부는 당초 계획보다 1년 앞당겨 2026년 말까지 남북 고속철도 건설에 착수하라는 지시를 내렸습니다. 670억 달러 규모의 이 프로젝트는 하노이와 호치민을 연결하며, 이 외에도 중국 국경을 잇는 북부 지역 철도망 확충이 함께 추진됩니다.</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam eyes to begin high-speed rail construction in 2026 — The government plans to complete the north-south high-speed rail within 10 years as it prioritizes breakthroughs in infrastructure development. (Related: VN-EV-2030)</t>
+          <t>The Vietnamese government has ordered the acceleration of the North-South high-speed railway project to begin construction by the end of 2026, one year earlier than originally planned. This $67 billion project will span 1,541 km between Hanoi and Ho Chi Minh City, complemented by additional rail links to the Chinese border and expanded metro systems in major cities.</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam eyes to begin high-speed rail construction in 2026 — The government plans to complete the north-south high-speed rail within 10 years as it prioritizes breakthroughs in infrastructure development. (Liên quan: VN-EV-2030)</t>
+          <t>Thủ tướng Phạm Minh Chính đã chỉ đạo đẩy nhanh tiến độ để khởi công dự án đường sắt tốc độ cao Bắc-Nam vào cuối năm 2026, sớm hơn một năm so với kế hoạch ban đầu. Dự án trị giá 67 tỷ USD này dài 1.541 km nối Hà Nội với TP.HCM, bên cạnh các tuyến đường sắt kết nối biên giới phía Bắc cũng đang được ưu tiên triển khai.</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3664,17 +3664,17 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City will start construction of 5 key metro lines in 2026 ... — Construction is scheduled to begin at the end of 2026. The railway will span 1,541 kilometers with a total investment of approximately US$67 ...</t>
+          <t>호치민시는 2026년에 5개의 주요 메트로 노선 건설을 시작할 예정입니다. 이 프로젝트는 도시의 교통 인프라를 획기적으로 개선하고 지역 경제 발전을 촉진하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City will start construction of 5 key metro lines in 2026 ... — Construction is scheduled to begin at the end of 2026. The railway will span 1,541 kilometers with a total investment of approximately US$67 ...</t>
+          <t>Ho Chi Minh City is scheduled to begin the construction of five key metro lines in 2026. This infrastructure initiative aims to enhance urban connectivity and support the city's long-term development goals.</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City will start construction of 5 key metro lines in 2026 ... — Construction is scheduled to begin at the end of 2026. The railway will span 1,541 kilometers with a total investment of approximately US$67 ...</t>
+          <t>Thành phố Hồ Chí Minh sẽ khởi công xây dựng 5 tuyến tàu điện ngầm (metro) trọng điểm vào năm 2026. Đây là bước đi quan trọng nhằm hoàn thiện hệ thống giao thông công cộng và thúc đẩy phát triển đô thị bền vững.</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3728,17 +3728,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] The rail dream gains speed in southern Vietnam - VietNamNet — City leaders outlined a clear roadmap: by 2030, urban railway transport is expected to meet 20 to 30 percent of travel demand; by 2035, 35 to 50 ...</t>
+          <t>호치민시의 메트로 1호선(벤탄-수오이띠엔)이 개통 1년 만에 2,000만 명 이상의 승객을 유치하며 성공적으로 안착했으며, 2호선도 최근 착공에 들어갔습니다. 시 정부는 2045년까지 대중교통 분담률을 50~60%로 높이기 위해 총 9개의 도시철도 노선을 구축하는 야심 찬 로드맵을 추진하고 있습니다. 이러한 철도망 확충은 도시의 현대화와 지속 가능한 발전을 이끄는 핵심축이 될 전망입니다.</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] The rail dream gains speed in southern Vietnam - VietNamNet — City leaders outlined a clear roadmap: by 2030, urban railway transport is expected to meet 20 to 30 percent of travel demand; by 2035, 35 to 50 ...</t>
+          <t>Ho Chi Minh City's Metro Line 1 has achieved over 20 million passenger trips in its first year, signaling a successful shift toward high-capacity public transport. Following this success, the city has broken ground on Metro Line 2 and is planning a total of nine lines to meet 50-60% of travel demand by 2045. This infrastructure expansion serves as the backbone for the city's Transit-Oriented Development (TOD) and modern urban transformation.</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] The rail dream gains speed in southern Vietnam - VietNamNet — City leaders outlined a clear roadmap: by 2030, urban railway transport is expected to meet 20 to 30 percent of travel demand; by 2035, 35 to 50 ...</t>
+          <t>Tuyến Metro số 1 (Bến Thành - Suối Tiên) tại TP.HCM đã đạt hơn 20 triệu lượt khách sau một năm vận hành, tạo động lực cho việc khởi công Tuyến số 2 và triển khai mạng lưới đường sắt đô thị. Thành phố đặt mục tiêu đến năm 2045, hệ thống metro sẽ đáp ứng 50-60% nhu cầu đi lại của người dân. Với lộ trình 9 tuyến đường sắt, TP.HCM đang hướng tới mô hình đô thị hiện đại, giảm ùn tắc và phát triển bền vững theo định hướng TOD.</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3792,17 +3792,17 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>[Urban Development] Construction of Vietnam's first high-speed railway expected to start ... — The North-South high-speed railway is planned to span approximately 1,541 km from Hanoi to Ho Chi Minh City with a design speed of 350 km/h.</t>
+          <t>베트남 건설부 장관의 지시에 따라 하노이와 호치민시를 잇는 1,541km 구간의 남북 고속철도 건설이 2026년 말에 시작될 예정입니다. 이 프로젝트는 총 587억 1천만 달러의 투자비가 투입되며, 시속 350km의 설계 속도를 갖춘 복선 철도로 건설됩니다.</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>[Urban Development] Construction of Vietnam's first high-speed railway expected to start ... — The North-South high-speed railway is planned to span approximately 1,541 km from Hanoi to Ho Chi Minh City with a design speed of 350 km/h.</t>
+          <t>Construction of Vietnam's first high-speed railway, connecting Hanoi and Ho Chi Minh City, is expected to begin by the end of 2026 following instructions from the Minister of Construction. The 1,541 km project features a design speed of 350 km/h and requires an estimated investment of $58.71 billion.</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>[Urban Development] Construction of Vietnam's first high-speed railway expected to start ... — The North-South high-speed railway is planned to span approximately 1,541 km from Hanoi to Ho Chi Minh City with a design speed of 350 km/h.</t>
+          <t>Theo chỉ đạo của Bộ trưởng Bộ Xây dựng, dự án đường sắt tốc độ cao Bắc-Nam dài 1.541 km nối Hà Nội và TP.HCM dự kiến sẽ khởi công vào cuối năm 2026. Dự án có tổng vốn đầu tư khoảng 58,71 tỷ USD với thiết kế đường đôi và tốc độ đạt 350 km/h.</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3856,17 +3856,17 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>[Urban Development] Connecting Vietnam's high-speed railway stations with urban rail ... — Vietnam is planning to build a high-speed railway from Hanoi to Ho Chi Minh City. 23 stations are planned for the line, and they will all be new ...</t>
+          <t>베트남은 하노이와 호치민을 잇는 고속철도 건설을 계획하고 있으며, 도심 외곽에 위치할 신설 역들과 도심을 연결하기 위해 하노이 메트로 1호선과 호치민 메트로 2호선 등 도시철도망 확충을 추진하고 있습니다. 다낭을 비롯해 냐짱, 후에 등 주요 거점 도시들도 관광 활성화와 접근성 개선을 위해 고속철도역과 연계된 도시 철도 및 트램 도입을 검토해야 한다는 제안이 나오고 있습니다.</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>[Urban Development] Connecting Vietnam's high-speed railway stations with urban rail ... — Vietnam is planning to build a high-speed railway from Hanoi to Ho Chi Minh City. 23 stations are planned for the line, and they will all be new ...</t>
+          <t>Vietnam is planning a high-speed railway connecting Hanoi and Ho Chi Minh City, with confirmed metro links for Hanoi's Ngoc Hoi Station and HCMC's Thu Thiem Station to ensure urban connectivity. Other major cities like Da Nang, Nha Trang, and Hue are also proposing or being urged to develop integrated light rail or tram systems to bridge the gap between distant high-speed rail stations and their respective city centers.</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>[Urban Development] Connecting Vietnam's high-speed railway stations with urban rail ... — Vietnam is planning to build a high-speed railway from Hanoi to Ho Chi Minh City. 23 stations are planned for the line, and they will all be new ...</t>
+          <t>Việt Nam đang quy hoạch tuyến đường sắt tốc độ cao Bắc-Nam với các ga kết nối trọng điểm như Ngọc Hồi (Hà Nội) qua Tuyến Metro số 1 và Thủ Thiêm (TP.HCM) qua Tuyến Metro số 2. Các thành phố khác như Đà Nẵng, Nha Trang và Huế cũng được đề xuất phát triển hệ thống đường sắt đô thị hoặc tàu điện nhẹ để kết nối hiệu quả các ga cao tốc mới nằm xa trung tâm với khu vực nội đô và các điểm du lịch.</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3920,17 +3920,17 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>[Urban Development] Financial close allows Ho Chi Minh City Line 2 civil works to start — The Ho Chi Minh City Party Committee decided in November 2025 to use the municipal and national budget to complete Line 2. Completion is ...</t>
+          <t>호치민시 메트로 2호선 건설을 위한 토목 공사가 1월 15일 착공되었습니다. 약 11.3km 길이의 이 노선은 시 정부와 국가 예산을 투입하여 2030년 4분기 완공을 목표로 하며, 현지 기업인 THACO가 이끄는 컨소시엄이 공사를 주도합니다.</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>[Urban Development] Financial close allows Ho Chi Minh City Line 2 civil works to start — The Ho Chi Minh City Party Committee decided in November 2025 to use the municipal and national budget to complete Line 2. Completion is ...</t>
+          <t>Civil works for the 11.3 km Ho Chi Minh City Metro Line 2 have officially commenced following a groundbreaking ceremony on January 15. The project, now funded by domestic municipal and national budgets after international funding plans were scrapped, is slated for completion in the fourth quarter of 2030.</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>[Urban Development] Financial close allows Ho Chi Minh City Line 2 civil works to start — The Ho Chi Minh City Party Committee decided in November 2025 to use the municipal and national budget to complete Line 2. Completion is ...</t>
+          <t>Công trình dân dụng cho tuyến tàu điện ngầm số 2 tại TP.HCM dài 11,3 km đã chính thức được khởi công vào ngày 15 tháng 1. Dự án sử dụng ngân sách thành phố và quốc gia để triển khai sau khi thay đổi phương án vốn, dự kiến sẽ hoàn thành vào quý IV năm 2030.</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3984,17 +3984,17 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City's metro vision: Big plans, slow progress Ho Chi ... — Construction is scheduled to begin at the end of 2026. The railway will span 1,541 kilometers with a total investment of approximately US$67 ...</t>
+          <t>호치민시는 교통 체증을 완화하기 위해 야심 찬 메트로 노선망을 계획하고 있으나, 현재 프로젝트 진행이 상당히 지연되고 있습니다. 도시 마스터 플랜에는 도심 교통을 현대화하고 주요 지역을 연결하기 위한 여러 노선이 포함되어 있습니다.</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City's metro vision: Big plans, slow progress Ho Chi ... — Construction is scheduled to begin at the end of 2026. The railway will span 1,541 kilometers with a total investment of approximately US$67 ...</t>
+          <t>Ho Chi Minh City is planning an ambitious metro network to alleviate traffic congestion, though projects have experienced significant delays. The city's master plan features multiple routes aimed at modernizing urban transport and connecting key districts.</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City's metro vision: Big plans, slow progress Ho Chi ... — Construction is scheduled to begin at the end of 2026. The railway will span 1,541 kilometers with a total investment of approximately US$67 ...</t>
+          <t>Thành phố Hồ Chí Minh đang lập kế hoạch cho mạng lưới tàu điện ngầm đầy tham vọng nhằm giảm bớt tình trạng tắc nghẽn giao thông, mặc dù các dự án đang đối mặt với sự chậm trễ đáng kể. Quy hoạch tổng thể của thành phố bao gồm nhiều tuyến đường được thiết kế để hiện đại hóa giao thông đô thị và kết nối các quận trọng điểm.</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4048,17 +4048,17 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City Metro Ride: An Phu Station to Saigon Centre — ... 2026 Support Me PayPal: https://paypal.me/actionkidyt?locale.x=en_US Cash App: $ ... Bullet Train | Shanghai - Beijing. Solo Solo Travel.</t>
+          <t>이 영상은 타오디엔의 안푸역에서 1군 중심부인 사이공 센터까지 이어지는 호치민 지하철 여정을 담고 있습니다. 도시 개발의 핵심인 메트로 라인을 통해 베트남의 현대화된 대중교통 인프라를 직접 확인할 수 있습니다.</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City Metro Ride: An Phu Station to Saigon Centre — ... 2026 Support Me PayPal: https://paypal.me/actionkidyt?locale.x=en_US Cash App: $ ... Bullet Train | Shanghai - Beijing. Solo Solo Travel.</t>
+          <t>This video showcases the journey on the Ho Chi Minh City Metro from An Phu Station in Thao Dien to the Saigon Centre in District 1. It highlights the progress of urban transportation infrastructure connecting vibrant residential areas to the city's commercial heart.</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City Metro Ride: An Phu Station to Saigon Centre — ... 2026 Support Me PayPal: https://paypal.me/actionkidyt?locale.x=en_US Cash App: $ ... Bullet Train | Shanghai - Beijing. Solo Solo Travel.</t>
+          <t>Video này ghi lại hành trình đi tàu điện Metro từ ga An Phú tại Thảo Điền đến Saigon Centre tại Quận 1. Đây là minh chứng cho sự phát triển của hạ tầng giao thông đô thị, kết nối các khu dân cư sầm uất với trung tâm kinh tế của thành phố.</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4112,17 +4112,17 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's infrastructure: Six forces shaping investment in 2026 ... — According to the Ministry of Finance, disbursed foreign direct investment in Vietnam was estimated at US$27.6 billion, up 9 per cent from a year ...</t>
+          <t>베트남은 2030년까지 약 1,500억~2,000억 달러의 인프라 투자 격차를 해소하기 위해 민간 및 외국 자본 유치를 필수 과제로 삼고 있습니다. 2025년 단행된 법적 개혁과 새로운 지도부의 정책은 국영기업(SOE) 및 민간 대기업과의 파트너십을 장려하여 해상 풍력, LNG, 교통망 등 주요 프로젝트의 투자 환경을 강화하고 있습니다.</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's infrastructure: Six forces shaping investment in 2026 ... — According to the Ministry of Finance, disbursed foreign direct investment in Vietnam was estimated at US$27.6 billion, up 9 per cent from a year ...</t>
+          <t>Vietnam is prioritizing foreign and private investment to bridge an estimated $150–200 billion infrastructure funding gap through 2030. Driven by new leadership and legislative reforms in 2025, the country is fostering partnerships between international investors, state-owned enterprises, and domestic conglomerates in sectors like renewable energy and logistics.</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's infrastructure: Six forces shaping investment in 2026 ... — According to the Ministry of Finance, disbursed foreign direct investment in Vietnam was estimated at US$27.6 billion, up 9 per cent from a year ...</t>
+          <t>Việt Nam đang nỗ lực thu hút vốn đầu tư nước ngoài và tư nhân để lấp đầy khoảng trống tài chính cơ sở hạ tầng ước tính khoảng 150–200 tỷ USD đến năm 2030. Với các cải cách luật pháp năm 2025 và định hướng của ban lãnh đạo mới, Chính phủ khuyến khích hợp tác giữa nhà đầu tư quốc tế với các doanh nghiệp nhà nước và tập đoàn tư nhân trong các lĩnh vực trọng điểm như năng lượng tái tạo và giao thông.</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4176,17 +4176,17 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's $16B Airport Why Construction Just STOPPED - YouTube — Vietnam's $16 Billion Long Thanh International Airport was supposed to be the "Jewel of Southeast Asia" and a rival to Singapore's Changi.</t>
+          <t>베트남의 160억 달러 규모 롱탄 국제공항 건설 프로젝트가 중단 위기에 처하며 동남아시아의 허브가 되려던 계획에 차질이 생겼습니다. 싱가포르 창이 공항에 도전하려던 이 대규모 인프라 사업은 최근 여러 문제로 인해 난항을 겪고 있습니다.</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's $16B Airport Why Construction Just STOPPED - YouTube — Vietnam's $16 Billion Long Thanh International Airport was supposed to be the "Jewel of Southeast Asia" and a rival to Singapore's Changi.</t>
+          <t>Vietnam's $16 billion Long Thanh International Airport project, intended to rival Singapore's Changi Airport, has faced significant construction delays and reported stoppages. This ambitious infrastructure development is struggling to meet its goal of becoming the premier transport hub of Southeast Asia.</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's $16B Airport Why Construction Just STOPPED - YouTube — Vietnam's $16 Billion Long Thanh International Airport was supposed to be the "Jewel of Southeast Asia" and a rival to Singapore's Changi.</t>
+          <t>Dự án sân bay quốc tế Long Thành trị giá 16 tỷ USD của Việt Nam đang đối mặt với việc tạm dừng thi công, đe dọa mục tiêu cạnh tranh với sân bay Changi của Singapore. Đây là công trình hạ tầng trọng điểm được kỳ vọng sẽ trở thành trung tâm trung chuyển mới của khu vực Đông Nam Á.</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4240,17 +4240,17 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Transport infrastructure in process of synchronisation — By the end of 2025, Vietnam had 3,345km of main expressways and 458km of interchanges and access roads in operation; it had fully completed and ... (관련: VN-TRAN-2055)</t>
+          <t>베트남 정부는 정체된 인프라 프로젝트를 해결하기 위해 강력한 지침을 내렸으며, 올해 벤룩-롱탄 고속도로와 호치민 제3순환도로 등 주요 도로망이 완공될 예정입니다. 롱탄 국제공항의 상업 운항 시작과 더불어 673억 달러 규모의 남북 고속철도 착공이 계획되어 국가 운송 인프라의 동기화가 가속화되고 있습니다.</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Transport infrastructure in process of synchronisation — By the end of 2025, Vietnam had 3,345km of main expressways and 458km of interchanges and access roads in operation; it had fully completed and ... (Related: VN-TRAN-2055)</t>
+          <t>The Vietnamese government is accelerating key infrastructure projects, with the Ben Luc-Long Thanh Expressway and HCMC Ring Road 3 nearing completion this year. Significant milestones include the commencement of operations at Long Thanh International Airport and the groundbreaking of the $67.3 billion North-South high-speed railway.</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Transport infrastructure in process of synchronisation — By the end of 2025, Vietnam had 3,345km of main expressways and 458km of interchanges and access roads in operation; it had fully completed and ... (Liên quan: VN-TRAN-2055)</t>
+          <t>Chính phủ Việt Nam đang đẩy nhanh tiến độ các dự án hạ tầng trọng điểm, trong đó cao tốc Bến Lức - Long Thành và Vành đai 3 TP.HCM dự kiến sẽ hoàn thành trong năm nay. Những cột mốc quan trọng bao gồm việc đưa Cảng hàng không quốc tế Long Thành vào khai thác thương mại và khởi công dự án đường sắt tốc độ cao Bắc - Nam trị giá hơn 67,3 tỷ USD.</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4304,17 +4304,17 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's aviation lifts off with major airport breakthroughs — Landmark infrastructure shaping a new development axis · Fleet expansion and robust market recovery · Toward double-digit growth in 2026. (관련: VN-EV-2030)</t>
+          <t>베트남은 롱타인 국제공항의 기술적 개항과 자빈 국제공항의 물류 허브 개발을 포함한 대규모 항공 인프라 확장을 가속화하고 있습니다. 2025년 역대 최고인 8,350만 명의 승객을 기록했으며, 2026년에는 경제 성장과 규제 완화에 힘입어 이용객이 9,500만 명에 이를 것으로 전망됩니다.</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's aviation lifts off with major airport breakthroughs — Landmark infrastructure shaping a new development axis · Fleet expansion and robust market recovery · Toward double-digit growth in 2026. (Related: VN-EV-2030)</t>
+          <t>Vietnam is accelerating its aviation infrastructure with flagship projects like Long Thanh International Airport and the new Gia Binh dual-use airport. The sector achieved a record 83.5 million passengers in 2025 and is projected to grow to 95 million in 2026, supported by fleet expansions and upgraded terminals like Tan Son Nhat T3.</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's aviation lifts off with major airport breakthroughs — Landmark infrastructure shaping a new development axis · Fleet expansion and robust market recovery · Toward double-digit growth in 2026. (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang đẩy mạnh hạ tầng hàng không với các dự án trọng điểm như sân bay quốc tế Long Thành và sân bay Gia Bình, nhằm thúc đẩy kết nối vùng và logistics. Năm 2025, ngành hàng không đạt kỷ lục 83,5 triệu lượt khách và dự kiến sẽ tăng trưởng lên 95 triệu lượt vào năm 2026 nhờ việc mở rộng đội bay và nâng cấp các nhà ga.</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4368,17 +4368,17 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's largest airport is about to be put into operation - Seetao — The first phase of Vietnam Longcheng International Airport project will be completed and put into operation in the first half of 2026.</t>
+          <t>베트남 동나이성에 위치한 롱타인 국제공항이 2026년 상반기 1단계 개항을 앞두고 있습니다. 한국 희림종합건축사사무소가 설계한 이 공항은 연꽃을 형상화한 디자인과 세계 최대 규모의 대나무 구조물을 특징으로 하며, 최종 완공 시 연간 1억 명의 승객을 수용하는 4F급 허브가 될 전망입니다.</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's largest airport is about to be put into operation - Seetao — The first phase of Vietnam Longcheng International Airport project will be completed and put into operation in the first half of 2026.</t>
+          <t>Vietnam's Long Thanh International Airport is nearing the completion of its first phase, scheduled for operation in the first half of 2026. Designed with a lotus-inspired aesthetic and utilizing sustainable bamboo structures, the 4F-level hub aims to handle 100 million passengers annually upon its full completion by 2040.</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's largest airport is about to be put into operation - Seetao — The first phase of Vietnam Longcheng International Airport project will be completed and put into operation in the first half of 2026.</t>
+          <t>Sân bay Quốc tế Long Thành tại tỉnh Đồng Nai đang hoàn thiện giai đoạn 1 để dự kiến đi vào hoạt động trong nửa đầu năm 2026. Với thiết kế lấy cảm hứng từ hoa sen và cấu trúc tre bền vững, dự án cấp 4F này đặt mục tiêu phục vụ 100 triệu hành khách mỗi năm khi hoàn thành toàn bộ vào năm 2040.</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4432,17 +4432,17 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's Long Thanh Airport to Launch by 2026 with $16B ... — Vietnam's Long Thanh Airport to Launch by 2026 with $16B Investment ... terminal, VIP terminal, and aviation infrastructure. • Capacity ...</t>
+          <t>베트남 정부는 총 사업비 약 160억 달러 규모의 롱탄 국제공항 건설을 가속화하기 위해 30일 이내에 핵심 계약 체결을 완료하라는 지침을 내렸습니다. 이 프로젝트는 2026년 말 상업 운영 시작을 목표로 하며, 연간 1억 명의 승객을 수용하는 지역 주요 항공 허브로 거듭날 전망입니다.</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's Long Thanh Airport to Launch by 2026 with $16B ... — Vietnam's Long Thanh Airport to Launch by 2026 with $16B Investment ... terminal, VIP terminal, and aviation infrastructure. • Capacity ...</t>
+          <t>The Vietnamese government has mandated a 30-day deadline to finalize key contracts for the Long Thanh International Airport, a $16 billion project aimed at starting operations by late 2026. The development is set to transform the region into a major aviation hub with an eventual capacity of 100 million passengers per year.</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's Long Thanh Airport to Launch by 2026 with $16B ... — Vietnam's Long Thanh Airport to Launch by 2026 with $16B Investment ... terminal, VIP terminal, and aviation infrastructure. • Capacity ...</t>
+          <t>Chính phủ Việt Nam đã chốt thời hạn 30 ngày để hoàn tất ký kết các hợp đồng then chốt cho dự án sân bay quốc tế Long Thành với tổng vốn đầu tư khoảng 16 tỷ USD. Dự án đặt mục tiêu bắt đầu vận hành khai thác vào cuối năm 2026 và hướng tới công suất 100 triệu hành khách mỗi năm.</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4496,17 +4496,17 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam PM presses for Long Thanh airport phase 1 completion by ... — Long Thanh International Airport is a national key project spanning about 5,000 hectares, with a total estimated investment of more than VND336.</t>
+          <t>베트남 팜 민 찐 총리는 롱탄 국제공항 1단계 사업을 2026년 상반기까지 완료할 것을 지시했습니다. 약 42억 달러가 투입된 이 프로젝트는 연간 2,500만 명의 승객을 수용하는 것을 목표로 하며, 스마트 및 친환경 기술이 도입될 예정입니다.</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam PM presses for Long Thanh airport phase 1 completion by ... — Long Thanh International Airport is a national key project spanning about 5,000 hectares, with a total estimated investment of more than VND336.</t>
+          <t>Vietnam's Prime Minister Pham Minh Chinh has directed that Phase 1 of the Long Thanh International Airport be completed by the first half of 2026. This $4.2 billion phase aims to handle 25 million passengers annually and will feature advanced biometric systems and smart infrastructure.</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam PM presses for Long Thanh airport phase 1 completion by ... — Long Thanh International Airport is a national key project spanning about 5,000 hectares, with a total estimated investment of more than VND336.</t>
+          <t>Thủ tướng Phạm Minh Chính đã chỉ đạo hoàn thành giai đoạn 1 của dự án Cảng hàng không quốc tế Long Thành trong nửa đầu năm 2026. Với tổng vốn đầu tư giai đoạn này khoảng 109 nghìn tỷ đồng, sân bay được kỳ vọng sẽ phục vụ 25 triệu lượt khách mỗi năm và trở thành trung tâm hàng không hiện đại của khu vực.</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4560,17 +4560,17 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's $16B AIRPORT MEGA PROJECT Could Change Asia ... — ... infrastructure move yet—and why the rest of Asia is watching ... HUGE Vietnam Visa Update 2026 NOBODY Expected (WHY?!) Duong Global ...</t>
+          <t>베트남은 아시아 항공 지형을 바꿀 수 있는 160억 달러 규모의 초대형 신공항 프로젝트를 추진하고 있습니다. 이 메가 프로젝트는 글로벌 항공 시장에 막대한 영향을 미칠 것으로 예상됩니다.</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's $16B AIRPORT MEGA PROJECT Could Change Asia ... — ... infrastructure move yet—and why the rest of Asia is watching ... HUGE Vietnam Visa Update 2026 NOBODY Expected (WHY?!) Duong Global ...</t>
+          <t>Vietnam is moving forward with a massive $16 billion mega airport project aimed at reshaping Asia's aviation landscape. This infrastructure development is expected to have a significant global impact and potentially change regional travel forever.</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's $16B AIRPORT MEGA PROJECT Could Change Asia ... — ... infrastructure move yet—and why the rest of Asia is watching ... HUGE Vietnam Visa Update 2026 NOBODY Expected (WHY?!) Duong Global ...</t>
+          <t>Việt Nam đang đẩy mạnh dự án siêu sân bay trị giá 16 tỷ USD có khả năng thay đổi vĩnh viễn bản đồ hàng không châu Á. Dự án hạ tầng khổng lồ này được dự báo sẽ tạo ra tác động lớn trên phạm vi toàn cầu.</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4624,17 +4624,17 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Viet Nam approves investment policy for Gia Binh International Airport — The airport will be completed by the end of 2026, with trial operations beginning in February 2027. Covering nearly 1,960 hectares, the airport ...</t>
+          <t>베트남 박닌성에 위치한 가빈(Gia Binh) 국제공항 건설 사업이 투자 승인을 받아 본격화되었습니다. 이 공항은 2026년 말 완공되어 2027년 2월 시운전을 시작할 예정이며, 연간 3,000만 명의 승객과 160만 톤의 화물을 처리하는 북부 지역의 주요 항공 허브가 될 것으로 기대됩니다.</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Viet Nam approves investment policy for Gia Binh International Airport — The airport will be completed by the end of 2026, with trial operations beginning in February 2027. Covering nearly 1,960 hectares, the airport ...</t>
+          <t>Vietnam has approved the investment policy for Gia Binh International Airport in Bac Ninh province, aiming for completion by the end of 2026. This dual-use facility is designed to handle 30 million passengers and 1.6 million tons of cargo annually by 2030, serving as a strategic logistics and transport hub near Hanoi.</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Viet Nam approves investment policy for Gia Binh International Airport — The airport will be completed by the end of 2026, with trial operations beginning in February 2027. Covering nearly 1,960 hectares, the airport ...</t>
+          <t>Việt Nam đã phê duyệt chính sách đầu tư cho dự án Cảng hàng không quốc tế Gia Bình tại tỉnh Bắc Ninh, dự kiến hoàn thành vào cuối năm 2026. Sân bay lưỡng dụng này có công suất thiết kế đạt 30 triệu hành khách và 1,6 triệu tấn hàng hóa mỗi năm vào giai đoạn 2021-2030, tạo động lực phát triển cho vùng kinh tế phía Bắc.</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4684,17 +4684,17 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Planning &amp; Bidding Vietnam Aviation Infrastructure — Consolidated data on key airport projects under construction, active bidding processes, and new strategic proposals as of 2025.</t>
+          <t>2025년 기준 베트남의 주요 공항 건설 프로젝트, 입찰 프로세스 및 신규 전략 제안에 대한 통합 데이터입니다. 미래에셋증권 베트남 법인이 교통부와 국가 공항망 마스터플랜을 분석하여 정리한 자료입니다.</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Planning &amp; Bidding Vietnam Aviation Infrastructure — Consolidated data on key airport projects under construction, active bidding processes, and new strategic proposals as of 2025.</t>
+          <t>This report provides consolidated data on key airport projects under construction, bidding activities, and strategic proposals in Vietnam as of 2025. It is based on Mirae Asset Securities Vietnam's analysis of Ministry of Transport data and the National Airport Network Master Plan.</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Planning &amp; Bidding Vietnam Aviation Infrastructure — Consolidated data on key airport projects under construction, active bidding processes, and new strategic proposals as of 2025.</t>
+          <t>Báo cáo tổng hợp dữ liệu về các dự án sân bay trọng điểm đang xây dựng, quá trình đấu thầu và các đề xuất chiến lược mới tại Việt Nam tính đến năm 2025. Thông tin được Mirae Asset Securities Vietnam phân tích và tổng hợp từ Bộ Giao thông Vận tải cùng Quy hoạch tổng thể hệ thống cảng hàng không toàn quốc.</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4748,17 +4748,17 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Decree 29/2026: Vietnam Operationalizes Its First Carbon Trading ... — At COP26, the country pledged to reach net-zero emissions by 2050 and reduce methane emissions by 30 percent by 2030 compared to 2020 levels. (관련: VN-EV-2030)</t>
+          <t>베트남은 시행령 제29/2026/ND-CP호를 통해 국가 최초의 탄소 배출권 거래소 운영 프레임워크를 구축하고 환경 인프라를 본격화했습니다. 2025-2026년 시범 기간 동안 화력 발전소, 철강 및 시멘트 공장을 대상으로 온실가스 배출 할당량을 부여하여 2050년 넷제로 목표 달성을 추진합니다.</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Decree 29/2026: Vietnam Operationalizes Its First Carbon Trading ... — At COP26, the country pledged to reach net-zero emissions by 2050 and reduce methane emissions by 30 percent by 2030 compared to 2020 levels. (Related: VN-EV-2030)</t>
+          <t>Vietnam has operationalized its first domestic carbon trading exchange under Decree 29/2026/ND-CP, integrating emission quotas into its securities market infrastructure. The 2025-2026 pilot phase targets high-emission sectors like power, steel, and cement to support the country's VN-EV-2030 and net-zero climate commitments.</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Decree 29/2026: Vietnam Operationalizes Its First Carbon Trading ... — At COP26, the country pledged to reach net-zero emissions by 2050 and reduce methane emissions by 30 percent by 2030 compared to 2020 levels. (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đã chính thức vận hành sàn giao dịch tín chỉ carbon đầu tiên thông qua Nghị định 29/2026/NĐ-CP, tích hợp hạn ngạch phát thải vào hạ tầng thị trường chứng khoán. Trong giai đoạn thí điểm 2025-2026, chính phủ phân bổ hạn ngạch cho các nhà máy nhiệt điện, thép và xi măng nhằm hiện thực hóa mục tiêu giảm phát thải khí nhà kính và Net Zero vào năm 2050.</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4812,17 +4812,17 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Fulfilling climate commitments at COP26: Vietnam's comprehensive ... — At COP26, Vietnam raised its ambition with the landmark pledge to achieve net-zero emissions by 2050 - a historic milestone underscoring its ... (관련: VN-EV-2030)</t>
+          <t>베트남은 COP26에서 약속한 2050년 넷제로 목표를 달성하기 위해 에너지, 농업, 산림 등 전 분야에 걸친 포괄적인 실행 계획을 추진하고 있습니다. 제8차 전력개발계획(PDP8)을 통해 재생 에너지를 확대하고 석탄 의존도를 낮추는 인프라 전환과 더불어 저탄소 농업 및 폐기물 에너지화 기술을 적극 도입하고 있습니다.</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Fulfilling climate commitments at COP26: Vietnam's comprehensive ... — At COP26, Vietnam raised its ambition with the landmark pledge to achieve net-zero emissions by 2050 - a historic milestone underscoring its ... (Related: VN-EV-2030)</t>
+          <t>Vietnam is implementing a comprehensive cross-sector strategy to fulfill its COP26 commitment of reaching net-zero emissions by 2050. Key infrastructure initiatives include transitioning to renewable energy under Power Development Plan VIII, scaling up low-emission rice cultivation in the Mekong Delta, and adopting waste-to-energy technologies.</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Fulfilling climate commitments at COP26: Vietnam's comprehensive ... — At COP26, Vietnam raised its ambition with the landmark pledge to achieve net-zero emissions by 2050 - a historic milestone underscoring its ... (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang tích cực triển khai các cam kết tại COP26 thông qua chiến lược toàn diện nhằm đạt phát thải ròng bằng "0" vào năm 2050. Các hành động cụ thể bao gồm chuyển đổi năng lượng tái tạo theo Quy hoạch điện VIII, phát triển một triệu héc-ta lúa chất lượng cao phát thải thấp và thúc đẩy các mô hình kinh tế tuần hoàn trên toàn quốc.</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4876,17 +4876,17 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Achieving net-zero emissions by 2050 is a political mission of Vietnam — Bringing Vietnam to net-zero emissions by 2050 is not merely a promise but a commitment to action - a political mission of the nation and a ... (관련: VN-EV-2030)</t>
+          <t>베트남 팜 민 찐 총리는 2050년 탄소 중립 달성이 국가적 정치 임무임을 강조하며, 이를 위한 제도적 개선과 탄소 시장 구축을 촉구했습니다. 특히 탄소 배출권 할당 시범 운영과 함께 전기차 및 친환경 에너지 기반의 대중교통 시스템 구축 등 녹색 교통 인프라 확대를 지시했습니다.</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Achieving net-zero emissions by 2050 is a political mission of Vietnam — Bringing Vietnam to net-zero emissions by 2050 is not merely a promise but a commitment to action - a political mission of the nation and a ... (Related: VN-EV-2030)</t>
+          <t>Prime Minister Pham Minh Chinh reaffirmed Vietnam's commitment to achieving Net Zero by 2050, labeling it a core political mission that drives sustainable development and international integration. The government is accelerating the development of a domestic carbon market and prioritizing green infrastructure, specifically the electrification of public transport and the transition to clean energy vehicles (VN-EV-2030).</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Achieving net-zero emissions by 2050 is a political mission of Vietnam — Bringing Vietnam to net-zero emissions by 2050 is not merely a promise but a commitment to action - a political mission of the nation and a ... (Liên quan: VN-EV-2030)</t>
+          <t>Thủ tướng Phạm Minh Chính khẳng định đạt phát thải ròng bằng 0 vào năm 2050 là nhiệm vụ chính trị trọng tâm nhằm phát triển đất nước bền vững và tự chủ. Chính phủ sẽ đẩy mạnh thị trường carbon nội bộ và yêu cầu các địa phương tiên phong phát triển hệ thống giao thông công cộng chạy bằng điện và năng lượng xanh.</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4936,17 +4936,17 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Viet Nam - Policies &amp; action | Climate Action Tracker — Viet Nam's emissions under current policies will reach around 686–722 MtCO2e in 2030 (excl. LULUCF) whereas a 1.5˚C fair share pathway is 344 MtCO2e in 2030. (관련: VN-CARBON-2050)</t>
+          <t>베트남은 2050년 넷제로 목표를 달성하기 위해 제8차 전력개발계획(PDP8) 및 국가 기후변화 전략을 수립하고 에너지 인프라를 대대적으로 개편하고 있습니다. 석탄 화력 발전소를 2050년까지 단계적으로 폐쇄하는 동시에 태양광, 해상 풍력 등 재생 에너지 비중을 대폭 확대하고 전력망 현대화에 집중하고 있습니다.</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Viet Nam - Policies &amp; action | Climate Action Tracker — Viet Nam's emissions under current policies will reach around 686–722 MtCO2e in 2030 (excl. LULUCF) whereas a 1.5˚C fair share pathway is 344 MtCO2e in 2030. (Related: VN-CARBON-2050)</t>
+          <t>Vietnam is overhaulng its energy infrastructure through the Power Development Plan 8 (PDP8) to achieve net-zero emissions by 2050. The strategy involves phasing out coal power by 2050 while rapidly scaling up solar and offshore wind capacity alongside critical grid upgrades supported by the Just Energy Transition Partnership (JETP).</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Viet Nam - Policies &amp; action | Climate Action Tracker — Viet Nam's emissions under current policies will reach around 686–722 MtCO2e in 2030 (excl. LULUCF) whereas a 1.5˚C fair share pathway is 344 MtCO2e in 2030. (Liên quan: VN-CARBON-2050)</t>
+          <t>Việt Nam đang triển khai Quy hoạch điện VIII (PDP8) và Chiến lược quốc gia về biến đổi khí hậu để hướng tới mục tiêu phát thải ròng bằng 0 vào năm 2050. Các kế hoạch tập trung vào việc loại bỏ dần điện than vào năm 2050, đẩy mạnh phát triển năng lượng tái tạo như điện gió ngoài khơi và hiện đại hóa hệ thống lưới điện truyền tải.</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5000,17 +5000,17 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Roadmap for Vietnam's carbon exchange | NetZero.VN — To realize its net-zero by 2050 target, Vietnam is currently promoting a wide range of emission reduction projects across industrial production, ...</t>
+          <t>베트남 정부는 2050년 넷제로 목표 달성을 위해 국내 탄소 거래소 설립에 관한 시행령 제29/2026/ND-CP호를 공표했습니다. 이 거래소는 2026년 말 공식 운영을 시작할 예정이며, 기업들의 저탄소 기술 투자 유도와 국제 탄소 시장 연결을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Roadmap for Vietnam's carbon exchange | NetZero.VN — To realize its net-zero by 2050 target, Vietnam is currently promoting a wide range of emission reduction projects across industrial production, ...</t>
+          <t>The Vietnamese government issued Decree No. 29/2026/ND-CP to establish a domestic carbon exchange, supporting the country's goal of achieving net-zero emissions by 2050. The exchange is expected to begin official operations by the end of 2026, providing a transparent platform for trading emission allowances and carbon credits.</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Roadmap for Vietnam's carbon exchange | NetZero.VN — To realize its net-zero by 2050 target, Vietnam is currently promoting a wide range of emission reduction projects across industrial production, ...</t>
+          <t>Chính phủ Việt Nam đã ban hành Nghị định số 29/2026/NĐ-CP về sàn giao dịch tín chỉ carbon trong nước nhằm hiện thực hóa mục tiêu phát thải ròng bằng 0 vào năm 2050. Sàn giao dịch dự kiến sẽ chính thức đi vào vận hành từ cuối năm 2026, tạo nền tảng minh bạch để các doanh nghiệp trao đổi hạn ngạch phát thải và tín chỉ carbon.</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5060,17 +5060,17 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Reporting on Vietnam's Pathways to Net Zero — The government of Vietnam approved a National Climate Change Strategy on 26 July 2022 to meet its pledge to become a net-zero carbon emissions country by 2050. (관련: VN-CARBON-2050)</t>
+          <t>베트남 정부는 2050년까지 탄소 중립을 달성하기 위한 '국가 기후 변화 전략'을 수립하고 재생 에너지 비중을 확대하고 있습니다. 이에 따라 Internews의 지구 저널리즘 네트워크(EJN)는 현지 언론인의 에너지 전환 보도 역량을 강화하기 위한 교육 및 지원 프로젝트를 운영하고 있습니다.</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Reporting on Vietnam's Pathways to Net Zero — The government of Vietnam approved a National Climate Change Strategy on 26 July 2022 to meet its pledge to become a net-zero carbon emissions country by 2050. (Related: VN-CARBON-2050)</t>
+          <t>The Vietnamese government has launched a National Climate Change Strategy to reach net-zero emissions by 2050, focusing on increasing renewable energy and cutting land-use emissions. Internews’ Earth Journalism Network (EJN) is supporting this transition by providing training, grants, and mentorship to local journalists to improve the quality of reporting on Vietnam's energy pathways.</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Reporting on Vietnam's Pathways to Net Zero — The government of Vietnam approved a National Climate Change Strategy on 26 July 2022 to meet its pledge to become a net-zero carbon emissions country by 2050. (Liên quan: VN-CARBON-2050)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Chiến lược quốc gia về biến đổi khí hậu nhằm đạt mục tiêu phát thải ròng bằng 0 vào năm 2050 thông qua chuyển đổi năng lượng và bảo vệ rừng. Dự án của Mạng lưới Báo chí Trái đất (EJN) đang hỗ trợ các phóng viên trong nước nâng cao kỹ năng truyền thông và kiến thức chuyên môn để phản ánh lộ trình tiến tới Net Zero của quốc gia.</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5124,17 +5124,17 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's 2050 Net-Zero Target Represents a $2.4 Trillion Opportunity — In this net-zero pathway, three drivers account for 78% of Vietnam's emissions abatement through to mid-century: clean power, carbon capture and ...</t>
+          <t>블룸버그NEF 보고서에 따르면 베트남이 2050년 넷제로 목표를 달성하기 위해서는 2.4조 달러 규모의 투자가 필요하며, 이는 재생 에너지와 탄소 포집 기술의 급격한 확대를 동반해야 합니다. 특히 태양광 및 풍력 발전은 2026년까지 전력 부문의 탄소 배출 정점을 달성하는 데 핵심적인 역할을 할 것으로 전망됩니다.</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's 2050 Net-Zero Target Represents a $2.4 Trillion Opportunity — In this net-zero pathway, three drivers account for 78% of Vietnam's emissions abatement through to mid-century: clean power, carbon capture and ...</t>
+          <t>According to a BloombergNEF report, Vietnam requires $2.4 trillion in investment to reach its 2050 net-zero target, necessitating a rapid scale-up of renewable energy and carbon capture technologies. The transition focuses on peaking power sector emissions by 2026 through massive solar and wind deployment while electrifying the transport sector by 2029.</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's 2050 Net-Zero Target Represents a $2.4 Trillion Opportunity — In this net-zero pathway, three drivers account for 78% of Vietnam's emissions abatement through to mid-century: clean power, carbon capture and ...</t>
+          <t>Báo cáo của BloombergNEF cho thấy Việt Nam cần huy động 2,4 nghìn tỷ USD đầu tư để đạt mục tiêu phát thải ròng bằng không vào năm 2050 thông qua việc đẩy mạnh năng lượng tái tạo và xe điện. Lộ trình này dự kiến giúp phát thải ngành điện đạt đỉnh vào năm 2026 và thúc đẩy tiềm năng trở thành trung tâm sản xuất xanh cho các tập đoàn đa quốc gia.</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5188,17 +5188,17 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam's shift to green growth | Vietnam Today - YouTube — Việt Nam's commitment to achieving net-zero emissions by 2050, announced at COP26, has triggered a fundamental shift in its economic ... (관련: VN-EV-2030)</t>
+          <t>베트남은 COP26에서 2050년까지 탄소 중립을 달성하겠다고 선언하며 경제 구조를 녹색 성장으로 전환하고 있습니다. 이러한 변화는 환경 및 기후 분야의 인프라 구축과 지속 가능한 발전을 촉진하는 중요한 계기가 되었습니다.</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam's shift to green growth | Vietnam Today - YouTube — Việt Nam's commitment to achieving net-zero emissions by 2050, announced at COP26, has triggered a fundamental shift in its economic ... (Related: VN-EV-2030)</t>
+          <t>Vietnam is fundamentally shifting its economic trajectory toward green growth following its COP26 commitment to reach net-zero emissions by 2050. This transition highlights a strategic focus on climate-resilient infrastructure and sustainable development within the Environment and Climate sector.</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam's shift to green growth | Vietnam Today - YouTube — Việt Nam's commitment to achieving net-zero emissions by 2050, announced at COP26, has triggered a fundamental shift in its economic ... (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang chuyển đổi mạnh mẽ lộ trình kinh tế sang hướng tăng trưởng xanh sau cam kết đạt phát thải ròng bằng 0 vào năm 2050 tại COP26. Sự thay đổi này thúc đẩy phát triển hạ tầng bền vững và các giải pháp thích ứng với biến đổi khí hậu theo định hướng kế hoạch VN-EV-2030.</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5252,17 +5252,17 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Net-zero emissions by 2050: Vietnam's action-driven commitment — The ministry is also preparing Vietnam's updated Nationally Determined Contribution for 2026-2035, known as NDC 3.0, with flexible emissions ...</t>
+          <t>베트남은 2050년까지 탄소 중립(Net-Zero) 달성을 단순한 외교적 약속이 아닌 국가적 정치 과제로 설정하고, 전기차 보급 확대 및 녹색 금융 활성화를 추진하고 있습니다. 팜 민 찐 총리는 이를 위해 제도 개선, 녹색 금융 동원, 기술 이전 가속화 등 5대 우선순위를 발표하며 지속 가능한 발전을 강조했습니다.</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Net-zero emissions by 2050: Vietnam's action-driven commitment — The ministry is also preparing Vietnam's updated Nationally Determined Contribution for 2026-2035, known as NDC 3.0, with flexible emissions ...</t>
+          <t>Vietnam has reaffirmed its commitment to achieving net-zero emissions by 2050 as a core political mission, focusing on green growth and energy transition across sectors like transport and agriculture. Prime Minister Pham Minh Chinh outlined key priorities including institutional improvements, mobilizing green finance, and accelerating technology transfer to drive sustainable development.</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Net-zero emissions by 2050: Vietnam's action-driven commitment — The ministry is also preparing Vietnam's updated Nationally Determined Contribution for 2026-2035, known as NDC 3.0, with flexible emissions ...</t>
+          <t>Việt Nam khẳng định mục tiêu đạt phát thải ròng bằng 0 vào năm 2050 không chỉ là lời hứa ngoại giao mà là một nhiệm vụ chính trị gắn liền với phát triển xanh và bền vững. Thủ tướng Phạm Minh Chính đã nêu rõ 5 ưu tiên chính gồm hoàn thiện thể chế, huy động tài chính xanh, chuyển giao công nghệ, quản trị thông minh và phát triển nguồn nhân lực.</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -5316,17 +5316,17 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>[Water Resources] ℹ The Mekong Flood and Drought Forecast ... — #Laos is currently experiencing significant flooding due to rising water levels in the #MekongRiver and its tributaries, exacerbated by ... (관련: VN-WAT-2050, VN-EV-2030)</t>
+          <t>ℹ The Mekong Flood and Drought Forecast ...</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>[Water Resources] ℹ The Mekong Flood and Drought Forecast ... — #Laos is currently experiencing significant flooding due to rising water levels in the #MekongRiver and its tributaries, exacerbated by ... (Related: VN-WAT-2050, VN-EV-2030)</t>
+          <t>ℹ The Mekong Flood and Drought Forecast ...</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>[Water Resources] ℹ The Mekong Flood and Drought Forecast ... — #Laos is currently experiencing significant flooding due to rising water levels in the #MekongRiver and its tributaries, exacerbated by ... (Liên quan: VN-WAT-2050, VN-EV-2030)</t>
+          <t>ℹ The Mekong Flood and Drought Forecast ...</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5380,17 +5380,17 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Floods in Vietnam: Will rising waters tame the Rising Dragon? — Vietnam faces mounting flood risk as climate change, land subsidence, and hydropower infrastructure combine with record typhoon activity.</t>
+          <t>베트남의 급격한 경제 성장과 수력 발전소 네트워크는 퇴적물 차단과 유량 변화를 유발하여 홍수 위험을 심화시키고 있습니다. 특히 호아빈 댐과 같은 전력 인프라는 하류 지역의 토양 보충을 방해하고 비상 방류 시 홍수 피해를 가중시키는 주요 요인으로 지목되었습니다.</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Floods in Vietnam: Will rising waters tame the Rising Dragon? — Vietnam faces mounting flood risk as climate change, land subsidence, and hydropower infrastructure combine with record typhoon activity.</t>
+          <t>Vietnam's rapid economic development and dense hydropower network are increasing flood risks through sediment trapping and altered water flows. Key energy infrastructure, such as the Hoa Binh Dam, contributes to downstream vulnerability by blocking essential sediment delivery and exacerbating floods during emergency water releases.</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Floods in Vietnam: Will rising waters tame the Rising Dragon? — Vietnam faces mounting flood risk as climate change, land subsidence, and hydropower infrastructure combine with record typhoon activity.</t>
+          <t>Sự phát triển kinh tế nhanh chóng và mạng lưới thủy điện dày đặc tại Việt Nam đang làm tăng nguy cơ lũ lụt thông qua việc bẫy trầm tích và thay đổi dòng chảy. Các cơ sở hạ tầng năng lượng như đập Hòa Bình đã góp phần làm trầm trọng thêm tình trạng ngập lụt ở hạ lưu do ngăn chặn bồi đắp phù sa và xả lũ khẩn cấp trong các đợt thiên tai.</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5440,17 +5440,17 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>[Water Resources] [PDF] Cumulative impact dams and climate change on the hydrology of the ... — More than 1,000 hydropower and irrigation reservoirs/ponds have been built in the. Mekong basin, and another 350 hydropower and irrigation dams are proposed. (관련: VN-WAT-2050)</t>
+          <t>[PDF] Cumulative impact dams and climate change on the hydrology of the ...</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>[Water Resources] [PDF] Cumulative impact dams and climate change on the hydrology of the ... — More than 1,000 hydropower and irrigation reservoirs/ponds have been built in the. Mekong basin, and another 350 hydropower and irrigation dams are proposed. (Related: VN-WAT-2050)</t>
+          <t>[PDF] Cumulative impact dams and climate change on the hydrology of the ...</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>[Water Resources] [PDF] Cumulative impact dams and climate change on the hydrology of the ... — More than 1,000 hydropower and irrigation reservoirs/ponds have been built in the. Mekong basin, and another 350 hydropower and irrigation dams are proposed. (Liên quan: VN-WAT-2050)</t>
+          <t>[PDF] Cumulative impact dams and climate change on the hydrology of the ...</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5504,17 +5504,17 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>[Water Resources] Drought and salinity expected near average levels this dry season — Drought and water shortages during the 2025-2026 dry season are expected to occur mainly in localized areas, while saltwater intrusion in ... (관련: VN-EV-2030)</t>
+          <t>Drought and salinity expected near average levels this dry season</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>[Water Resources] Drought and salinity expected near average levels this dry season — Drought and water shortages during the 2025-2026 dry season are expected to occur mainly in localized areas, while saltwater intrusion in ... (Related: VN-EV-2030)</t>
+          <t>Drought and salinity expected near average levels this dry season</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>[Water Resources] Drought and salinity expected near average levels this dry season — Drought and water shortages during the 2025-2026 dry season are expected to occur mainly in localized areas, while saltwater intrusion in ... (Liên quan: VN-EV-2030)</t>
+          <t>Drought and salinity expected near average levels this dry season</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5568,17 +5568,17 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>[Water Resources] Mekong Flood and Drought Forecast Channel on 13 January 2026 — ... Vietnamese) ☀️Drought forecast: Mild drought ... Water levels updates: ⬆️Water levels from Chiang ... (관련: VN-WAT-2050, VN-EV-2030)</t>
+          <t>메콩강 위원회(MRC)는 2026년 1월 13일자 메콩강 홍수 및 가뭄 예측 보고서를 발표했습니다. 이 보고서는 베트남의 수자원 인프라 관리 및 VN-WAT-2050 계획에 필수적인 하류 지역의 수위 변화와 기상 정보를 제공합니다.</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>[Water Resources] Mekong Flood and Drought Forecast Channel on 13 January 2026 — ... Vietnamese) ☀️Drought forecast: Mild drought ... Water levels updates: ⬆️Water levels from Chiang ... (Related: VN-WAT-2050, VN-EV-2030)</t>
+          <t>The Mekong River Commission released its flood and drought forecast for January 13, 2026, focusing on water levels across the Mekong basin. This data supports Vietnam's water resource management and infrastructure planning under frameworks like VN-WAT-2050 and VN-EV-2030.</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>[Water Resources] Mekong Flood and Drought Forecast Channel on 13 January 2026 — ... Vietnamese) ☀️Drought forecast: Mild drought ... Water levels updates: ⬆️Water levels from Chiang ... (Liên quan: VN-WAT-2050, VN-EV-2030)</t>
+          <t>Ủy ban Sông Mê Công đã công bố bản tin dự báo lũ và hạn hán ngày 13 tháng 1 năm 2026 cho khu vực hạ lưu sông. Thông tin này đóng vai trò quan trọng trong việc vận hành cơ sở hạ tầng tài nguyên nước của Việt Nam theo các quy hoạch VN-WAT-2050 và VN-EV-2030.</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5632,17 +5632,17 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>[Water Resources] Mekong Delta races to respond to peak flood levels — Water levels on the Mekong River are rising rapidly and expected to peak in the coming days, according to meteorological agencies. (관련: VN-EV-2030)</t>
+          <t>메콩강의 수위가 빠르게 상승하고 있으며 앞으로 며칠 내에 정점에 도달할 것으로 예보되었습니다. 남부 지역 당국은 시장, 도로, 주거 지역 침수와 같은 피해를 줄이기 위해 경고 발령과 재해 방지 조치를 신속하게 시행하고 있습니다.</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>[Water Resources] Mekong Delta races to respond to peak flood levels — Water levels on the Mekong River are rising rapidly and expected to peak in the coming days, according to meteorological agencies. (Related: VN-EV-2030)</t>
+          <t>Water levels on the Mekong River are rising rapidly and are forecast to peak between October 8 and 10, causing severe flooding in Can Tho City and other parts of the Mekong Delta. Local authorities are issuing flood warnings and implementing emergency measures to protect vulnerable infrastructure and residents.</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>[Water Resources] Mekong Delta races to respond to peak flood levels — Water levels on the Mekong River are rising rapidly and expected to peak in the coming days, according to meteorological agencies. (Liên quan: VN-EV-2030)</t>
+          <t>Mực nước sông Mê Kông đang tăng nhanh và dự báo sẽ đạt đỉnh từ ngày 8 đến 10 tháng 10, gây ngập lụt nghiêm trọng tại thành phố Cần Thơ và các khu vực khác ở đồng bằng sông Cửu Long. Chính quyền địa phương đang triển khai nhiều biện pháp cảnh báo ngập lụt và bảo vệ cơ sở hạ tầng, cư dân khu vực dễ bị ảnh hưởng.</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5696,17 +5696,17 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City Charts A New Path For Urban ... — The city is piloting a new approach: integrating digital transformation, green growth, and modern finance to restructure urban space, ...</t>
+          <t>호치민시는 디지털 전환과 녹색 성장을 통합한 '이중 전환' 전략을 통해 2050년까지 저탄소 메가시티로의 도약을 목표로 하고 있습니다. 도시는 인공지능(AI), 반도체 등 하이테크 산업 육성과 국제금융센터(IFC) 구축을 포함한 5대 핵심 발전축을 기반으로 다극 성장 모델을 추진하고 있습니다.</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City Charts A New Path For Urban ... — The city is piloting a new approach: integrating digital transformation, green growth, and modern finance to restructure urban space, ...</t>
+          <t>Ho Chi Minh City is implementing a dual transformation strategy that integrates digital and green growth to become a low-carbon mega-city by 2050. The development focuses on five strategic pillars, including high-tech industries like AI and semiconductors, and the establishment of an International Financial Center to enhance global competitiveness.</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City Charts A New Path For Urban ... — The city is piloting a new approach: integrating digital transformation, green growth, and modern finance to restructure urban space, ...</t>
+          <t>Thành phố Hồ Chí Minh đang triển khai chiến lược chuyển đổi kép, kết hợp giữa chuyển đổi số và tăng trưởng xanh để trở thành siêu đô thị phát thải thấp vào năm 2050. Thành phố tập trung vào mô hình tăng trưởng đa cực với 5 trụ cột chiến lược, bao gồm phát triển công nghệ cao, trung tâm tài chính quốc tế và hiện đại hóa quản trị đô thị.</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5760,17 +5760,17 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Ho Chi Minh City outlines roadmap of new urban development — To reach double-digit growth, Ho Chi Minh City is adding three new pillars, including VIFC-HCM, urban railways and a Free Trade Zone. (관련: VN-EV-2030)</t>
+          <t>호치민시는 메트로 2호선 건설과 국제금융센터(VIFC-HCM) 및 자유무역지대 조성을 포함한 새로운 도시 개발 로드맵을 발표했습니다. 이 계획은 행정 구역 통합과 교통 인프라 확충을 통해 2050년까지 인구 2,000만 명 규모의 글로벌 메가시티로 도약하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Ho Chi Minh City outlines roadmap of new urban development — To reach double-digit growth, Ho Chi Minh City is adding three new pillars, including VIFC-HCM, urban railways and a Free Trade Zone. (Related: VN-EV-2030)</t>
+          <t>Ho Chi Minh City has unveiled a strategic roadmap focusing on three new pillars: a financial center, urban railways including Metro Line No. 2, and a Free Trade Zone. The plan aims to transform the city into a regional megacity by 2050, leveraging integrated transport networks and administrative consolidation to drive double-digit economic growth.</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Ho Chi Minh City outlines roadmap of new urban development — To reach double-digit growth, Ho Chi Minh City is adding three new pillars, including VIFC-HCM, urban railways and a Free Trade Zone. (Liên quan: VN-EV-2030)</t>
+          <t>Thành phố Hồ Chí Minh đã công bố lộ trình phát triển đô thị mới với ba trụ cột chiến lược gồm Trung tâm Tài chính Quốc tế, đường sắt đô thị (tuyến Metro số 2) và Khu thương mại tự do. Kế hoạch này hướng tới mục tiêu đưa thành phố trở thành siêu đô thị khu vực vào năm 2050 thông qua việc kết nối hạ tầng giao thông đồng bộ và cải cách quản trị.</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5824,17 +5824,17 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>[Urban Development] Satellite cities to be centres of real estate development for ... — The urbanisation rate is projected at 50 per cent, equivalent to 51 million urban residents, while the middle class could expand to 75 per cent ... (관련: VN-EV-2030)</t>
+          <t>베트남은 490억 달러 규모의 인프라 투자를 통해 남북 고속도로와 롱타 Thành 국제공항 등을 건설하며 도시 지형을 재편하고 있습니다. 새빌스 베트남은 급격한 도시화와 위성 도시의 성장이 향후 10년간 부동산 개발의 핵심이 될 것으로 전망했습니다.</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>[Urban Development] Satellite cities to be centres of real estate development for ... — The urbanisation rate is projected at 50 per cent, equivalent to 51 million urban residents, while the middle class could expand to 75 per cent ... (Related: VN-EV-2030)</t>
+          <t>Vietnam is investing US$49 billion in nationwide infrastructure, including major expressways and airports, to redefine its urban landscape and connect emerging growth hubs. Savills Vietnam predicts that satellite cities and rapid urbanization will drive the real estate market over the next decade, supported by a growing middle class and high-tech industrial shifts.</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>[Urban Development] Satellite cities to be centres of real estate development for ... — The urbanisation rate is projected at 50 per cent, equivalent to 51 million urban residents, while the middle class could expand to 75 per cent ... (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang triển khai 49 tỷ USD vào hạ tầng chiến lược như cao tốc Bắc-Nam và sân bay Long Thành để kết nối các hành lang phát triển kinh tế. Savills dự báo các đô thị vệ tinh sẽ trở thành trọng tâm phát triển bất động sản trong thập kỷ tới nhờ tốc độ đô thị hóa nhanh và sự gia tăng của tầng lớp trung lưu.</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -5888,17 +5888,17 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City moves to real smart urban governance in ... — Ho Chi Minh City is building a governance model where real-time data, AI and digital twins guide decisions and reshape daily urban life.</t>
+          <t>호치민시는 2026년까지 데이터 표준화와 AI 기술을 활용하여 진정한 스마트 도시 거버넌스로 전환할 계획입니다. 시민 앱과 스마트 도시 운영 센터를 통해 교통 체증 및 홍수 예측 등 실시간 데이터 기반의 공공 서비스를 제공하고자 합니다.</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City moves to real smart urban governance in ... — Ho Chi Minh City is building a governance model where real-time data, AI and digital twins guide decisions and reshape daily urban life.</t>
+          <t>By 2026, Ho Chi Minh City aims to transition to a smart urban governance model by standardizing data and integrating AI and Digital Twin technology. The initiative focuses on enhancing public services through the Citizen App and a centralized Operations Center to manage traffic, flooding, and administrative procedures in real-time.</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City moves to real smart urban governance in ... — Ho Chi Minh City is building a governance model where real-time data, AI and digital twins guide decisions and reshape daily urban life.</t>
+          <t>Đến năm 2026, TP.HCM sẽ tập trung chuẩn hóa dữ liệu và ứng dụng AI để vận hành hệ thống quản trị đô thị thông minh thực thụ. Thành phố hướng tới việc chuyển đổi dịch vụ công từ "xử lý hồ sơ" sang "phục vụ nhu cầu" thông qua Ứng dụng Công dân và Trung tâm Điều hành Đô thị Thông minh.</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -5952,17 +5952,17 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam's Ho Chi Minh City adopts multi-center urban model — The project, linking Ben Thanh to Can Gio, is being positioned as a major infrastructure upgrade that could reshape mobility, tourism, and real ...</t>
+          <t>호치민시는 파편화된 개발을 해결하기 위해 '1공간-3지역-1특구' 체계의 다중심 도시 모델을 도입하여 메가시티로의 도약을 준비하고 있습니다. 메트로 시스템과 지역 교통망을 중심으로 한 대중교통 지향 개발(TOD) 모델을 통해 2030년까지 핵심 교통망 완성을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam's Ho Chi Minh City adopts multi-center urban model — The project, linking Ben Thanh to Can Gio, is being positioned as a major infrastructure upgrade that could reshape mobility, tourism, and real ...</t>
+          <t>Ho Chi Minh City is adopting a multi-center urban model under a "one space – three regions – one special zone" framework to transform into a sustainable megacity. The plan prioritizes Transit-Oriented Development (TOD), focusing on metro systems and regional transport to link finance, high-tech, and maritime economic hubs by 2030.</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam's Ho Chi Minh City adopts multi-center urban model — The project, linking Ben Thanh to Can Gio, is being positioned as a major infrastructure upgrade that could reshape mobility, tourism, and real ...</t>
+          <t>Thành phố Hồ Chí Minh đang triển khai mô hình đô thị đa trung tâm với khung sườn "một trục – ba vùng – một khu vực đặc thù" để hướng tới mục tiêu siêu đô thị bền vững. Kế hoạch tập trung vào mô hình phát triển đô thị gắn kết với giao thông công cộng (TOD), ưu tiên hoàn thiện mạng lưới metro và hạ tầng kết nối vùng trước năm 2030.</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6016,17 +6016,17 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam set for US$115bil mega urban projects — Vietnam had 27 large-scale urban development projects with combined investment exceeding three quadrillion dong (US$115bil) in 2025, ... (관련: VN-EV-2030)</t>
+          <t>베트남은 빈그룹(Vingroup)과 선그룹(Sun Group) 등 주요 개발사들의 주도로 총 1,150억 달러 규모의 27개 대형 도시 개발 프로젝트를 추진하고 있습니다. 법적 규제 완화와 인프라 확장을 통해 하노이와 호치민 인근에 대규모 신도시가 건설 중이나, 급격한 가격 상승에 따른 주택 공급 흡수 능력에 대한 우려도 제기되고 있습니다.</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam set for US$115bil mega urban projects — Vietnam had 27 large-scale urban development projects with combined investment exceeding three quadrillion dong (US$115bil) in 2025, ... (Related: VN-EV-2030)</t>
+          <t>Vietnam is launching 27 mega urban development projects worth $115 billion, led by major developers like Vingroup and Sun Group across the Northern, Central, and Southern regions. These projects, including the massive $35.6 billion Olympic sports urban area in Hanoi, are supported by improved legal frameworks and expanding infrastructure but face challenges regarding housing affordability and market absorption.</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>[Urban Development] Vietnam set for US$115bil mega urban projects — Vietnam had 27 large-scale urban development projects with combined investment exceeding three quadrillion dong (US$115bil) in 2025, ... (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang triển khai 27 dự án đô thị quy mô lớn với tổng vốn đầu tư lên tới 115 tỷ USD, tập trung tại ba miền Bắc, Trung và Nam dưới sự dẫn dắt của các tập đoàn lớn như Vingroup và Sun Group. Mặc dù các cải cách pháp lý và cơ sở hạ tầng đang thúc đẩy làn sóng phát triển này, các chuyên gia vẫn cảnh báo về áp lực giá nhà tăng cao và khả năng hấp thụ của thị trường.</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6080,17 +6080,17 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>[Urban Development] Cushman &amp; Wakefield Spotlights Vietnam's Next Urban ... — The country is now entering a more mature phase of development, where growth is increasingly defined not only by scale, but by productivity, ... (관련: VN-EV-2030)</t>
+          <t>베트남은 2030년까지 동남아시아 3위 경제 대국으로 도약하기 위해 단순 확장을 넘어 전략적 인프라와 통합 도시 계획 중심의 질적 성장을 추진하고 있습니다. 첨단 기술 중심의 FDI 유치와 함께 주거, 교육, 의료가 결합된 복합 도시 구역 개발을 통해 장기적인 도시 경쟁력을 강화할 계획입니다.</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>[Urban Development] Cushman &amp; Wakefield Spotlights Vietnam's Next Urban ... — The country is now entering a more mature phase of development, where growth is increasingly defined not only by scale, but by productivity, ... (Related: VN-EV-2030)</t>
+          <t>Vietnam is transitioning toward a high-quality urban growth model that integrates strategic infrastructure, innovation, and sustainable planning to become Southeast Asia’s third-largest economy by 2030. The focus is shifting from fragmented expansion to developing integrated mega-townships and high-tech investment hubs in sectors like semiconductors and AI.</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>[Urban Development] Cushman &amp; Wakefield Spotlights Vietnam's Next Urban ... — The country is now entering a more mature phase of development, where growth is increasingly defined not only by scale, but by productivity, ... (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang chuyển mình sang giai đoạn phát triển đô thị chất lượng cao, kết hợp chặt chẽ giữa quy hoạch tích hợp và đầu tư hạ tầng chiến lược nhằm hướng tới mục tiêu trở thành nền kinh tế lớn thứ ba khu vực vào năm 2030. Quốc gia đang ưu tiên phát triển các khu đô thị phức hợp bền vững và thu hút đầu tư vào các ngành công nghệ cao như bán dẫn và trí tuệ nhân tạo.</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6144,17 +6144,17 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>[Urban Development] New urbanisation cycle set to define Vietnam's next ... — Vietnam is shifting to sustainable growth, with urban planning and infrastructure set to define the next decade.</t>
+          <t>베트남은 2030년까지 전략적 인프라 개발과 통합 도시 계획을 통해 단순한 확장을 넘어 고부가가치 성장의 새로운 도시화 주기에 진입하고 있습니다. 쿠시먼앤드웨이크필드는 향후 도시 개발이 주거 공급을 넘어 일자리, 교육, 의료가 결합된 복합 생태계를 구축하는 데 집중될 것이라고 전망했습니다.</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>[Urban Development] New urbanisation cycle set to define Vietnam's next ... — Vietnam is shifting to sustainable growth, with urban planning and infrastructure set to define the next decade.</t>
+          <t>Vietnam is entering a new urbanization cycle focused on strategic infrastructure development and integrated urban planning to achieve high-value growth by 2030. Experts emphasize that future development must move beyond mere housing to create complete ecosystems that align infrastructure with employment clusters and quality living environments.</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>[Urban Development] New urbanisation cycle set to define Vietnam's next ... — Vietnam is shifting to sustainable growth, with urban planning and infrastructure set to define the next decade.</t>
+          <t>Việt Nam đang bước vào chu kỳ đô thị hóa mới tập trung vào phát triển hạ tầng chiến lược và quy hoạch đô thị tích hợp để đạt được tăng trưởng giá trị cao vào năm 2030. Các chuyên gia nhấn mạnh rằng phát triển trong tương lai phải vượt xa việc chỉ cung cấp nhà ở để tạo ra các hệ sinh thái hoàn chỉnh, kết nối hạ tầng với các cụm việc làm và môi trường sống chất lượng.</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6208,17 +6208,17 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City targets global Top 50 smart cities by 2030 — Ho Chi Minh City aims to rank among the world's top 50 smart cities by 2030 under a draft smart urban development plan for 2026–2030, ... (관련: VN-EV-2030)</t>
+          <t>호치민시는 2030년까지 세계 50대 스마트 시티 진입을 목표로 하는 도시 개발 계획을 발표했습니다. 이 계획은 단순한 기술 도입을 넘어 데이터 기반의 거버넌스 혁신과 디지털 트윈 기술 구축에 중점을 두고 있습니다.</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City targets global Top 50 smart cities by 2030 — Ho Chi Minh City aims to rank among the world's top 50 smart cities by 2030 under a draft smart urban development plan for 2026–2030, ... (Related: VN-EV-2030)</t>
+          <t>Ho Chi Minh City aims to rank among the world's top 50 smart cities by 2030, focusing on data-driven governance and digital twin technology. The plan prioritizes institutional reform and infrastructure development to serve as a national hub for innovation by 2035.</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City targets global Top 50 smart cities by 2030 — Ho Chi Minh City aims to rank among the world's top 50 smart cities by 2030 under a draft smart urban development plan for 2026–2030, ... (Liên quan: VN-EV-2030)</t>
+          <t>Thành phố Hồ Chí Minh đặt mục tiêu lọt vào nhóm 50 thành phố thông minh hàng đầu thế giới vào năm 2030 thông qua việc chuyển đổi quản trị dựa trên dữ liệu. Kế hoạch ưu tiên xây dựng hạ tầng số, hệ thống bản sao số (digital twin) và cải cách thể chế để trở thành trung tâm điều hành thông minh quốc gia vào năm 2035.</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6272,17 +6272,17 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City And Hanoi Redefine Urban Futures — On the cusp of 2026, two of Vietnam's most dynamic cities—Ho Chi Minh City and Hanoi—are charting bold, divergent courses in urban development. (관련: VN-EV-2030)</t>
+          <t>베트남의 양대 도시인 호찌민과 하노이는 2026년을 기점으로 혁신적인 도시 개발 계획을 추진하고 있습니다. 호찌민은 '더 글로벌 시티'와 같은 대규모 통합 도시 프로젝트를 통해 거주와 상업이 결합된 환경을 구축하고 있으며, 하노이는 교통 혼잡 해결을 위해 1,000m 이하의 '저고도 경제'와 드론 물류 시스템 도입에 집중하고 있습니다.</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City And Hanoi Redefine Urban Futures — On the cusp of 2026, two of Vietnam's most dynamic cities—Ho Chi Minh City and Hanoi—are charting bold, divergent courses in urban development. (Related: VN-EV-2030)</t>
+          <t>Ho Chi Minh City and Hanoi are redefining their urban landscapes by 2026 through divergent infrastructure strategies. Ho Chi Minh City is focusing on integrated mega-projects like 'The Global City' to create holistic living environments, while Hanoi is pioneering a 'low-altitude economy' using UAVs and eVTOLs to bypass ground-level traffic congestion and modernize logistics.</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>[Urban Development] Ho Chi Minh City And Hanoi Redefine Urban Futures — On the cusp of 2026, two of Vietnam's most dynamic cities—Ho Chi Minh City and Hanoi—are charting bold, divergent courses in urban development. (Liên quan: VN-EV-2030)</t>
+          <t>Thành phố Hồ Chí Minh và Hà Nội đang định hình lại tương lai đô thị vào năm 2026 với những hướng đi đột phá. Trong khi TP.HCM tập trung vào các siêu dự án đô thị tích hợp như The Global City để tạo ra môi trường sống toàn diện, Hà Nội lại khai thác kinh tế tầm thấp dưới 1.000m, sử dụng flycam và thiết bị bay không người lái để tối ưu hóa hậu cần và giảm thiểu ùn tắc giao thông.</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6336,17 +6336,17 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>[Other] VinFast Records Biggest-Ever Single-Day Sales on April 11, 2026 ... — VinFast achieves record-breaking EV sales as global charging infrastructure expands, marking a shift from hype to practical adoption ... (관련: VN-EV-2030)</t>
+          <t>베트남의 선도적인 전기차 제조업체인 빈패스트(VinFast)는 2026년 4월 11일 사상 최대 일일 판매량을 기록하며 전기차 시장의 성숙을 알렸습니다. 이러한 성장은 베트남의 급속한 충전 인프라 확충과 정부의 친환경 에너지 정책 덕분에 가능했으며, 베트남은 글로벌 전기 모빌리티 분야의 핵심 국가로 부상하고 있습니다.</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>[Other] VinFast Records Biggest-Ever Single-Day Sales on April 11, 2026 ... — VinFast achieves record-breaking EV sales as global charging infrastructure expands, marking a shift from hype to practical adoption ... (Related: VN-EV-2030)</t>
+          <t>VinFast achieved record-breaking single-day sales on April 11, 2026, signaling a major transition toward mass-market EV adoption. This milestone is supported by Vietnam's rapid expansion of charging infrastructure and government mandates, positioning the country as a global powerhouse in the electric mobility sector.</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>[Other] VinFast Records Biggest-Ever Single-Day Sales on April 11, 2026 ... — VinFast achieves record-breaking EV sales as global charging infrastructure expands, marking a shift from hype to practical adoption ... (Liên quan: VN-EV-2030)</t>
+          <t>VinFast đã ghi nhận doanh số bán xe điện trong một ngày cao nhất lịch sử vào ngày 11 tháng 4 năm 2026, đánh dấu bước ngoặt chuyển dịch sang thị trường đại chúng. Thành tựu này được thúc đẩy bởi việc mở rộng nhanh chóng cơ sở hạ tầng sạc tại Việt Nam và các chính sách hỗ trợ của chính phủ, giúp quốc gia này trở thành trung tâm mới của ngành xe điện toàn cầu.</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6396,17 +6396,17 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] analyzing the public voice on electric vehicles and the rise of VinFast — Specifically, Hanoi will pilot a “Low Emission Zone” starting on July 1, 2026, which will restrict highly polluting gasoline vehicles from entering inner-city ... (관련: VN-EV-2030)</t>
+          <t>베트남은 2030년까지 하노이와 호치민시의 주요 교통수단을 전기차(EV)로 전환하는 국가 전략을 추진하고 있습니다. 2026년부터 하노이에 저배출 구역이 도입되고 호치민시는 2025년까지 모든 신규 공공 버스를 전기차로 교체할 계획이지만, 충전 인프라 확충은 여전히 시급한 과제로 남아 있습니다.</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] analyzing the public voice on electric vehicles and the rise of VinFast — Specifically, Hanoi will pilot a “Low Emission Zone” starting on July 1, 2026, which will restrict highly polluting gasoline vehicles from entering inner-city ... (Related: VN-EV-2030)</t>
+          <t>Vietnam is implementing a national strategy to make electric vehicles the primary mode of transport in Hanoi and Ho Chi Minh City by 2030. While initiatives include low-emission zones starting in 2026 and electric public buses by 2025, public discourse highlights that the success of this energy transition depends heavily on expanding the charging infrastructure ecosystem.</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] analyzing the public voice on electric vehicles and the rise of VinFast — Specifically, Hanoi will pilot a “Low Emission Zone” starting on July 1, 2026, which will restrict highly polluting gasoline vehicles from entering inner-city ... (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang thực hiện chiến lược quốc gia nhằm đưa xe điện trở thành phương tiện giao thông chính tại Hà Nội và TP.HCM vào năm 2030. Mặc dù các lộ trình như khu vực phát thải thấp (2026) và xe buýt điện (2025) đã được thiết lập, dư luận khẳng định rằng việc phát triển hạ tầng trạm sạc là yếu tố then chốt cho sự thành công của kế hoạch này.</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6460,17 +6460,17 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>[Other] VinFast's breakout year: Vietnamese EV maker nearly doubles sales ... — With nearly 200,000 EVs sold in 2025 and a 300,000-unit target for 2026, VinFast is no longer just an ambitious startup from Vietnam. It is ... (관련: VN-EV-2030)</t>
+          <t>베트남 전기차 제조업체 빈패스트(VinFast)는 2025년 전 세계적으로 약 20만 대의 차량을 인도하며 판매 실적을 두 배로 늘렸습니다. 이러한 성장은 베트남 내수 시장의 강력한 수요와 충전 네트워크 인프라 확장에 힘입은 결과이며, 회사는 2026년까지 30만 대 인도를 목표로 하고 있습니다.</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>[Other] VinFast's breakout year: Vietnamese EV maker nearly doubles sales ... — With nearly 200,000 EVs sold in 2025 and a 300,000-unit target for 2026, VinFast is no longer just an ambitious startup from Vietnam. It is ... (Related: VN-EV-2030)</t>
+          <t>Vietnamese EV maker VinFast nearly doubled its global sales in 2025 by delivering 196,919 vehicles, driven by a robust charging network and domestic demand. Following this record growth, the company has set an ambitious target of 300,000 deliveries for 2026 as it expands its international footprint.</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>[Other] VinFast's breakout year: Vietnamese EV maker nearly doubles sales ... — With nearly 200,000 EVs sold in 2025 and a 300,000-unit target for 2026, VinFast is no longer just an ambitious startup from Vietnam. It is ... (Liên quan: VN-EV-2030)</t>
+          <t>Nhà sản xuất xe điện VinFast đã gần như gấp đôi doanh số toàn cầu trong năm 2025 với 196.919 xe được bàn giao, nhờ vào sự bùng nổ của thị trường nội địa và hạ tầng trạm sạc. Công ty hiện đặt mục tiêu đầy tham vọng là đạt 300.000 xe trong năm 2026 để củng cố vị thế trên thị trường xe điện thế giới.</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6524,17 +6524,17 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vingroup Extends Emergency Support Program for Electric Vehicle ... — Vingroup Extends Emergency Support Program for Electric Vehicle Transition Until April 30, 2026, to Continue Alleviating Fuel Supply and ... (관련: VN-EV-2030)</t>
+          <t>빈그룹(Vingroup)은 베트남의 전기차 전환을 가속화하기 위해 긴급 지원 프로그램을 연장했습니다. 이 이니셔티브는 VN-EV-2030 계획에 따라 교통 인프라를 현대화하고 친환경 모빌리티 채택을 장려하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vingroup Extends Emergency Support Program for Electric Vehicle ... — Vingroup Extends Emergency Support Program for Electric Vehicle Transition Until April 30, 2026, to Continue Alleviating Fuel Supply and ... (Related: VN-EV-2030)</t>
+          <t>Vingroup has extended its emergency support program to facilitate the transition to electric vehicles in Vietnam. This move supports the VN-EV-2030 infrastructure plan by enhancing accessibility to green transport solutions across the country.</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vingroup Extends Emergency Support Program for Electric Vehicle ... — Vingroup Extends Emergency Support Program for Electric Vehicle Transition Until April 30, 2026, to Continue Alleviating Fuel Supply and ... (Liên quan: VN-EV-2030)</t>
+          <t>Tập đoàn Vingroup đã gia hạn chương trình hỗ trợ khẩn cấp cho quá trình chuyển đổi xe điện tại Việt Nam. Sáng kiến này đóng góp vào kế hoạch VN-EV-2030 nhằm thúc đẩy hạ tầng giao thông xanh và giảm thiểu phát thải.</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -6588,17 +6588,17 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam pushes EV shift as energy security risks mount — Incentives to support electric vehicle production and adoption are required to be introduced by June. (관련: VN-EV-2030)</t>
+          <t>베트남 정부는 에너지 안보 위기에 대응하기 위해 2026년 3분기까지 전기차 충전 인프라 표준을 마련하고 6월까지 생산 및 도입 인센티브를 발표할 계획입니다. 팜 민 찐 총리는 수입 연료 의존도를 낮추기 위해 공공 부문의 전기차 전환과 민간 충전 시설 확대를 가속화하라는 지침을 내렸습니다.</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam pushes EV shift as energy security risks mount — Incentives to support electric vehicle production and adoption are required to be introduced by June. (Related: VN-EV-2030)</t>
+          <t>Vietnam is accelerating its transition to electric vehicles (EV) to mitigate energy security risks and reduce reliance on imported fuels. The government has set deadlines to establish charging infrastructure standards by Q3 2026 and introduce EV production incentives by June, while pushing for the electrification of public fleets and urban residential projects.</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam pushes EV shift as energy security risks mount — Incentives to support electric vehicle production and adoption are required to be introduced by June. (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang đẩy mạnh chuyển đổi sang xe điện (EV) nhằm đảm bảo an ninh năng lượng và giảm phụ thuộc vào nhiên liệu nhập khẩu. Thủ tướng Phạm Minh Chính đã yêu cầu ban hành các quy chuẩn kỹ thuật cho trạm sạc vào quý 3 năm 2026 và các chính sách ưu đãi sản xuất xe điện trước tháng 6 tới.</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6648,17 +6648,17 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] The electric vehicle transition as a green window of opportunity ... — The general tendency of weak technology ownership in the Vietnamese automotive industry applies to locally made EVs. Vinfast sources key technologies such as ... (관련: VN-EV-2030)</t>
+          <t>베트남 정부는 2030년까지 도시 차량의 50%를 전기차로 전환하고 2050년까지 완전한 녹색 에너지 교통 체계를 구축한다는 '결정 제876/QD-TTg' 계획을 승인했습니다. 이에 따라 민간 기업인 빈패스트(Vinfast)는 전국에 15만 개의 충전 지점을 설치하며 인프라 구축을 주도하고 있으나, 규모의 경제 달성이 향후 과제로 남아있습니다.</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] The electric vehicle transition as a green window of opportunity ... — The general tendency of weak technology ownership in the Vietnamese automotive industry applies to locally made EVs. Vinfast sources key technologies such as ... (Related: VN-EV-2030)</t>
+          <t>The Vietnamese government has approved Decision 876/QD-TTg, targeting 50% of urban vehicles to be electric by 2030 and achieving a complete transition to green energy by 2050. Private leader Vinfast is driving this shift by installing 150,000 charging points nationwide, though the sector still faces significant entry barriers and the need for higher production scales.</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] The electric vehicle transition as a green window of opportunity ... — The general tendency of weak technology ownership in the Vietnamese automotive industry applies to locally made EVs. Vinfast sources key technologies such as ... (Liên quan: VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Quyết định 876/QD-TTg với mục tiêu 50% phương tiện đô thị sử dụng điện vào năm 2030 và chuyển đổi hoàn toàn sang năng lượng xanh vào năm 2050. Vinfast đang dẫn đầu nỗ lực này với việc lắp đặt 150.000 cổng sạc trên toàn quốc, tuy nhiên ngành vẫn đang đối mặt với thách thức lớn về quy mô sản xuất để duy trì tính bền vững.</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6712,17 +6712,17 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] The Future of Sustainable Vehicles in Vietnam - Milken Scholars — I traveled to Vietnam to learn more about VinFast's rapid rise and to investigate whether its pledge to promote a more sustainable energy ecosystem holds up in ...</t>
+          <t>베트남의 전기차 산업은 빈패스트(VinFast)를 중심으로 급성장하고 있으나, 전력 인프라와 에너지 생산의 지속가능성 문제가 남아있습니다. 현재 베트남 전력 생산의 약 80%는 석탄에 의존하고 있으며, 노후화된 전기 시스템과 충전소 부족이 인프라 확장의 주요 장애물로 지적됩니다.</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] The Future of Sustainable Vehicles in Vietnam - Milken Scholars — I traveled to Vietnam to learn more about VinFast's rapid rise and to investigate whether its pledge to promote a more sustainable energy ecosystem holds up in ...</t>
+          <t>Vietnam's electric vehicle market is expanding through VinFast's initiatives, but the country faces significant infrastructure challenges including a lack of public charging stations. Furthermore, approximately 80% of Vietnam's energy mix is still derived from coal, questioning the true environmental impact of EV adoption under the current power grid.</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] The Future of Sustainable Vehicles in Vietnam - Milken Scholars — I traveled to Vietnam to learn more about VinFast's rapid rise and to investigate whether its pledge to promote a more sustainable energy ecosystem holds up in ...</t>
+          <t>Thị trường xe điện Việt Nam đang phát triển mạnh mẽ thông qua VinFast, nhưng vẫn đối mặt với thách thức lớn về hạ tầng trạm sạc và hệ thống lưới điện cũ kỹ. Hiện nay, khoảng 80% sản lượng điện của Việt Nam vẫn dựa vào than đá, gây ra những nghi vấn về tính bền vững thực sự của xe điện đối với môi trường.</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6776,17 +6776,17 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>[Other] VinFast Extends Free Charging Policy Across Markets - LinkedIn — Vietnamese automotive company VINFAST has announced a three-year extension of its free charging policy across its operational markets.</t>
+          <t>베트남 자동차 제조사 빈패스트(VinFast)가 운영 시장 전역에서 무료 충전 정책을 3년 연장한다고 발표했습니다. 또한 모기업 빈그룹은 베트남을 포함한 주요국에서 내연기관차를 전기차로 전환할 시 할인 혜택을 제공하는 'Trade Gas for Electric' 프로그램을 시행합니다.</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>[Other] VinFast Extends Free Charging Policy Across Markets - LinkedIn — Vietnamese automotive company VINFAST has announced a three-year extension of its free charging policy across its operational markets.</t>
+          <t>Vietnamese automaker VinFast has announced a three-year extension of its free charging policy for private and commercial customers across its operational markets. Additionally, parent company Vingroup introduced the 'Trade Gas for Electric' initiative, offering discounts on electric cars and scooters through March 2026 to encourage the transition from petrol vehicles.</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>[Other] VinFast Extends Free Charging Policy Across Markets - LinkedIn — Vietnamese automotive company VINFAST has announced a three-year extension of its free charging policy across its operational markets.</t>
+          <t>Công ty ô tô Việt Nam VinFast đã thông báo gia hạn chính sách sạc miễn phí thêm ba năm tại các thị trường đang hoạt động. Bên cạnh đó, tập đoàn Vingroup cũng triển khai chương trình 'Đổi xe xăng lấy xe điện' với các ưu đãi giảm giá đặc biệt cho khách hàng chuyển đổi sang xe điện đến hết tháng 3 năm 2026.</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6840,17 +6840,17 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>[Other] Vietnam's EV market is gaining momentum In 2025, VinFast ... — Vietnamese EV maker VinFast has posted a 63% jump in electric vehicle deliveries in 2025, delivering 196,919 EVs and generating US$3.6 ... (관련: VN-EV-2030)</t>
+          <t>베트남 전기차 시장이 급성장하며 빈패스트가 2025년 약 175,000대의 판매고를 올려 업계 1위를 차지했습니다. 40만 대 이상의 전기 오토바이 판매와 인프라 개선이 동반되고 있으나, 여전히 충전소 확충과 내연기관차 규제 정책에 대한 논의가 진행 중입니다.</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>[Other] Vietnam's EV market is gaining momentum In 2025, VinFast ... — Vietnamese EV maker VinFast has posted a 63% jump in electric vehicle deliveries in 2025, delivering 196,919 EVs and generating US$3.6 ... (Related: VN-EV-2030)</t>
+          <t>Vietnam's EV market is surging, with VinFast leading the sector after delivering 175,000 electric cars and generating $3.6 billion in revenue in 2025. While electric motorbike sales exceeded 400,000 units, the country faces a transition phase involving infrastructure improvements and debates over gas-vehicle restrictions.</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>[Other] Vietnam's EV market is gaining momentum In 2025, VinFast ... — Vietnamese EV maker VinFast has posted a 63% jump in electric vehicle deliveries in 2025, delivering 196,919 EVs and generating US$3.6 ... (Liên quan: VN-EV-2030)</t>
+          <t>Thị trường xe điện Việt Nam đang bùng nổ khi VinFast đạt kỷ lục bàn giao 175.000 ô tô điện và trở thành thương hiệu dẫn đầu trong năm 2025. Bên cạnh đó, doanh số xe máy điện đạt hơn 400.000 chiếc, đánh dấu giai đoạn chuyển đổi mạnh mẽ dù vẫn còn những thách thức về hạ tầng trạm sạc.</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6904,17 +6904,17 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam outlines new plan to cut waste, protect coastal ... — HÀ NỘI — Việt Nam has launched a fresh push to curb pollution across its fisheries sector, warning that rising seas, degraded ecosystems and ...</t>
+          <t>베트남은 수산업 분야의 오염을 줄이고 해안 생태계를 보호하기 위해 2026-2030년 기간의 새로운 환경 보호 우선순위를 발표했습니다. 캐나다 대사관 및 UNDP와 협력하여 진행되는 이 계획은 기후 변화에 대응하고 폐기물 관리를 현대화하여 지속 가능한 수산물 생산을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam outlines new plan to cut waste, protect coastal ... — HÀ NỘI — Việt Nam has launched a fresh push to curb pollution across its fisheries sector, warning that rising seas, degraded ecosystems and ...</t>
+          <t>Vietnam has launched a new national plan for 2026–2030 to curb pollution in the fisheries sector and protect coastal ecosystems from climate change. Supported by Canada and the UNDP, the initiative focuses on waste reduction, mangrove restoration, and adopting cleaner technologies to ensure sustainable livelihoods for coastal communities.</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam outlines new plan to cut waste, protect coastal ... — HÀ NỘI — Việt Nam has launched a fresh push to curb pollution across its fisheries sector, warning that rising seas, degraded ecosystems and ...</t>
+          <t>Việt Nam vừa công bố kế hoạch mới giai đoạn 2026–2030 nhằm giảm thiểu ô nhiễm trong ngành thủy sản và bảo vệ hệ sinh thái ven biển. Với sự hỗ trợ từ Canada và UNDP, sáng kiến này tập trung vào kiểm soát chất lượng chất thải, phục hồi rừng ngập mặn và áp dụng công nghệ sạch để phát triển kinh tế biển bền vững.</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6968,17 +6968,17 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Study Reveals Water and Air Pollution Risks in Vietnam — Environmental study finds elevated lead, manganese, and PM2.5 pollution affecting workers and families near Hanoi's industrial zones. (관련: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>RTI International은 베트남의 산업 위험 연구를 통해 대기 및 수질 오염 문제 해결을 위한 과학적 솔루션을 제공합니다. 이 프로젝트는 환경 및 기후 분야의 인프라 발전을 목표로 하며 VN-ENV-IND-1894 및 VN-EV-2030 계획과 연계됩니다.</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Study Reveals Water and Air Pollution Risks in Vietnam — Environmental study finds elevated lead, manganese, and PM2.5 pollution affecting workers and families near Hanoi's industrial zones. (Related: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>RTI International conducts an industrial risk study on air and water pollution in Vietnam to provide science-based environmental solutions. This initiative supports infrastructure goals in the Environment &amp; Climate sector, aligning with the VN-ENV-IND-1894 and VN-EV-2030 strategic plans.</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Study Reveals Water and Air Pollution Risks in Vietnam — Environmental study finds elevated lead, manganese, and PM2.5 pollution affecting workers and families near Hanoi's industrial zones. (Liên quan: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>RTI International thực hiện nghiên cứu rủi ro công nghiệp về ô nhiễm không khí và nguồn nước tại Việt Nam nhằm đưa ra các giải pháp khoa học. Dự án này hỗ trợ phát triển hạ tầng trong lĩnh vực Môi trường &amp; Khí hậu, phù hợp với các kế hoạch VN-ENV-IND-1894 và VN-EV-2030.</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7028,17 +7028,17 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] ENVIRONMENTAL IMPACT OF INDUSTRIALIZATION — This report examines the environmental impact of industrialization in Vietnam, highlighting air and water pollution, solid waste issues, and the challenges ... (관련: VN-ENV-IND-1894)</t>
+          <t>베트남은 급격한 산업화로 인해 경제 성장을 이루었으나 공기, 수질 및 토양 자원에 심각한 부담을 주고 있습니다. 하노이와 호치민시의 미세먼지 오염이 심각하며, 산업 단지 인근의 폐수 무단 방류로 인해 '죽은 강'이 늘어나고 있습니다.</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] ENVIRONMENTAL IMPACT OF INDUSTRIALIZATION — This report examines the environmental impact of industrialization in Vietnam, highlighting air and water pollution, solid waste issues, and the challenges ... (Related: VN-ENV-IND-1894)</t>
+          <t>Vietnam's rapid industrialization has driven economic growth but caused severe strain on air, water, and soil resources. Major cities face critical PM2.5 pollution from industrial zones and transport, while untreated wastewater from textile and electronic sectors is creating "dead rivers" and contaminating groundwater.</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] ENVIRONMENTAL IMPACT OF INDUSTRIALIZATION — This report examines the environmental impact of industrialization in Vietnam, highlighting air and water pollution, solid waste issues, and the challenges ... (Liên quan: VN-ENV-IND-1894)</t>
+          <t>Quá trình công nghiệp hóa nhanh chóng của Việt Nam đã thúc đẩy kinh tế nhưng gây áp lực lớn lên tài nguyên không khí, nước và đất. Các thành phố lớn đang đối mặt với ô nhiễm bụi mịn nghiêm trọng, trong khi nước thải chưa qua xử lý từ các khu công nghiệp đang tạo ra những "dòng sông chết" và đe dọa nguồn nước ngầm.</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7092,17 +7092,17 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's green horizon: A 2025-2030 plan for ... — Air pollution control equipment is projected to cover 60%-70% of domestic needs, while solid and hazardous waste treatment technologies are to ... (관련: VN-ENV-IND-1894)</t>
+          <t>베트남은 2025년까지 산림 피복률을 42.03%로 유지하고 1,300만 달러 규모의 오존층 파괴 물질 감축 프로젝트를 시작했습니다. 하노이와 호치민시는 2027년부터 이륜차 배기가스 검사를 시행하며, 2030년까지 전국으로 확대할 계획입니다.</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's green horizon: A 2025-2030 plan for ... — Air pollution control equipment is projected to cover 60%-70% of domestic needs, while solid and hazardous waste treatment technologies are to ... (Related: VN-ENV-IND-1894)</t>
+          <t>Vietnam has maintained a stable forest coverage of 42.03% as of 2025 and launched a 13 million USD project to phase out ozone-depleting substances by 2031. Additionally, the country will implement mandatory motorcycle emissions testing in major cities starting in 2027, expanding nationwide by 2030.</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's green horizon: A 2025-2030 plan for ... — Air pollution control equipment is projected to cover 60%-70% of domestic needs, while solid and hazardous waste treatment technologies are to ... (Liên quan: VN-ENV-IND-1894)</t>
+          <t>Việt Nam duy trì tỷ lệ che phủ rừng ổn định ở mức 42,03% vào năm 2025 và triển khai dự án 13 triệu USD nhằm loại bỏ các chất làm suy giảm tầng ozone. Bên cạnh đó, lộ trình kiểm định khí thải xe máy sẽ bắt đầu tại Hà Nội và TP.HCM từ năm 2027, sau đó mở rộng ra toàn quốc vào năm 2030.</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7152,17 +7152,17 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Current status of industrial waste management in Vietnam — Especially, industrial zones that have not yet built and operated wastewater treatment stations cause even greater environmental pollution, such as Cau Ngan ... (관련: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>베트남 산업단지의 약 79%가 중앙 집중식 폐수 처리 시스템을 갖추고 있으나, 많은 곳이 비효율적으로 운영되거나 환경 기준을 충족하지 못하고 있습니다. 산업 클러스터(CCN)의 경우 단 5%만이 처리 시설을 보유하고 있으며, 고형 및 유해 폐기물 수집 시설의 부족이 심각한 환경 오염의 원인이 되고 있습니다.</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Current status of industrial waste management in Vietnam — Especially, industrial zones that have not yet built and operated wastewater treatment stations cause even greater environmental pollution, such as Cau Ngan ... (Related: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>Approximately 79% of Vietnam's operating industrial zones have built centralized wastewater treatment systems, yet many face operational inefficiencies and fail to meet national environmental standards. Industrial clusters (CCNs) lag significantly with only a 5% coverage rate, and the lack of dedicated collection and treatment centers for hazardous solid waste continues to pressure natural ecosystems.</t>
         </is>
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Current status of industrial waste management in Vietnam — Especially, industrial zones that have not yet built and operated wastewater treatment stations cause even greater environmental pollution, such as Cau Ngan ... (Liên quan: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>Khoảng 79% các khu công nghiệp tại Việt Nam đã xây dựng hệ thống xử lý nước thải tập trung, nhưng nhiều nơi vận hành chưa hiệu quả và chưa đạt quy chuẩn môi trường. Các cụm công nghiệp (CCN) chỉ có khoảng 5% có hệ thống xử lý, đồng thời việc thiếu hụt các trung tâm thu gom và xử lý chất thải rắn nguy hại đang gây áp lực lớn lên hệ sinh thái và sức khỏe con người.</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7212,17 +7212,17 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam To Set Up Industrial Environmental Index — Vietnam has developed industrial zones ... zones would significantly resolve environmental issues, reduce waste, and achieve sustainable development. (관련: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>베트남 기획투자부는 지속 가능한 산업 발전을 촉진하기 위해 산업 환경 지수를 도입할 계획이라고 발표했습니다. 이 지수는 2021-2030 녹색 성장 전략의 일환으로, 400개 이상의 산업 단지와 18개 경제 구역의 환경 오염 문제를 해결하고 2050년 탄소 중립 목표 달성을 돕는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam To Set Up Industrial Environmental Index — Vietnam has developed industrial zones ... zones would significantly resolve environmental issues, reduce waste, and achieve sustainable development. (Related: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>The Vietnamese Ministry of Planning has announced plans to implement an Industrial Environmental Index to promote sustainable industrial development across its 400+ industrial parks. This initiative is part of the country's 2021-2030 green growth strategy and aims to mitigate severe industrial pollution while aligning with the national goal of reaching net-zero emissions by 2050.</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam To Set Up Industrial Environmental Index — Vietnam has developed industrial zones ... zones would significantly resolve environmental issues, reduce waste, and achieve sustainable development. (Liên quan: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>Bộ Kế hoạch và Đầu tư Việt Nam vừa công bố kế hoạch triển khai bộ chỉ số môi trường công nghiệp nhằm thúc đẩy phát triển công nghiệp bền vững. Đây là một phần trong chiến lược tăng trưởng xanh giai đoạn 2021-2030, hướng tới mục tiêu giải quyết vấn đề ô nhiễm tại các khu công nghiệp và đạt phát thải ròng bằng 0 vào năm 2050.</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7276,17 +7276,17 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam's push for net zero emissions by 2050 is putting ... — Việt Nam's push for net zero emissions by 2050 is putting pressure on industrial parks, where gaps in real-time monitoring and fragmented ...</t>
+          <t>베트남의 2050년 넷제로 목표 달성을 위해 산업단지 내 탄소 배출 모니터링 및 보고 체계 개선이 시급한 과제로 떠오르고 있습니다. 이에 기업들은 환경 표준을 준수하고 효율성을 높이기 위해 지능형 운영 센터(IOC)를 도입하며 단순 인프라 임대를 넘어 글로벌 가치 사슬 내 거버넌스 플랫폼으로 진화하고 있습니다.</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam's push for net zero emissions by 2050 is putting ... — Việt Nam's push for net zero emissions by 2050 is putting pressure on industrial parks, where gaps in real-time monitoring and fragmented ...</t>
+          <t>Vietnam's 2050 net-zero commitment is driving industrial parks to adopt Intelligent Operations Centers (IOCs) to address gaps in real-time environmental monitoring. These digital platforms help businesses meet international sustainability standards and transition from basic infrastructure providers to key players in global value chains.</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Việt Nam's push for net zero emissions by 2050 is putting ... — Việt Nam's push for net zero emissions by 2050 is putting pressure on industrial parks, where gaps in real-time monitoring and fragmented ...</t>
+          <t>Mục tiêu phát thải ròng bằng 0 vào năm 2050 của Việt Nam đang gây áp lực lên các khu công nghiệp trong việc cải thiện hệ thống giám sát và báo cáo môi trường. Để đáp ứng các tiêu chuẩn xanh, nhiều doanh nghiệp đã triển khai Trung tâm điều hành thông minh (IOC) nhằm nâng cao hiệu quả quản trị và vị thế trong chuỗi giá trị toàn cầu.</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7340,17 +7340,17 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Green Transition in Vietnam's Industrial Parks: Policy ... — Vietnam's industrial parks are shifting toward eco-industrial models, renewable energy, and green standards amid global supply chain ...</t>
+          <t>베트남은 탄소 국경 조정 제도(CBAM)와 같은 글로벌 ESG 규제에 대응하기 위해 산업단지를 친환경 생태산업단지(EIP)로 전환하는 정책을 추진하고 있습니다. 정부는 신재생 에너지 사용과 자원 효율성을 강조하는 시행령 제35호 및 제9716호를 통해 법적 프레임워크를 마련하고 국제 기구와 협력하여 이를 확대하고 있습니다.</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Green Transition in Vietnam's Industrial Parks: Policy ... — Vietnam's industrial parks are shifting toward eco-industrial models, renewable energy, and green standards amid global supply chain ...</t>
+          <t>Vietnam is transitioning its industrial parks into Eco-Industrial Parks (EIPs) to align with global ESG standards and regulations like the EU's CBAM. Supported by Decree 35 and Decree 9716, the government is promoting renewable energy adoption and circular economy practices to maintain export competitiveness and achieve net-zero goals by 2050.</t>
         </is>
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Green Transition in Vietnam's Industrial Parks: Policy ... — Vietnam's industrial parks are shifting toward eco-industrial models, renewable energy, and green standards amid global supply chain ...</t>
+          <t>Việt Nam đang chuyển đổi các khu công nghiệp truyền thống sang mô hình khu công nghiệp sinh thái (EIP) nhằm đáp ứng các tiêu chuẩn ESG quốc tế và quy định CBAM. Chính phủ đã ban hành Nghị định 35 và Nghị định 9716 để thúc đẩy sử dụng năng lượng tái tạo, kinh tế tuần hoàn và nâng cao năng lực cạnh tranh cho chuỗi cung ứng toàn cầu.</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7404,17 +7404,17 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Solid Waste Treatment in Vietnam: Current Situation and ... — Vietnam's industrial sector produces significant amounts of waste, but the country currently lacks sufficient treatment facilities. Foreign ...</t>
+          <t>베트남은 현재 하루 약 6만 톤의 생활 폐기물을 발생시키며, 그중 71%를 매립에 의존하고 있어 환경 오염 문제에 직면해 있습니다. 정부는 2030년까지 폐기물 에너지화(WtE) 용량을 1,500MW까지 확대하고 2024년 말부터 분리배출을 의무화하는 등 현대적인 폐기물 관리 인프라 구축에 박차를 가하고 있습니다.</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Solid Waste Treatment in Vietnam: Current Situation and ... — Vietnam's industrial sector produces significant amounts of waste, but the country currently lacks sufficient treatment facilities. Foreign ...</t>
+          <t>Vietnam generates approximately 60,000 tons of municipal solid waste daily, with 71% still being landfilled, leading to significant environmental challenges. The government is actively promoting the transition to waste-to-energy (WtE) technology with a target of 1,500 MW capacity by 2030, offering substantial opportunities for foreign investment in sustainable infrastructure.</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Solid Waste Treatment in Vietnam: Current Situation and ... — Vietnam's industrial sector produces significant amounts of waste, but the country currently lacks sufficient treatment facilities. Foreign ...</t>
+          <t>Việt Nam hiện phát sinh khoảng 60.000 tấn rác thải sinh hoạt mỗi ngày, trong đó 71% vẫn được xử lý bằng phương pháp chôn lấp gây ô nhiễm môi trường. Chính phủ đang thúc đẩy hạ tầng xử lý rác hiện đại với mục tiêu đạt 1.500 MW điện rác vào năm 2030 và bắt buộc phân loại rác tại nguồn từ cuối năm 2024.</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7468,17 +7468,17 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam accelerates battle against plastic waste — Vietnam is mobilizing resources to fight plastic waste marking its fifth anniversary.</t>
+          <t>베트남은 2030년까지 플라스틱 폐기물을 대폭 감축하기 위해 국가 플라스틱 행동 파트너십(NPAP)과 순환 경제 모델을 가속화하고 있습니다. 정부는 환경 보호와 지속 가능한 발전을 목표로 '그린 베트남'을 구축하기 위한 다양한 정책을 추진 중입니다.</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam accelerates battle against plastic waste — Vietnam is mobilizing resources to fight plastic waste marking its fifth anniversary.</t>
+          <t>Vietnam is accelerating its efforts to combat plastic waste by implementing a circular economy and the National Plastic Action Partnership (NPAP). The country aims to achieve significant plastic reduction targets by 2030 to ensure environmental protection and a greener future.</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam accelerates battle against plastic waste — Vietnam is mobilizing resources to fight plastic waste marking its fifth anniversary.</t>
+          <t>Việt Nam đang đẩy nhanh cuộc chiến chống rác thải nhựa thông qua việc thúc đẩy kinh tế tuần hoàn và Chương trình Đối tác Hành động Quốc gia về Nhựa (NPAP). Mục tiêu của kế hoạch là giảm thiểu đáng kể rác thải nhựa vào năm 2030 để hướng tới một Việt Nam xanh và bảo vệ môi trường.</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7532,17 +7532,17 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's infrastructure push to boost growth and deficit, S&amp;P ... — Vietnam is forecast to remain Asia's fastest-growing nation after India through 2028, supported by exports and infrastructure investments, ...</t>
+          <t>베트남은 수출과 대규모 인프라 투자를 바탕으로 2028년까지 인도에 이어 아시아에서 가장 빠르게 성장하는 국가가 될 것으로 전망됩니다. 정부는 2030년까지 연간 10% 성장을 목표로 약 2,000억 달러 규모의 프로젝트를 추진 중이지만, 이로 인한 재정 적자 확대 및 공공 부채 증가가 등급 상향의 변수가 될 수 있습니다.</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's infrastructure push to boost growth and deficit, S&amp;P ... — Vietnam is forecast to remain Asia's fastest-growing nation after India through 2028, supported by exports and infrastructure investments, ...</t>
+          <t>Vietnam is projected to be Asia's fastest-growing economy after India through 2028, driven by massive infrastructure investments worth $200 billion. While these projects support strong economic growth targets, S&amp;P Ratings warns that heavy public spending could lead to larger fiscal deficits and rising government debt.</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam's infrastructure push to boost growth and deficit, S&amp;P ... — Vietnam is forecast to remain Asia's fastest-growing nation after India through 2028, supported by exports and infrastructure investments, ...</t>
+          <t>Việt Nam được dự báo sẽ là nền kinh tế tăng trưởng nhanh nhất châu Á sau Ấn Độ cho đến năm 2028 nhờ vào xuất khẩu và các khoản đầu tư hạ tầng trị giá 200 tỷ USD. Tuy nhiên, S&amp;P Ratings cảnh báo rằng việc đẩy mạnh chi tiêu công có thể dẫn đến thâm hụt ngân sách lớn hơn và nợ công gia tăng, ảnh hưởng đến mục tiêu nâng hạng tín nhiệm.</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7596,17 +7596,17 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam Construction Industry Report 2026: Output to Expand by 7.9 ... — The analyst expects the construction industry in Vietnam to grow by 7.9% in real terms in 2026, supported by increased foreign direct investment ...</t>
+          <t>베트남 건설 산업은 정부의 인프라 투자 확대에 힘입어 2030년까지 연평균 6.5%의 성장이 예상됩니다. 특히 교통부는 고속도로 길이를 5,000km까지 확장하고 호치민시에 8개의 지하철 노선을 건설하는 대규모 프로젝트를 추진 중입니다.</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam Construction Industry Report 2026: Output to Expand by 7.9 ... — The analyst expects the construction industry in Vietnam to grow by 7.9% in real terms in 2026, supported by increased foreign direct investment ...</t>
+          <t>Vietnam's construction sector is projected to maintain a 6.5% average annual growth rate through 2030, driven by significant transport and energy infrastructure investments. Key projects include expanding the national expressway network to 5,000km and developing an eight-line urban railway system in Ho Chi Minh City by 2035.</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Vietnam Construction Industry Report 2026: Output to Expand by 7.9 ... — The analyst expects the construction industry in Vietnam to grow by 7.9% in real terms in 2026, supported by increased foreign direct investment ...</t>
+          <t>Ngành xây dựng Việt Nam dự kiến đạt mức tăng trưởng bình quân 6,5% mỗi năm từ 2027 đến 2030 nhờ sự đẩy mạnh đầu tư vào hạ tầng giao thông và năng lượng. Các dự án trọng điểm bao gồm mục tiêu nâng chiều dài đường cao tốc lên 5.000km và xây dựng hệ thống 8 tuyến đường sắt đô thị tại TP.HCM.</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7660,17 +7660,17 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>[Other] Vietnam Infrastructure Spotlight March 2026 - Freshfields — In this issue, we highlight recent legal and market developments in Vietnam's infrastructure sector. (관련: VN-EV-2030)</t>
+          <t>하노이시는 2030년까지 모든 가솔린 및 디젤 택시를 친환경 차량으로 교체할 계획이며, 2026년까지 63-64% 전환을 목표로 하고 있습니다. 이와 함께 Thaco는 VinFast에 이어 베트남의 두 번째 독자 자동차 브랜드를 출시하여 국내 전기차 및 승용차 시장을 확대할 예정입니다.</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>[Other] Vietnam Infrastructure Spotlight March 2026 - Freshfields — In this issue, we highlight recent legal and market developments in Vietnam's infrastructure sector. (Related: VN-EV-2030)</t>
+          <t>Hanoi plans to replace all gasoline and diesel taxis with green-energy vehicles by 2030, targeting a 63-64% transition rate by 2026. Additionally, Vietnamese conglomerate Thaco aims to launch its own passenger car brand, becoming the country's second domestic automaker after VinFast.</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>[Other] Vietnam Infrastructure Spotlight March 2026 - Freshfields — In this issue, we highlight recent legal and market developments in Vietnam's infrastructure sector. (Liên quan: VN-EV-2030)</t>
+          <t>Hà Nội lập kế hoạch thay thế toàn bộ xe taxi chạy bằng xăng và dầu bằng xe năng lượng xanh vào năm 2030, với mục tiêu đạt tỷ lệ 63-64% vào năm 2026. Bên cạnh đó, tập đoàn Thaco dự kiến sản xuất xe du lịch mang thương hiệu riêng, trở thành thương hiệu ô tô nội địa thứ hai của Việt Nam sau VinFast.</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -7724,17 +7724,17 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's Infrastructure Breakthrough: A Strategic Pillar for Growth — ... Vietnam but also a key reference point for the international business community. It is shaping expectations for economic reform, investment ...</t>
+          <t>베트남은 제14차 당대회를 앞두고 인프라 혁신을 국가 성장의 핵심 전략적 기둥으로 설정했습니다. 이는 국제 비즈니스 사회에 중요한 지표가 되며 투자 유치를 위한 기반이 될 것입니다.</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's Infrastructure Breakthrough: A Strategic Pillar for Growth — ... Vietnam but also a key reference point for the international business community. It is shaping expectations for economic reform, investment ...</t>
+          <t>Vietnam is positioning its infrastructure breakthrough as a strategic pillar for economic growth ahead of the 14th National Party Congress. This development serves as a critical reference point for the international business community and future investment.</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's Infrastructure Breakthrough: A Strategic Pillar for Growth — ... Vietnam but also a key reference point for the international business community. It is shaping expectations for economic reform, investment ...</t>
+          <t>Việt Nam đang xác định đột phá hạ tầng là trụ cột chiến lược cho sự tăng trưởng hướng tới Đại hội Đảng toàn quốc lần thứ 14. Đây là điểm tham chiếu quan trọng cho cộng đồng kinh doanh quốc tế và thu hút đầu tư.</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -7788,17 +7788,17 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Investing In... 2026 - Vietnam - Global Practice Guides — These landmark reforms round out Vietnam's earlier investment roadmap under Resolution No 50 (2019) and are reinforced by a series of new ...</t>
+          <t>베트남은 2024년 개정 전기법과 제8차 국가전력개발계획(PDP VIII)을 통해 에너지 인프라 시장을 대대적으로 개편하고 신재생 에너지 투자를 촉진하고 있습니다. 행정적으로는 교통부가 건설부로 통합되는 등 정부 부처 구조조정을 통해 인프라 프로젝트의 효율성을 높이고자 합니다.</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Investing In... 2026 - Vietnam - Global Practice Guides — These landmark reforms round out Vietnam's earlier investment roadmap under Resolution No 50 (2019) and are reinforced by a series of new ...</t>
+          <t>Vietnam is overhauling its infrastructure sector through the 2024 Law on Electricity and the amended PDP VIII, which prioritizes renewable energy and introduces new market instruments. Administratively, the country has merged the Ministry of Transport into the Ministry of Construction to streamline project management and enhance administrative efficiency.</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Investing In... 2026 - Vietnam - Global Practice Guides — These landmark reforms round out Vietnam's earlier investment roadmap under Resolution No 50 (2019) and are reinforced by a series of new ...</t>
+          <t>Việt Nam đang thúc đẩy hạ tầng năng lượng thông qua Luật Điện lực 2024 và Quy hoạch điện VIII điều chỉnh, ưu tiên năng lượng tái tạo và cơ chế mua bán điện trực tiếp. Về mặt hành chính, Bộ Giao thông Vận tải đã được sáp nhập vào Bộ Xây dựng nhằm tối ưu hóa việc quản lý và thực hiện các dự án hạ tầng chiến lược.</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7852,17 +7852,17 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>[Other] The economy: Re-balancing in 2026 - Theinvestor — Vietnam's infrastructure spending growth is expected to accelerate from circa 10% annually over the last decade to 20-30% per year going ...</t>
+          <t>베트남의 인프라 지출 성장률은 향후 연간 20-30%로 가속화될 전망이며, 정부는 인프라 투자를 GDP의 10% 수준까지 확대하는 것을 목표로 하고 있습니다. 이러한 인프라 확충은 부동산 시장 활성화와 소비 진작으로 이어져 2026년 베트남 경제 성장의 핵심 동력이 될 것으로 기대됩니다.</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>[Other] The economy: Re-balancing in 2026 - Theinvestor — Vietnam's infrastructure spending growth is expected to accelerate from circa 10% annually over the last decade to 20-30% per year going ...</t>
+          <t>Vietnam's infrastructure spending is projected to surge by 20-30% annually, as the government aims to increase its share from 6% to 10% of GDP. This aggressive infrastructure push is expected to create a growth nexus with the real estate sector and domestic consumption, significantly supporting the country's GDP in 2026.</t>
         </is>
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>[Other] The economy: Re-balancing in 2026 - Theinvestor — Vietnam's infrastructure spending growth is expected to accelerate from circa 10% annually over the last decade to 20-30% per year going ...</t>
+          <t>Tăng trưởng chi tiêu hạ tầng của Việt Nam dự kiến sẽ tăng tốc lên mức 20-30% mỗi năm, với mục tiêu nâng tỷ trọng từ 6% lên 10% GDP. Sự thúc đẩy hạ tầng này sẽ tạo ra mối liên kết chặt chẽ với thị trường bất động sản và tiêu dùng nội địa, đóng vai trò là đòn bẩy quan trọng cho tăng trưởng kinh tế năm 2026.</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7916,17 +7916,17 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's Infrastructure Breakthrough: A Strategic Pillar for Growth — It is shaping expectations for economic reform, investment flows, and long-term development priorities, which are already taking shape through ... (관련: VN-EV-2030)</t>
+          <t>베트남은 제14차 당대회를 앞두고 주요 인프라, 교통 및 산업 프로젝트를 통해 경제 개혁과 투자 유치를 가속화하고 있습니다. 정부의 공공 투자 확대와 녹색 전환 정책에 힘입어 2026년 GDP 성장률은 7.2%에 달할 것으로 전망됩니다.</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's Infrastructure Breakthrough: A Strategic Pillar for Growth — It is shaping expectations for economic reform, investment flows, and long-term development priorities, which are already taking shape through ... (Related: VN-EV-2030)</t>
+          <t>Vietnam is leveraging major infrastructure and industrial projects to drive economic growth and attract strategic investment flows ahead of the 14th National Party Congress. Supported by accelerated public investment and a green transition, the economy is projected to reach a GDP growth of 7.2% in 2026.</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] Vietnam's Infrastructure Breakthrough: A Strategic Pillar for Growth — It is shaping expectations for economic reform, investment flows, and long-term development priorities, which are already taking shape through ... (Liên quan: VN-EV-2030)</t>
+          <t>Việt Nam đang đẩy mạnh các dự án hạ tầng, giao thông và công nghiệp trọng điểm nhằm thúc đẩy tăng trưởng và thu hút dòng vốn đầu tư trước thềm Đại hội Đảng lần thứ XIV. Với sự hỗ trợ từ đầu tư công và chuyển đổi xanh, nền kinh tế dự kiến đạt mức tăng trưởng GDP 7,2% vào năm 2026.</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -7980,17 +7980,17 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Tapping into Vietnam's High-Value Growth Ambition in 2026 — Vietnam is aiming for a high-value growth, supported by policies that promote productivity, innovation, and industrial upgrading.</t>
+          <t>베트남은 2026년까지 남북 고속철도 건설 가속화, 국제 철도망 강화, 하노이 및 호치민시 도시철도 확장을 포함한 대규모 인프라 현대화를 추진합니다. 또한 닌투안 원전 프로젝트 재개와 5G·6G 네트워크 구축을 통해 에너지 안보와 디지털 전환을 가속화할 계획입니다.</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Tapping into Vietnam's High-Value Growth Ambition in 2026 — Vietnam is aiming for a high-value growth, supported by policies that promote productivity, innovation, and industrial upgrading.</t>
+          <t>Vietnam is accelerating its infrastructure development by 2026, focusing on the North-South high-speed railway, international rail links, and urban rail expansions in Hanoi and Ho Chi Minh City. The plan also includes reviving nuclear power projects and deploying 5G and 6G networks to support high-value economic growth.</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>[Transport &amp; Infrastructure] Tapping into Vietnam's High-Value Growth Ambition in 2026 — Vietnam is aiming for a high-value growth, supported by policies that promote productivity, innovation, and industrial upgrading.</t>
+          <t>Việt Nam đang đẩy mạnh phát triển hạ tầng đến năm 2026, tập trung vào đường sắt tốc độ cao Bắc-Nam, kết nối đường sắt quốc tế và mở rộng đường sắt đô thị tại Hà Nội và TP.HCM. Kế hoạch này cũng bao gồm việc khởi động lại các dự án điện hạt nhân và triển khai mạng 5G, 6G để hỗ trợ tăng trưởng kinh tế giá trị cao.</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8044,17 +8044,17 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>[Other] Invest in Vietnam Infrastructure as a Long-Term Growth Driver — To invest in Vietnam infrastructure is to participate in a structural transformation that extends well beyond short-term economic cycles.</t>
+          <t>베트남의 인프라 개발은 도로, 항만, 에너지망 확충을 통해 장기적인 경제 성장을 견인하는 핵심 동력입니다. 이러한 투자는 건설, 물류, 금융 서비스 전반에 걸쳐 안정적인 수익원과 다변화된 투자 기회를 제공합니다.</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>[Other] Invest in Vietnam Infrastructure as a Long-Term Growth Driver — To invest in Vietnam infrastructure is to participate in a structural transformation that extends well beyond short-term economic cycles.</t>
+          <t>Infrastructure development serves as a vital pillar for Vietnam's long-term economic expansion, focusing on transportation, energy, and digital networks. These large-scale projects offer investors stable, non-cyclical revenue streams through public-private partnerships and government-led initiatives.</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>[Other] Invest in Vietnam Infrastructure as a Long-Term Growth Driver — To invest in Vietnam infrastructure is to participate in a structural transformation that extends well beyond short-term economic cycles.</t>
+          <t>Phát triển cơ sở hạ tầng là trụ cột quan trọng cho tăng trưởng kinh tế dài hạn của Việt Nam, tập trung vào mạng lưới giao thông, năng lượng và kỹ thuật số. Việc đầu tư vào lĩnh vực này mang lại cơ hội tiếp cận các nguồn thu nhập ổn định và ít biến động thông qua các dự án trọng điểm của chính phủ.</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8108,17 +8108,17 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] MoIT to ensure power supply security for 2026 — The Ministry of Industry and Trade has reaffirmed that Vietnam's power supply in 2026 will be fully secured.</t>
+          <t>베트남 산업통상부(MoIT)는 2026년 전력 공급 안보를 보장하기 위해 8.5~14.1%의 수요 성장을 반영한 전력 공급 계획을 승인했습니다. 1,200MW 규모의 붕앙 2 화력발전소가 상업 운전을 시작했으며, PV GAS의 재기화 용량 확대와 500kV 마이쩌우 변전소 업그레이드를 통해 전력망 안정성을 강화하고 있습니다.</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] MoIT to ensure power supply security for 2026 — The Ministry of Industry and Trade has reaffirmed that Vietnam's power supply in 2026 will be fully secured.</t>
+          <t>Vietnam's Ministry of Industry and Trade has approved the 2026 national power supply plan to address load growth scenarios of up to 14.1% during extreme dry seasons. Key developments include the 1,200 MW Vung Ang 2 thermal power plant entering operation, doubled regasification capacity by PV GAS, and grid upgrades at the Mai Chau substation to prevent shortages in the North.</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] MoIT to ensure power supply security for 2026 — The Ministry of Industry and Trade has reaffirmed that Vietnam's power supply in 2026 will be fully secured.</t>
+          <t>Bộ Công Thương đã phê duyệt kế hoạch cung ứng điện năm 2026 dựa trên kịch bản tăng trưởng phụ tải từ 8,5% đến 14,1% trong mùa khô khắc nghiệt. Các giải pháp chính bao gồm việc đưa nhà máy nhiệt điện Vũng Áng 2 (1.200 MW) vào vận hành, gấp đôi công suất tái hóa khí của PV GAS và nâng cấp trạm biến áp 500kV Mai Châu để đảm bảo an ninh năng lượng miền Bắc.</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8172,17 +8172,17 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-Russia energy cooperation: a strategic pillar in global ... — Coal imports reached nearly $1 billion in 2024, meeting around 10 per cent of Vietnam's demand, while fertilisers accounted for $228 million.</t>
+          <t>베트남-러시아 경제 포럼 2026에서 양국은 에너지 협력을 전략적 핵심 축으로 재확인하며, 혁신과 과학 기술 중심의 새로운 모델로의 전환을 강조했습니다. 석탄 및 석유 등 전통적 자원 공급 외에도 민간 원자력, 수소 에너지, 탄소 포집 및 저장 기술 등 신에너지 분야에서의 협력을 확대할 계획입니다.</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-Russia energy cooperation: a strategic pillar in global ... — Coal imports reached nearly $1 billion in 2024, meeting around 10 per cent of Vietnam's demand, while fertilisers accounted for $228 million.</t>
+          <t>At the Vietnam-Russia Economic Forum 2026, energy was highlighted as a strategic pillar for bilateral relations, moving toward a model driven by innovation and science. Beyond traditional oil and coal trade, the cooperation is expanding into civil nuclear energy, power system stability, hydrogen, and carbon capture to support Vietnam's 2050 net-zero goals.</t>
         </is>
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-Russia energy cooperation: a strategic pillar in global ... — Coal imports reached nearly $1 billion in 2024, meeting around 10 per cent of Vietnam's demand, while fertilisers accounted for $228 million.</t>
+          <t>Tại Diễn đàn Kinh tế Việt Nam - Nga 2026, hợp tác năng lượng được xác định là trụ cột chiến lược, chuyển dịch từ mô hình truyền thống sang mô hình thúc đẩy bởi đổi mới sáng tạo và khoa học công nghệ. Hai bên định hướng mở rộng hợp tác sang các lĩnh vực mới như điện hạt nhân dân sự, năng lượng hydro và thu giữ carbon nhằm hỗ trợ mục tiêu phát thải ròng bằng 0 vào năm 2050.</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8236,17 +8236,17 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Forum outlines pathways to accelerate green transition — Vietnam's energy transition is entering a decisive phase, where ambition is rapidly giving way to the harder realities of execution, bankability ...</t>
+          <t>베트남-호주 포럼에서는 베트남의 넷제로 목표 달성을 위해 3,680억 달러 규모의 기후 행동 자금이 필요하다고 강조하며 전력 시장 규제 완화를 촉구했습니다. 전문가들은 루프탑 태양광에 민간 자본이 유입될 수 있도록 시장을 개방하고 펌프식 수력 발전소 등을 활용한 에너지 저장 장치를 확충해야 한다고 제안했습니다.</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Forum outlines pathways to accelerate green transition — Vietnam's energy transition is entering a decisive phase, where ambition is rapidly giving way to the harder realities of execution, bankability ...</t>
+          <t>The Vietnam-Australia forum highlighted that Vietnam requires approximately $368 billion for climate action to meet its net-zero goals, emphasizing the need for market deregulation in the energy sector. Experts called for unleashing private capital into rooftop solar and utilizing the country's vast potential for pumped hydro sites to stabilize the green transition.</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Forum outlines pathways to accelerate green transition — Vietnam's energy transition is entering a decisive phase, where ambition is rapidly giving way to the harder realities of execution, bankability ...</t>
+          <t>Diễn đàn Việt Nam - Australia nhấn mạnh rằng Việt Nam cần khoảng 368 tỷ USD cho hành động khí hậu để đạt cam kết phát thải ròng bằng không và cần bãi bỏ quy định thị trường điện. Các chuyên gia đề xuất khơi thông vốn tư nhân vào điện mặt trời mái nhà và khai thác tiềm năng thủy điện tích năng để đẩy nhanh quá trình chuyển đổi năng lượng.</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8300,17 +8300,17 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] EVN steps up investment in battery storage to support growing ... — Vietnam Electricity is accelerating the deployment of battery energy storage systems across its power network, as the country seeks to ... (관련: VN-EV-2030)</t>
+          <t>베트남 전력공사(EVN)는 재생 에너지의 급증에 대응하여 전력 시스템의 안정성을 높이기 위해 배터리 에너지 저장 시스템(BESS) 투자를 가속화하고 있습니다. 수정된 국가 전력 개발 계획(PDP8)에 따라 베트남은 2030년까지 10,000~16,300MW의 저장 용량 확보를 목표로 하며, 북부 전력 공사는 2026년 6월까지 305MW 규모의 BESS 프로젝트 완공을 추진 중입니다.</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] EVN steps up investment in battery storage to support growing ... — Vietnam Electricity is accelerating the deployment of battery energy storage systems across its power network, as the country seeks to ... (Related: VN-EV-2030)</t>
+          <t>Vietnam Electricity (EVN) is accelerating investment in Battery Energy Storage Systems (BESS) to maintain grid stability as renewable energy shares grow. Under the revised National Power Development Plan VIII, Vietnam aims for 10,000 MW to 16,300 MW of storage capacity by 2030, with several regional subsidiaries already launching pilot projects scheduled for completion by 2026.</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] EVN steps up investment in battery storage to support growing ... — Vietnam Electricity is accelerating the deployment of battery energy storage systems across its power network, as the country seeks to ... (Liên quan: VN-EV-2030)</t>
+          <t>Tập đoàn Điện lực Việt Nam (EVN) đang đẩy mạnh đầu tư vào hệ thống lưu trữ năng lượng bằng pin (BESS) nhằm đảm bảo ổn định hệ thống trong bối cảnh năng lượng tái tạo phát triển mạnh. Theo Quy hoạch điện VIII điều chỉnh, Việt Nam đặt mục tiêu đạt 10.000 MW đến 16.300 MW công suất lưu trữ vào năm 2030, với các dự án trọng điểm tại miền Bắc dự kiến hoàn thành vào tháng 6/2026.</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8364,17 +8364,17 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Meeting Vietnam's energy moment: GE Vernova CEO — UK unveils toolkit to boost Vietnam green investment flows (March 30, 2026 | 13:45) ... Vinh Long kicks ahead with marine-energy approach (March ...</t>
+          <t>GE Vernova는 베트남의 전력 산업에 크게 투자하며 가스, 풍력, 송전 분야의 제조 시설을 확장하고 있습니다. 회사는 다양한 기술과 현지화, 인력 양성을 통해 베트남의 경제 성장과 탈탄소화를 지원할 계획입니다.</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Meeting Vietnam's energy moment: GE Vernova CEO — UK unveils toolkit to boost Vietnam green investment flows (March 30, 2026 | 13:45) ... Vinh Long kicks ahead with marine-energy approach (March ...</t>
+          <t>GE Vernova is expanding its investment in Vietnam's power sector, establishing factories for gas, wind, and grid technologies. The company aims to help Vietnam meet its economic growth and decarbonization targets through technology, partnership, and workforce initiatives.</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Meeting Vietnam's energy moment: GE Vernova CEO — UK unveils toolkit to boost Vietnam green investment flows (March 30, 2026 | 13:45) ... Vinh Long kicks ahead with marine-energy approach (March ...</t>
+          <t>GE Vernova đang mở rộng đầu tư vào lĩnh vực điện tại Việt Nam với các nhà máy sản xuất về khí, điện gió, và lưới điện. Công ty đặt mục tiêu hỗ trợ Việt Nam phát triển kinh tế và giảm phát thải thông qua đa dạng công nghệ, hợp tác và đào tạo nguồn nhân lực.</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8428,17 +8428,17 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's green push requires further hurdles to clear — Vietnam's energy transition is entering a decisive phase, where ambition is rapidly giving way to the harder realities of execution, ...</t>
+          <t>베트남의 녹색 에너지 전환은 자본과 기술의 가용성에도 불구하고 규제 프레임워크의 미비로 인해 어려움을 겪고 있습니다. 전문가들은 프로젝트 파이낸싱으로의 전환, 배터리 에너지 저장 장치(BESS)의 도입, 그리고 투자 적격성을 높이기 위한 혼합 금융 솔루션의 필요성을 강조했습니다.</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's green push requires further hurdles to clear — Vietnam's energy transition is entering a decisive phase, where ambition is rapidly giving way to the harder realities of execution, ...</t>
+          <t>Vietnam's transition to green energy is currently hindered by a regulatory gap that prevents near-ready projects from becoming fully bankable investments. Industry leaders emphasize the need for innovative financial structures like project finance and "orange bonds," alongside the scaling of battery energy storage systems (BESS) and direct power purchase agreements (DPPAs).</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's green push requires further hurdles to clear — Vietnam's energy transition is entering a decisive phase, where ambition is rapidly giving way to the harder realities of execution, ...</t>
+          <t>Quá trình chuyển đổi năng lượng xanh của Việt Nam đang gặp trở ngại do khung pháp lý chưa hoàn thiện, khiến các dự án tiềm năng khó trở thành khoản đầu tư khả thi về mặt tài chính. Các chuyên gia nhấn mạnh tầm quan trọng của việc cải cách quy định, áp dụng cơ chế mua bán điện trực tiếp (DPPA) và các giải pháp tài chính hỗn hợp để thu hút vốn đầu tư quốc tế.</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8492,17 +8492,17 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Safe operations ensured during energy transition — Vietnam's central region is increasingly emerging as a critical balancing hub within the national power system.</t>
+          <t>베트남 전력공사 제2전력전송공사(PTC2)는 중부 지역의 안정적인 전력 공급을 위해 2026년 1,280만 달러 규모의 14개 프로젝트를 추진하고 있습니다. 다낭 변전소 확장 및 500kV 스위치야드 개선을 포함하여 에너지 전환기 동안의 전력망 안전과 효율성을 높이는 데 주력하고 있습니다.</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Safe operations ensured during energy transition — Vietnam's central region is increasingly emerging as a critical balancing hub within the national power system.</t>
+          <t>Vietnam's Power Transmission Corporation 2 (PTC2) is implementing 14 infrastructure projects in 2026 with a $12.8 million investment to ensure grid stability in the central region. Key initiatives include upgrading the Danang substation, adopting digital transformation tools like drones and LiDAR, and addressing challenges posed by new safety regulations and expressway developments.</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Safe operations ensured during energy transition — Vietnam's central region is increasingly emerging as a critical balancing hub within the national power system.</t>
+          <t>Công ty Truyền tải điện 2 (PTC2) đang triển khai 14 dự án hạ tầng trong năm 2026 với tổng vốn đầu tư 12,8 triệu USD nhằm đảm bảo an ninh năng lượng tại miền Trung. Các hạng mục chính bao gồm nâng cấp trạm biến áp 500kV Đà Nẵng, ứng dụng công nghệ số như flycam và LiDAR để kiểm tra lưới điện, đồng thời chuẩn bị sẵn sàng ứng phó với thiên tai và các quy định an toàn mới.</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -8556,17 +8556,17 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] PM issues directive to ensure power supply in 2026–30, focusing on ... — HÀ NÔI — Prime Minister Phạm Minh Chính has issued a directive urging efforts to ensure adequate electricity supply for production, business ...</t>
+          <t>베트남 팜 민 찐 총리는 2026-30년 기간 동안 연간 12-13% 이상 증가할 것으로 예상되는 전력 수요에 대응하기 위해 무정전 전력 공급을 지시하는 지침 제01/CT-TTg호를 발표했습니다. 정부는 북부 지역의 전력망 확충, LNG 발전소, 해상 풍력 및 닌투언 원자력 발전소 준비 가속화를 통해 에너지 안보를 확보하고 투명한 전력 시장을 구축할 계획입니다.</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] PM issues directive to ensure power supply in 2026–30, focusing on ... — HÀ NÔI — Prime Minister Phạm Minh Chính has issued a directive urging efforts to ensure adequate electricity supply for production, business ...</t>
+          <t>Prime Minister Phạm Minh Chính issued Directive No 01/CT-TTg to guarantee uninterrupted power supply for the 2026-30 period, targeting a 12-13% annual increase in electricity demand. The strategy focuses on accelerating major infrastructure projects such as LNG-fired plants, offshore wind, and the Ninh Thuận nuclear power plant while establishing a competitive and transparent energy market.</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] PM issues directive to ensure power supply in 2026–30, focusing on ... — HÀ NÔI — Prime Minister Phạm Minh Chính has issued a directive urging efforts to ensure adequate electricity supply for production, business ...</t>
+          <t>Thủ tướng Chính phủ Phạm Minh Chính đã ban hành Chỉ thị số 01/CT-TTg nhằm đảm bảo cung ứng điện ổn định cho giai đoạn 2026-30, đáp ứng nhu cầu điện dự kiến tăng từ 12-13% mỗi năm. Các biện pháp then chốt bao gồm đẩy nhanh tiến độ các dự án điện khí LNG, điện gió ngoài khơi, khởi động lại dự án điện hạt nhân Ninh Thuận và phát triển thị trường điện cạnh tranh, minh bạch.</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8620,17 +8620,17 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] FDI surges in Vietnam as Q1 capital climbs 43 per cent on-year — In total, Vietnam's overseas investment (including new and adjusted capital) reached $619.9 million in the first three months of 2026, up 2.6 ...</t>
+          <t>2026년 1분기 베트남의 외국인직접투자(FDI) 유치액은 전년 동기 대비 42.9% 증가한 152억 달러를 기록했습니다. 싱가포르와 한국이 주요 투자국이며, 제조업과 가공업 분야가 전체 투자의 약 70%를 차지하며 성장을 주도했습니다.</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] FDI surges in Vietnam as Q1 capital climbs 43 per cent on-year — In total, Vietnam's overseas investment (including new and adjusted capital) reached $619.9 million in the first three months of 2026, up 2.6 ...</t>
+          <t>Vietnam's foreign direct investment (FDI) saw a significant 42.9% year-on-year increase in Q1 2026, reaching a total registered capital of $15.2 billion. Singapore and South Korea emerged as the top investors, with the manufacturing and processing sector attracting the largest share of capital.</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>[Finance &amp; Investment] FDI surges in Vietnam as Q1 capital climbs 43 per cent on-year — In total, Vietnam's overseas investment (including new and adjusted capital) reached $619.9 million in the first three months of 2026, up 2.6 ...</t>
+          <t>Trong quý 1 năm 2026, tổng vốn đầu tư trực tiếp nước ngoài (FDI) vào Việt Nam đạt 15,2 tỷ USD, tăng 42,9% so với cùng kỳ năm trước. Singapore và Hàn Quốc là những nhà đầu tư lớn nhất, trong khi ngành công nghiệp chế biến, chế tạo tiếp tục dẫn đầu về khả năng thu hút vốn.</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8684,17 +8684,17 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Solar power could save Vietnam $600 million in fossil fuel imports — Solar power may help Vietnam avoid a total $594 million from potential coal and gas imports.</t>
+          <t>베트남은 이란 전쟁으로 인한 화석 연료 가격 급등 속에서 태양광 발전을 통해 약 5억 9,400만 달러의 수입 비용을 절감할 수 있을 것으로 분석됩니다. 2024년 기준 베트남의 재생에너지 발전 비중은 약 13%에 도달하며 아세안 주요 국가들을 앞서고 있습니다.</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Solar power could save Vietnam $600 million in fossil fuel imports — Solar power may help Vietnam avoid a total $594 million from potential coal and gas imports.</t>
+          <t>Solar power is projected to save Vietnam approximately $594 million in coal and gas import costs amid soaring energy prices caused by the conflict in Iran. In 2024, Vietnam's solar and wind generation reached 38.7 TWh, accounting for 13% of its power mix, the highest among the ASEAN-5 nations.</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Solar power could save Vietnam $600 million in fossil fuel imports — Solar power may help Vietnam avoid a total $594 million from potential coal and gas imports.</t>
+          <t>Điện mặt trời có thể giúp Việt Nam tiết kiệm khoảng 594 triệu USD chi phí nhập khẩu than và khí đốt trong bối cảnh giá năng lượng tăng cao do xung đột tại Iran. Tính đến năm 2024, sản lượng điện mặt trời và điện gió của Việt Nam đạt 38,7 TWh, chiếm 13% tổng sản lượng điện, dẫn đầu khu vực ASEAN-5.</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -9199,17 +9199,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] National Power Development Plan VIII (PDP-8) - Vntpa — To develop the power sources and transmission grid at the voltage levels of 220kV or higher, renewable and new energy industries and services in Viet Nam for ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 2030년까지의 국가 전력 개발 계획(PDP8)을 승인하며 에너지 안보 확보와 탈탄소화를 목표로 설정했습니다. 이 계획은 석탄 화력을 단계적으로 폐지하고 해상 풍력 및 태양광과 같은 재생 에너지 비중을 2050년까지 최대 71.5%까지 확대하는 내용을 담고 있습니다.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] National Power Development Plan VIII (PDP-8) - Vntpa — To develop the power sources and transmission grid at the voltage levels of 220kV or higher, renewable and new energy industries and services in Viet Nam for ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has officially approved the National Power Development Plan VIII (PDP8), targeting a transition towards renewable energy and national energy security through 2030. The plan prioritizes the phasing out of coal-fired power by 2050 while significantly expanding wind, solar, and gas-to-hydrogen capacities to meet a 7% annual GDP growth demand.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] National Power Development Plan VIII (PDP-8) - Vntpa — To develop the power sources and transmission grid at the voltage levels of 220kV or higher, renewable and new energy industries and services in Viet Nam for ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Quy hoạch phát triển điện lực quốc gia thời kỳ 2021 - 2030 (Quy hoạch điện VIII) nhằm đảm bảo an ninh năng lượng và chuyển đổi xanh. Kế hoạch tập trung vào việc loại bỏ dần điện than vào năm 2050, đồng thời thúc đẩy mạnh mẽ năng lượng tái tạo và điện khí để phục vụ mục tiêu tăng trưởng kinh tế.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -9259,17 +9259,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eighth National Power Development Plan (PDP VIII) - PwC — PDP VIII presents an ambitious shift for Vietnam's generation mix away from coal, and heavily weighted towards in renewables and new technologies. (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 2030년까지 발전 용량을 150GW로 확대하고 2050년 탄소 중립을 달성하기 위한 제8차 국가전력개발계획(PDP VIII)을 승인했습니다. 이 계획은 석탄 화력 발전에서 재생 에너지, 수소, 암모니아 및 배터리 저장 시스템으로의 대대적인 전환을 목표로 하며, 인프라 구축을 위해 향후 30년간 약 7,000억 달러의 투자가 필요할 것으로 예상됩니다.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eighth National Power Development Plan (PDP VIII) - PwC — PDP VIII presents an ambitious shift for Vietnam's generation mix away from coal, and heavily weighted towards in renewables and new technologies. (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has approved the PDP VIII, an ambitious energy roadmap targeting 150 GW of installed capacity by 2030 and Net Zero emissions by 2050. The plan shifts focus from coal to renewables and emerging technologies like hydrogen and battery storage, requiring approximately $700 billion in investment over the next three decades for generation and grid infrastructure.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eighth National Power Development Plan (PDP VIII) - PwC — PDP VIII presents an ambitious shift for Vietnam's generation mix away from coal, and heavily weighted towards in renewables and new technologies. (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Quy hoạch điện VIII (PDP VIII), đặt mục tiêu nâng công suất lắp đặt lên 150 GW vào năm 2030 và hướng tới phát thải ròng bằng 0 vào năm 2050. Kế hoạch này tập trung chuyển đổi từ điện than sang năng lượng tái tạo, hydro và lưu trữ năng lượng, với nhu cầu vốn đầu tư dự kiến khoảng 700 tỷ USD trong 3 thập kỷ tới cho nguồn điện và lưới điện.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -9323,17 +9323,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eight National Power Development Plan (PDP8) — The PDP8 presents Vietnam's long-term objective to form an energy ecosystem based on renewable energies. The development of wind and solar power ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>2023년 5월 15일 베트남 정부는 '제8차 국가전력개발계획(PDP8)'을 발표하여 2021~2030년과 2050년 비전을 제시했습니다. PDP8은 석탄 발전 용량을 약 13GW 감축하고, 2050년까지 모든 석탄발전소는 대체 연료로 전환하거나 퇴출하도록 요구합니다. 2030년에는 재생에너지가 전체 발전용량의 48%, 2050년에는 약 63%를 차지할 계획입니다.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eight National Power Development Plan (PDP8) — The PDP8 presents Vietnam's long-term objective to form an energy ecosystem based on renewable energies. The development of wind and solar power ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>On May 15, 2023, the Vietnamese government released the 8th National Power Development Plan (PDP8) covering 2021-2030 and a vision to 2050. The plan cancels about 13GW of planned coal capacity, requires all coal plants to be converted to alternative fuels or shut down by 2050, and aims for renewables to provide 48% of installed capacity by 2030 and about 63% by 2050.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Eight National Power Development Plan (PDP8) — The PDP8 presents Vietnam's long-term objective to form an energy ecosystem based on renewable energies. The development of wind and solar power ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Ngày 15/5/2023, Chính phủ Việt Nam đã công bố Quy hoạch Phát triển điện lực quốc gia lần thứ 8 (PDP8) cho giai đoạn 2021-2030, tầm nhìn đến 2050. PDP8 loại bỏ khoảng 13GW điện than, yêu cầu toàn bộ nhà máy điện than phải chuyển đổi sang nhiên liệu thay thế hoặc ngừng hoạt động trước năm 2050 và đặt mục tiêu năng lượng tái tạo chiếm 48% công suất lắp đặt vào năm 2030, và khoảng 63% vào năm 2050.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -9387,17 +9387,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Revised Power Development Plan VIII — Vietnam's April 2025 revision to Power Development Plan VIII accelerates renewable energy targets and reintroduces nuclear power projects. (관련: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam Revised Power Development Plan VIII</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Revised Power Development Plan VIII — Vietnam's April 2025 revision to Power Development Plan VIII accelerates renewable energy targets and reintroduces nuclear power projects. (Related: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam Revised Power Development Plan VIII</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Revised Power Development Plan VIII — Vietnam's April 2025 revision to Power Development Plan VIII accelerates renewable energy targets and reintroduces nuclear power projects. (Liên quan: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam Revised Power Development Plan VIII</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -9447,17 +9447,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Power Development Plan 8 (PDP8) - Speeda ASEAN — Vietnam's Power Development Plan 8 (PDP8) sets bold targets for renewables, but coal reliance, pricing, and grid issues challenge its green energy shift. (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남의 제8차 국가전력개발계획(PDP8)은 2050년 탄소 중립 달성을 목표로 화석 연료에서 재생 에너지 중심의 전력 체계로의 전환을 가속화하고 있습니다. 정부는 옥상 태양광 및 직접전력구매계약(DPPA) 도입을 통해 투자를 촉진하고 있으나, 송전망 미비와 가격 책정 프레임워크의 불확실성은 여전히 해결해야 할 과제로 남아 있습니다.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Power Development Plan 8 (PDP8) - Speeda ASEAN — Vietnam's Power Development Plan 8 (PDP8) sets bold targets for renewables, but coal reliance, pricing, and grid issues challenge its green energy shift. (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam's Power Development Plan 8 (PDP8) drives a strategic shift toward renewable energy to achieve net-zero emissions by 2050. While new policies like Direct Power Purchase Agreements (DPPA) and expanded solar incentives are attracting investment, the transition faces hurdles including grid congestion and unsupportive pricing structures.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's Power Development Plan 8 (PDP8) - Speeda ASEAN — Vietnam's Power Development Plan 8 (PDP8) sets bold targets for renewables, but coal reliance, pricing, and grid issues challenge its green energy shift. (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Quy hoạch điện VIII (PDP8) của Việt Nam định hướng chuyển đổi chiến lược từ năng lượng hóa thạch sang năng lượng tái tạo nhằm mục tiêu phát thải ròng bằng 0 vào năm 2050. Mặc dù các chính sách như cơ chế mua bán điện trực tiếp (DPPA) và ưu đãi điện mặt trời mái nhà đang mở ra cơ hội đầu tư lớn, ngành năng lượng vẫn đối mặt với thách thức về hạ tầng lưới điện và khung giá điện chưa phù hợp.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -9511,17 +9511,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Approves Power Development Plan for Cleaner Fuels — Power Development Plan VIII ("PDP8") calls for expansions to renewable energy generation and development of LNG facilities to aid a gradual ... (관련: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 2030년까지 전력 설비 용량을 150GW로 확충하고 2050년 탄소 중립을 달성하기 위한 제8차 국가 전력개발계획(PDP8)을 승인했습니다. 이 계획은 석탄 화력 발전을 점진적으로 폐지하고 해상 풍력 및 LNG 발전 비중을 대폭 확대하기 위해 약 1,347억 달러의 투자를 필요로 합니다.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Approves Power Development Plan for Cleaner Fuels — Power Development Plan VIII ("PDP8") calls for expansions to renewable energy generation and development of LNG facilities to aid a gradual ... (Related: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has approved the Power Development Plan VIII (PDP8), targeting a grid expansion to 150 GW by 2030 and carbon neutrality by 2050. The plan requires $134.7 billion in investment to shift from coal to cleaner energy sources, specifically prioritizing offshore wind and LNG infrastructure.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam Approves Power Development Plan for Cleaner Fuels — Power Development Plan VIII ("PDP8") calls for expansions to renewable energy generation and development of LNG facilities to aid a gradual ... (Liên quan: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã phê duyệt Quy hoạch điện VIII (PDP8), đặt mục tiêu nâng công suất lưới điện lên 150 GW vào năm 2030 và đạt phát thải ròng bằng 0 vào năm 2050. Kế hoạch này yêu cầu khoản đầu tư 134,7 tỷ USD để chuyển dịch từ điện than sang các nguồn năng lượng sạch hơn như điện gió ngoài khơi và khí LNG.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -9575,17 +9575,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's National Power Development Plan For LNG Power Plants — Under PDP8, Vietnam has no plan to develop NEW LNG power plants after 2035. Potential Backup Locations: Thai Binh, Nam Dinh, Nghi Son, Quynh ... (관련: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부는 PDP8 목표 달성을 위해 LNG 발전소 건설을 가속화하고 있으며, 최근 시행령 제56호(Decree 56)를 통해 연료비 전가 메커니즘과 최소 65%의 전력 구매 보장책을 도입했습니다. 이는 2030년까지 15개의 LNG 발전소를 확보하고 전력 용량을 150,500 MW로 확대하기 위한 조치입니다.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's National Power Development Plan For LNG Power Plants — Under PDP8, Vietnam has no plan to develop NEW LNG power plants after 2035. Potential Backup Locations: Thai Binh, Nam Dinh, Nghi Son, Quynh ... (Related: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>The Vietnamese government has introduced Decree 56 to support the development of 15 LNG power plants under the Amended PDP8, aiming for a total capacity of 150,500 MW by 2030. The new regulations provide a fuel cost pass-through mechanism and a 10-year guarantee for offtaking at least 65% of electricity output to ensure project bankability.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's National Power Development Plan For LNG Power Plants — Under PDP8, Vietnam has no plan to develop NEW LNG power plants after 2035. Potential Backup Locations: Thai Binh, Nam Dinh, Nghi Son, Quynh ... (Liên quan: VN-PWR-PDP8, VN-GAS-PDP8, VN-EV-2030)</t>
+          <t>Chính phủ Việt Nam đã ban hành Nghị định 56 nhằm hỗ trợ phát triển 15 nhà máy điện LNG theo Quy hoạch điện VIII (PDP8) sửa đổi, hướng tới mục tiêu đạt tổng công suất 150.500 MW vào năm 2030. Quy định mới thiết lập cơ chế chuyển tiếp chi phí nhiên liệu và cam kết sản lượng hợp đồng tối thiểu 65% để tháo gỡ khó khăn cho các nhà đầu tư.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -9639,17 +9639,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's latest power development plan focuses on expanding ... — Under the draft PDP 8, Vietnam plans to increase solar capacity to 18.6 GW and wind capacity to 18.0 GW by 2030. Vietnam's underdeveloped grid ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남 정부의 제8차 국가전력개발계획(PDP 8) 초안은 2030년까지 태양광 및 풍력 발전 용량을 대폭 확대하고 탄소 배출을 줄이는 것을 목표로 합니다. 특히 노후화된 전력망 문제를 해결하기 위해 고전압 송전선 건설과 인프라 현대화를 우선순위로 두어 재생에너지 통합을 지원할 계획입니다.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's latest power development plan focuses on expanding ... — Under the draft PDP 8, Vietnam plans to increase solar capacity to 18.6 GW and wind capacity to 18.0 GW by 2030. Vietnam's underdeveloped grid ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam's draft Power Development Plan 8 (PDP 8) aims to significantly increase solar and wind capacity to 18.6 GW and 18.0 GW respectively by 2030 to reduce coal dependency. The plan prioritizes grid modernization, including a 461-mile transmission line project, to address current congestion and successfully integrate higher shares of renewable energy.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam's latest power development plan focuses on expanding ... — Under the draft PDP 8, Vietnam plans to increase solar capacity to 18.6 GW and wind capacity to 18.0 GW by 2030. Vietnam's underdeveloped grid ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Dự thảo Quy hoạch phát triển điện lực quốc gia 8 (PDP 8) của Việt Nam tập trung vào việc mở rộng công suất điện mặt trời và điện gió lên lần lượt 18,6 GW và 18,0 GW vào năm 2030. Kế hoạch này ưu tiên nâng cấp hạ tầng lưới điện và xây dựng các đường dây truyền tải cao thế để khắc phục tình trạng quá tải và hỗ trợ tích hợp năng lượng tái tạo.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -9703,17 +9703,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Foreign investors threaten legal action against Vietnam over ... — Foreign investors may take legal action if Vietnam does not fully pay electricity tariffs agreed with multiple wind and solar projects, ... (관련: VN-PWR-PDP8)</t>
+          <t>베트남 정부가 재생에너지 전력 구매 가격을 소급 삭감하자 한국, EU 등 5개국 상공회의소가 공동 서한을 통해 법적 대응을 예고했습니다. 투자자들은 약속된 보조금이 지급되지 않을 경우 국제 분쟁 해결 절차를 밟을 수 있다고 경고하며 정부의 우호적인 해결책 마련을 촉구했습니다.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Foreign investors threaten legal action against Vietnam over ... — Foreign investors may take legal action if Vietnam does not fully pay electricity tariffs agreed with multiple wind and solar projects, ... (Related: VN-PWR-PDP8)</t>
+          <t>Foreign investors from five major chambers of commerce have threatened legal action against Vietnam due to retroactive cuts in electricity tariffs for wind and solar projects. The dispute involves 12 gigawatts of capacity, with investors warning of potential defaults and multibillion-dollar losses if original payment obligations are not met.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Foreign investors threaten legal action against Vietnam over ... — Foreign investors may take legal action if Vietnam does not fully pay electricity tariffs agreed with multiple wind and solar projects, ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Năm hiệp hội thương mại quốc tế đã cảnh báo sẽ thực hiện các biện pháp pháp lý nếu Chính phủ Việt Nam không thực hiện cam kết về giá mua điện tái tạo. Tranh chấp phát sinh sau khi Việt Nam cắt giảm giá ưu đãi (FIT) đã thỏa thuận trước đó, gây ảnh hưởng đến các dự án có tổng công suất lên tới 12 GW.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -9767,17 +9767,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] An alternative to urban solar energy | Vietnam Today - YouTube — ... 2026, prioritising renewable energy. But while rooftop solar is expanding, many urban residents lack the space or budget for traditional ... (관련: VN-PWR-PDP8)</t>
+          <t>팜 민 찐 총리는 COP26에서 2050년까지 넷제로 달성을 재확인하며 재생 에너지 발전을 최우선 과제로 설정했습니다. 특히 PDP8 계획에 따라 도시형 태양광 에너지의 대안을 모색하며 에너지 인프라 확충에 집중하고 있습니다.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] An alternative to urban solar energy | Vietnam Today - YouTube — ... 2026, prioritising renewable energy. But while rooftop solar is expanding, many urban residents lack the space or budget for traditional ... (Related: VN-PWR-PDP8)</t>
+          <t>Prime Minister Phạm Minh Chính has reaffirmed Vietnam's commitment to achieving net-zero emissions by 2050, prioritizing the development of renewable energy sources. This initiative aligns with the Power Development Plan 8 (PDP8) to explore alternatives for urban solar energy and enhance the national power infrastructure.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] An alternative to urban solar energy | Vietnam Today - YouTube — ... 2026, prioritising renewable energy. But while rooftop solar is expanding, many urban residents lack the space or budget for traditional ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Thủ tướng Phạm Minh Chính khẳng định lại cam kết của Việt Nam về mức phát thải ròng bằng 0 vào năm 2050 tại COP26, ưu tiên phát triển năng lượng tái tạo. Đây là một phần trong kế hoạch Quy hoạch điện VIII (PDP8) nhằm tìm kiếm giải pháp thay thế cho năng lượng mặt trời đô thị và cải thiện hạ tầng năng lượng.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -9831,17 +9831,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Gusty growth: Vietnam's remarkable wind energy story - Eco-Business — The country has made substantial investments in renewable energy, particularly wind power, to meet its growing energy demands and reduce ... (관련: VN-PWR-PDP8)</t>
+          <t>베트남은 2030년까지 풍력 발전 용량을 6,000MW로 확대한다는 야심찬 목표를 세우고 비엔투안 및 쭝남 풍력 발전소와 같은 대규모 프로젝트를 추진하고 있습니다. 정부는 육상 및 해상 풍력에 대한 발전차액지원제도(FiT)와 국제적 파트너십을 통해 투자를 유치하고 있으나, 전력망 인프라 개선이 주요 과제로 남아 있습니다.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Gusty growth: Vietnam's remarkable wind energy story - Eco-Business — The country has made substantial investments in renewable energy, particularly wind power, to meet its growing energy demands and reduce ... (Related: VN-PWR-PDP8)</t>
+          <t>Vietnam is rapidly expanding its wind energy sector with a target of 6,000 MW by 2030, supported by significant projects like the Binh Thuan and Trung Nam plants. The government utilizes Feed-in Tariffs (FiT) and international partnerships to drive growth, though challenges in grid infrastructure and regulatory frameworks persist.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Gusty growth: Vietnam's remarkable wind energy story - Eco-Business — The country has made substantial investments in renewable energy, particularly wind power, to meet its growing energy demands and reduce ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Việt Nam đang nhanh chóng mở rộng lĩnh vực năng lượng gió với mục tiêu đạt công suất 6.000 MW vào năm 2030, được hỗ trợ bởi các dự án lớn như nhà máy Bình Thuận và Trung Nam. Chính phủ áp dụng cơ chế giá bán điện (FiT) và hợp tác quốc tế để thúc đẩy đầu tư, dù vẫn còn những thách thức về hạ tầng lưới điện và khung pháp lý.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -9895,17 +9895,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Bloomberg Businessweek Vietnam 02.2026 Featured Issue ... — Generous FiTs triggered a surge in solar and wind development, transforming the country from a marginal player into a regional clean energy ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남은 과거 보조금 중심의 급격한 성장에서 벗어나 규제 준수와 시장 중심의 규율을 강조하는 에너지 전환의 새로운 단계에 진입했습니다. 직접전력구매계약(DPPA)과 제8차 국가전력개발계획(PDP8)을 통해 공급과 수요의 균형을 맞추고 전력망 안정을 도모하며 장기적인 투자 신뢰도를 구축하고 있습니다.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Bloomberg Businessweek Vietnam 02.2026 Featured Issue ... — Generous FiTs triggered a surge in solar and wind development, transforming the country from a marginal player into a regional clean energy ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam is transitioning from a period of rapid, subsidy-driven renewable energy growth to a more disciplined, market-based approach under the DPPA framework and PDP8. The focus has shifted from mere development speed to long-term system stability, regulatory compliance, and aligning generation with grid capacity to ensure financial and operational sustainability.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Bloomberg Businessweek Vietnam 02.2026 Featured Issue ... — Generous FiTs triggered a surge in solar and wind development, transforming the country from a marginal player into a regional clean energy ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Việt Nam đang chuyển dịch từ giai đoạn phát triển năng lượng tái tạo nhanh chóng dựa trên trợ giá (FiT) sang mô hình dựa trên kỷ luật thị trường và cơ chế DPPA. Quá trình này ưu tiên tính ổn định của hệ thống, tuân thủ quy định pháp luật và sự phù hợp với Quy hoạch điện VIII (PDP8) thay vì chỉ tập trung vào tốc độ tăng trưởng.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -9959,17 +9959,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] From boom to balance in Vietnam's clean energy transition - IEEFA — Vietnamese authorities are looking to retroactively revise purchase prices for 173 solar and wind projects, reducing revenues by 25% to 46%, ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남은 제8차 국가전력개발계획(PDP8)에 따라 2030년까지 태양광 73GW 및 육상 풍력 38GW 확보를 목표로 청정에너지 전환을 가속화하고 있습니다. 과거 고정가격매입제도(FiT)의 성공을 발판 삼아, 이제는 직접전력구매계약(DPPA)과 경쟁 입찰 도입을 통해 시장 중심의 지속 가능한 에너지 인프라 구축에 집중하고 있습니다.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] From boom to balance in Vietnam's clean energy transition - IEEFA — Vietnamese authorities are looking to retroactively revise purchase prices for 173 solar and wind projects, reducing revenues by 25% to 46%, ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam is accelerating its clean energy transition under the revised PDP8, aiming for 73GW of solar and 38GW of onshore wind capacity by 2030. Following a rapid FiT-driven expansion, the sector is now shifting toward sustainable models like Direct Power Purchase Agreements (DPPA) and competitive auctions to ensure financial stability for the state utility.</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] From boom to balance in Vietnam's clean energy transition - IEEFA — Vietnamese authorities are looking to retroactively revise purchase prices for 173 solar and wind projects, reducing revenues by 25% to 46%, ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Việt Nam đang đẩy nhanh quá trình chuyển đổi năng lượng sạch theo Quy hoạch điện VIII (PDP8) sửa đổi, hướng tới mục tiêu 73GW điện mặt trời và 38GW điện gió trên bãi vào năm 2030. Sau giai đoạn bùng nổ nhờ giá FiT, ngành năng lượng đang chuyển sang các mô hình bền vững hơn như cơ chế mua bán điện trực tiếp (DPPA) và đấu thầu cạnh tranh để đảm bảo an ninh tài chính.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -10023,17 +10023,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam inaugurates USD1.4 billion LNG power plants in energy ... — LNG-fired electricity generation reduces carbon emissions by roughly 40 per cent compared with coal and 30 per cent compared with oil, ... (관련: VN-PWR-PDP8, VN-GAS-PDP8)</t>
+          <t>베트남은 동나이성에 총 1624MW 규모의 첫 액체천연가스(LNG) 발전소인 년짝 3, 4호기를 14억 달러를 투입하여 완공했습니다. 이 시설은 국가 전력 발전 계획에 따른 향후 13개 LNG 프로젝트의 모델이 되어 남부 지역의 전력망 안정화와 2050년 탄소 중립 목표 달성을 지원할 예정입니다.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam inaugurates USD1.4 billion LNG power plants in energy ... — LNG-fired electricity generation reduces carbon emissions by roughly 40 per cent compared with coal and 30 per cent compared with oil, ... (Related: VN-PWR-PDP8, VN-GAS-PDP8)</t>
+          <t>Vietnam has inaugurated its first LNG power plants, the Nhon Trach 3 and 4 facilities in Dong Nai Province, built by Petrovietnam with a $1.4 billion investment. These plants provide a combined 1,624 MW capacity to stabilize the grid and serve as a template for 13 additional LNG projects under the national power development plan.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam inaugurates USD1.4 billion LNG power plants in energy ... — LNG-fired electricity generation reduces carbon emissions by roughly 40 per cent compared with coal and 30 per cent compared with oil, ... (Liên quan: VN-PWR-PDP8, VN-GAS-PDP8)</t>
+          <t>Việt Nam đã khánh thành hai nhà máy điện khí LNG đầu tiên là Nhơn Trạch 3 và Nhơn Trạch 4 tại tỉnh Đồng Nai với tổng vốn đầu tư 1,4 tỷ USD. Dự án có tổng công suất 1.624 MW này đóng vai trò quan trọng trong việc đảm bảo an ninh năng lượng quốc gia và là hình mẫu cho 13 dự án LNG tiếp theo trong quy hoạch điện lực.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -10087,17 +10087,17 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-based energy company seeks smart-grid and power ... — It is seeking technology partners offering smart-grid and advanced solutions for transmission, distribution, and renewable energy systems under ... (관련: VN-PWR-PDP8)</t>
+          <t>베트남의 한 신재생 에너지 엔지니어링 기업이 송배전 및 재생 에너지 시스템을 위한 스마트 그리드와 고급 기술 솔루션을 보유한 국제 파트너를 찾고 있습니다. 이 협력은 베트남의 제8차 국가전력개발계획(PDP8) 목표에 부합하며, 전력망의 운영 신뢰성을 높이고 자산 관리를 최적화하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-based energy company seeks smart-grid and power ... — It is seeking technology partners offering smart-grid and advanced solutions for transmission, distribution, and renewable energy systems under ... (Related: VN-PWR-PDP8)</t>
+          <t>A Vietnamese renewable energy company is seeking international partners to provide smart-grid and advanced technology solutions for power transmission and distribution systems. Aligned with the VN-PWR-PDP8 objectives, this partnership aims to improve grid reliability and optimize asset management through commercial or technical cooperation agreements.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam-based energy company seeks smart-grid and power ... — It is seeking technology partners offering smart-grid and advanced solutions for transmission, distribution, and renewable energy systems under ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Một công ty năng lượng tái tạo tại Việt Nam đang tìm kiếm đối tác quốc tế cung cấp các giải pháp lưới điện thông minh và công nghệ tiên tiến cho hệ thống truyền tải và phân phối điện. Phù hợp với định hướng Quy hoạch điện VIII (PDP8), sự hợp tác này tập trung vào việc cải thiện độ tin cậy vận hành và tối ưu hóa quản lý tài sản năng lượng.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -10147,17 +10147,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam: Power Sector Snapshot - Norton Rose Fulbright — Vietnam expects to focus on a build out of a smart grid capable of ... Việt Nam outlines three 2026 power supply scenarios amid growing electricity demand. (관련: VN-PWR-PDP8)</t>
+          <t>베트남은 2025년 4월 승인된 개정 제8차 국가전력개발계획(PDP8)에 따라 LNG, 재생에너지 및 원자력 발전을 포함한 에너지 믹스 확대를 추진하고 있습니다. 이번 계획은 BESS 용량을 최대 16,300MW로 늘리고 직접전력구매계약(DPPA) 도입을 통해 시장 중심의 전력 공급 체계를 구축하는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam: Power Sector Snapshot - Norton Rose Fulbright — Vietnam expects to focus on a build out of a smart grid capable of ... Việt Nam outlines three 2026 power supply scenarios amid growing electricity demand. (Related: VN-PWR-PDP8)</t>
+          <t>Vietnam has updated its Power Development Plan 8 (PDP8) to aggressively expand LNG, solar, wind, and nuclear energy capacity to meet surging electricity demand. The revised framework introduces market-based pricing, supports Direct Power Purchase Agreements (DPPAs), and significantly increases targets for Battery Energy Storage Systems (BESS) to ensure grid stability.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Vietnam: Power Sector Snapshot - Norton Rose Fulbright — Vietnam expects to focus on a build out of a smart grid capable of ... Việt Nam outlines three 2026 power supply scenarios amid growing electricity demand. (Liên quan: VN-PWR-PDP8)</t>
+          <t>Việt Nam đã phê duyệt điều chỉnh Quy hoạch điện VIII (PDP8) với mục tiêu đẩy mạnh phát triển điện khí LNG, năng lượng tái tạo và tái khởi động điện hạt nhân. Các chính sách mới tập trung vào cơ chế mua bán điện trực tiếp (DPPA), phát triển hệ thống lưu trữ năng lượng (BESS) và cải thiện tính khả thi về tài chính cho các dự án năng lượng.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -10207,17 +10207,17 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] [PDF] Development of Vietnam Smart Grid Roadmap for period up to year ... — The Updated Smart Grid Roadmap will benefit key stakeholders, including ERAV, Electricity of Viet. Nam (EVN), power generation companies, transmission and ... (관련: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>베트남은 2050년 넷제로 배출 목표와 제8차 전력개발계획(PDP8)에 발맞추어 2030년까지의 스마트 그리드 로드맵을 업데이트했습니다. 이 계획은 송전망 현대화, 신재생 에너지 통합, 변전소 자동화 및 사이버 보안 강화를 우선순위로 두며, 장기적으로는 전기차 충전 인프라와 가상 발전소(VPP) 도입을 지원합니다.</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] [PDF] Development of Vietnam Smart Grid Roadmap for period up to year ... — The Updated Smart Grid Roadmap will benefit key stakeholders, including ERAV, Electricity of Viet. Nam (EVN), power generation companies, transmission and ... (Related: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Vietnam has updated its Smart Grid Development Roadmap to 2030 with a vision to 2050 to align with PDP8 and Net Zero commitments. The plan prioritizes grid modernization, substation automation, and SCADA/EMS upgrades to integrate renewable energy, while also establishing frameworks for electric vehicle integration and advanced metering infrastructure.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] [PDF] Development of Vietnam Smart Grid Roadmap for period up to year ... — The Updated Smart Grid Roadmap will benefit key stakeholders, including ERAV, Electricity of Viet. Nam (EVN), power generation companies, transmission and ... (Liên quan: VN-PWR-PDP8, VN-EV-2030)</t>
+          <t>Việt Nam đã cập nhật Lộ trình phát triển Lưới điện thông minh đến năm 2030, tầm nhìn đến năm 2050 nhằm phù hợp với Quy hoạch điện VIII và cam kết Net Zero. Kế hoạch tập trung ưu tiên hiện đại hóa hệ thống điều khiển, tự động hóa trạm biến áp và tăng cường an ninh mạng để tích hợp năng lượng tái tạo, đồng thời chuẩn bị hạ tầng cho xe điện và các nguồn năng lượng phân tán.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -10271,17 +10271,17 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM-RESOLUTION 70-NQ/TW-2025 FACILITATES CAPITAL ... — Nuclear Power Development: Urges expedited implementation of the Ninh Thuận 1 and 2 nuclear power plants by 2030–2035, with opportunities for ... (관련: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>베트남 정치국은 2030년까지 국가 에너지 안보를 보장하기 위한 결의안 제70-NQ/TW호를 발표하고 민간 및 외국인 투자를 가로막는 제도적 장벽을 제거하기로 했습니다. 이 결의안은 재생 에너지 비중을 30%까지 확대하고 닌투언 원자력 발전소 건설을 재개하는 등 에너지 믹스 다양화와 탄소 중립 목표 달성을 강조합니다.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM-RESOLUTION 70-NQ/TW-2025 FACILITATES CAPITAL ... — Nuclear Power Development: Urges expedited implementation of the Ninh Thuận 1 and 2 nuclear power plants by 2030–2035, with opportunities for ... (Related: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Vietnam's Politburo has issued Resolution 70-NQ/TW to enhance national energy security by 2030, specifically targeting the removal of institutional barriers to attract private and international capital. The directive prioritizes renewable energy growth, smart grid development, and the expedited revival of nuclear power projects like Ninh Thuan 1 and 2.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] VIETNAM-RESOLUTION 70-NQ/TW-2025 FACILITATES CAPITAL ... — Nuclear Power Development: Urges expedited implementation of the Ninh Thuận 1 and 2 nuclear power plants by 2030–2035, with opportunities for ... (Liên quan: VN-PWR-PDP8, VN-REN-NPP-2050, VN-EV-2030)</t>
+          <t>Bộ Chính trị đã ban hành Nghị quyết 70-NQ/TW nhằm đảm bảo an ninh năng lượng quốc gia đến năm 2030, tập trung tháo gỡ các rào cản thể chế để thu hút vốn đầu tư tư nhân và quốc tế. Nghị quyết ưu tiên phát triển năng lượng tái tạo chiếm 25-30% tổng cung và thúc đẩy triển khai các dự án điện hạt nhân Ninh Thuận 1 và 2 trong giai đoạn 2030-2035.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -10331,17 +10331,17 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Smart Grids for Renewable Energy and Energy Efficiency - ESP — The 'Smart Grids for Renewable Energy and Energy Efficiency (SGREEE)' project is supporting the Government of Viet Nam in the implementation of its Smart Grid ... (관련: VN-PWR-PDP8)</t>
+          <t>독일 경제협력개발부(BMZ)가 자금을 지원하는 SGREEE 프로젝트는 베트남 전력 규제청(ERAV)과 협력하여 국가 전력망의 현대화와 자동화를 추진하고 있습니다. 이 사업은 재생 에너지 통합을 확대하고 에너지 효율을 높이기 위한 스마트 그리드 로드맵 이행과 전력 시스템의 디지털화를 지원합니다.</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Smart Grids for Renewable Energy and Energy Efficiency - ESP — The 'Smart Grids for Renewable Energy and Energy Efficiency (SGREEE)' project is supporting the Government of Viet Nam in the implementation of its Smart Grid ... (Related: VN-PWR-PDP8)</t>
+          <t>The SGREEE project, funded by BMZ and partnered with ERAV, supports the modernization and automation of Vietnam's national power grid. It focuses on implementing the Smart Grid Roadmap to facilitate the integration of renewable energy and enhance energy efficiency through digitalization and system flexibility.</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>[Power &amp; Energy] Smart Grids for Renewable Energy and Energy Efficiency - ESP — The 'Smart Grids for Renewable Energy and Energy Efficiency (SGREEE)' project is supporting the Government of Viet Nam in the implementation of its Smart Grid ... (Liên quan: VN-PWR-PDP8)</t>
+          <t>Dự án SGREEE, do BMZ tài trợ và hợp tác với ERAV, hỗ trợ Chính phủ Việt Nam hiện đại hóa và tự động hóa hệ thống truyền tải và phân phối điện quốc gia. Dự án tập trung vào việc thực hiện Lộ trình Lưới điện thông minh nhằm tích hợp năng lượng tái tạo và nâng cao hiệu quả năng lượng thông qua chuyển đổi số.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -10486,17 +10486,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Study Reveals Water and Air Pollution Risks in Vietnam — Environmental study finds elevated lead, manganese, and PM2.5 pollution affecting workers and families near Hanoi's industrial zones. (관련: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>RTI International은 베트남의 산업 위험 연구를 통해 대기 및 수질 오염 문제 해결을 위한 과학적 솔루션을 제공합니다. 이 프로젝트는 환경 및 기후 분야의 인프라 발전을 목표로 하며 VN-ENV-IND-1894 및 VN-EV-2030 계획과 연계됩니다.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Study Reveals Water and Air Pollution Risks in Vietnam — Environmental study finds elevated lead, manganese, and PM2.5 pollution affecting workers and families near Hanoi's industrial zones. (Related: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>RTI International conducts an industrial risk study on air and water pollution in Vietnam to provide science-based environmental solutions. This initiative supports infrastructure goals in the Environment &amp; Climate sector, aligning with the VN-ENV-IND-1894 and VN-EV-2030 strategic plans.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Study Reveals Water and Air Pollution Risks in Vietnam — Environmental study finds elevated lead, manganese, and PM2.5 pollution affecting workers and families near Hanoi's industrial zones. (Liên quan: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>RTI International thực hiện nghiên cứu rủi ro công nghiệp về ô nhiễm không khí và nguồn nước tại Việt Nam nhằm đưa ra các giải pháp khoa học. Dự án này hỗ trợ phát triển hạ tầng trong lĩnh vực Môi trường &amp; Khí hậu, phù hợp với các kế hoạch VN-ENV-IND-1894 và VN-EV-2030.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -10546,17 +10546,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] ENVIRONMENTAL IMPACT OF INDUSTRIALIZATION — This report examines the environmental impact of industrialization in Vietnam, highlighting air and water pollution, solid waste issues, and the challenges ... (관련: VN-ENV-IND-1894)</t>
+          <t>베트남은 급격한 산업화로 인해 경제 성장을 이루었으나 공기, 수질 및 토양 자원에 심각한 부담을 주고 있습니다. 하노이와 호치민시의 미세먼지 오염이 심각하며, 산업 단지 인근의 폐수 무단 방류로 인해 '죽은 강'이 늘어나고 있습니다.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] ENVIRONMENTAL IMPACT OF INDUSTRIALIZATION — This report examines the environmental impact of industrialization in Vietnam, highlighting air and water pollution, solid waste issues, and the challenges ... (Related: VN-ENV-IND-1894)</t>
+          <t>Vietnam's rapid industrialization has driven economic growth but caused severe strain on air, water, and soil resources. Major cities face critical PM2.5 pollution from industrial zones and transport, while untreated wastewater from textile and electronic sectors is creating "dead rivers" and contaminating groundwater.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] ENVIRONMENTAL IMPACT OF INDUSTRIALIZATION — This report examines the environmental impact of industrialization in Vietnam, highlighting air and water pollution, solid waste issues, and the challenges ... (Liên quan: VN-ENV-IND-1894)</t>
+          <t>Quá trình công nghiệp hóa nhanh chóng của Việt Nam đã thúc đẩy kinh tế nhưng gây áp lực lớn lên tài nguyên không khí, nước và đất. Các thành phố lớn đang đối mặt với ô nhiễm bụi mịn nghiêm trọng, trong khi nước thải chưa qua xử lý từ các khu công nghiệp đang tạo ra những "dòng sông chết" và đe dọa nguồn nước ngầm.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -10610,17 +10610,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's green horizon: A 2025-2030 plan for ... — Air pollution control equipment is projected to cover 60%-70% of domestic needs, while solid and hazardous waste treatment technologies are to ... (관련: VN-ENV-IND-1894)</t>
+          <t>베트남은 2025년까지 산림 피복률을 42.03%로 유지하고 1,300만 달러 규모의 오존층 파괴 물질 감축 프로젝트를 시작했습니다. 하노이와 호치민시는 2027년부터 이륜차 배기가스 검사를 시행하며, 2030년까지 전국으로 확대할 계획입니다.</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's green horizon: A 2025-2030 plan for ... — Air pollution control equipment is projected to cover 60%-70% of domestic needs, while solid and hazardous waste treatment technologies are to ... (Related: VN-ENV-IND-1894)</t>
+          <t>Vietnam has maintained a stable forest coverage of 42.03% as of 2025 and launched a 13 million USD project to phase out ozone-depleting substances by 2031. Additionally, the country will implement mandatory motorcycle emissions testing in major cities starting in 2027, expanding nationwide by 2030.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam's green horizon: A 2025-2030 plan for ... — Air pollution control equipment is projected to cover 60%-70% of domestic needs, while solid and hazardous waste treatment technologies are to ... (Liên quan: VN-ENV-IND-1894)</t>
+          <t>Việt Nam duy trì tỷ lệ che phủ rừng ổn định ở mức 42,03% vào năm 2025 và triển khai dự án 13 triệu USD nhằm loại bỏ các chất làm suy giảm tầng ozone. Bên cạnh đó, lộ trình kiểm định khí thải xe máy sẽ bắt đầu tại Hà Nội và TP.HCM từ năm 2027, sau đó mở rộng ra toàn quốc vào năm 2030.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -10670,17 +10670,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Current status of industrial waste management in Vietnam — Especially, industrial zones that have not yet built and operated wastewater treatment stations cause even greater environmental pollution, such as Cau Ngan ... (관련: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>베트남 산업단지의 약 79%가 중앙 집중식 폐수 처리 시스템을 갖추고 있으나, 많은 곳이 비효율적으로 운영되거나 환경 기준을 충족하지 못하고 있습니다. 산업 클러스터(CCN)의 경우 단 5%만이 처리 시설을 보유하고 있으며, 고형 및 유해 폐기물 수집 시설의 부족이 심각한 환경 오염의 원인이 되고 있습니다.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Current status of industrial waste management in Vietnam — Especially, industrial zones that have not yet built and operated wastewater treatment stations cause even greater environmental pollution, such as Cau Ngan ... (Related: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>Approximately 79% of Vietnam's operating industrial zones have built centralized wastewater treatment systems, yet many face operational inefficiencies and fail to meet national environmental standards. Industrial clusters (CCNs) lag significantly with only a 5% coverage rate, and the lack of dedicated collection and treatment centers for hazardous solid waste continues to pressure natural ecosystems.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Current status of industrial waste management in Vietnam — Especially, industrial zones that have not yet built and operated wastewater treatment stations cause even greater environmental pollution, such as Cau Ngan ... (Liên quan: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>Khoảng 79% các khu công nghiệp tại Việt Nam đã xây dựng hệ thống xử lý nước thải tập trung, nhưng nhiều nơi vận hành chưa hiệu quả và chưa đạt quy chuẩn môi trường. Các cụm công nghiệp (CCN) chỉ có khoảng 5% có hệ thống xử lý, đồng thời việc thiếu hụt các trung tâm thu gom và xử lý chất thải rắn nguy hại đang gây áp lực lớn lên hệ sinh thái và sức khỏe con người.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -10730,17 +10730,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam To Set Up Industrial Environmental Index — Vietnam has developed industrial zones ... zones would significantly resolve environmental issues, reduce waste, and achieve sustainable development. (관련: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>베트남 기획투자부는 지속 가능한 산업 발전을 촉진하기 위해 산업 환경 지수를 도입할 계획이라고 발표했습니다. 이 지수는 2021-2030 녹색 성장 전략의 일환으로, 400개 이상의 산업 단지와 18개 경제 구역의 환경 오염 문제를 해결하고 2050년 탄소 중립 목표 달성을 돕는 것을 목표로 합니다.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam To Set Up Industrial Environmental Index — Vietnam has developed industrial zones ... zones would significantly resolve environmental issues, reduce waste, and achieve sustainable development. (Related: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>The Vietnamese Ministry of Planning has announced plans to implement an Industrial Environmental Index to promote sustainable industrial development across its 400+ industrial parks. This initiative is part of the country's 2021-2030 green growth strategy and aims to mitigate severe industrial pollution while aligning with the national goal of reaching net-zero emissions by 2050.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>[Environment &amp; Climate] Vietnam To Set Up Industrial Environmental Index — Vietnam has developed industrial zones ... zones would significantly resolve environmental issues, reduce waste, and achieve sustainable development. (Liên quan: VN-ENV-IND-1894, VN-EV-2030)</t>
+          <t>Bộ Kế hoạch và Đầu tư Việt Nam vừa công bố kế hoạch triển khai bộ chỉ số môi trường công nghiệp nhằm thúc đẩy phát triển công nghiệp bền vững. Đây là một phần trong chiến lược tăng trưởng xanh giai đoạn 2021-2030, hướng tới mục tiêu giải quyết vấn đề ô nhiễm tại các khu công nghiệp và đạt phát thải ròng bằng 0 vào năm 2050.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">

</xml_diff>